<commit_message>
Kitchens default to a staff kitchenette on non-domestic buildings
'Default option' on '4. Scope rules' now also takes building-use codes:
"RES STU" makes an option the default for those uses, ahead of the general
Yes. Kitchens uses it — domestic kitchen on residential and student, staff
kitchenette everywhere else — so an office no longer prices its per-floor
kitchenettes as £6,000 domestic kitchens. The user's own choice still wins.
Codes are checked like every other building-use code in the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\AppData\Local\Temp\claude\C--Users-nabil-estates-ai-tool\dabfa264-632a-467f-bca3-d20315440194\scratchpad\build\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\estates-ai-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3195DDB5-609B-44BC-95F7-77A89C0572BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C215B59C-5C55-471D-A7A4-2530608F6CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="41340" yWindow="2940" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4081" uniqueCount="1634">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4084" uniqueCount="1635">
   <si>
     <t>3. Settings</t>
   </si>
@@ -4932,7 +4932,10 @@
     <t>v5.6 — 28 Sept 2026</t>
   </si>
   <si>
-    <t>Owner's review of v5.5: rates edited by the owner (roof, internal doors, toilets, fixed joinery, signage, AV, loose furniture, heating High, water, cooling, controls, lighting, fire alarm, sprinklers, solar PV); frame, upper floors and stairs no longer offered on refurbishment. Toilets: one rate for every building use (HOS and HEA variants removed). Changing Places Standard £45,000. Showers 900 / 1,400 / 2,500. Bathroom pods and bin store removed (bin store's old code 8.12 retired). Tea point renamed Staff kitchenette (non-domestic). Mezzanine offered on Fit-out, not Refurbishment.</t>
+    <t>Yes = the option chosen unless the user picks another. Building-use codes (e.g. RES STU) = the default for those uses only, ahead of Yes — Kitchens defaults to a domestic kitchen on residential and student buildings and a staff kitchenette everywhere else.</t>
+  </si>
+  <si>
+    <t>Owner's review of v5.5: rates edited by the owner (roof, internal doors, toilets, fixed joinery, signage, AV, loose furniture, heating High, water, cooling, controls, lighting, fire alarm, sprinklers, solar PV); frame, upper floors and stairs no longer offered on refurbishment. Toilets: one rate for every building use (HOS and HEA variants removed). Changing Places Standard £45,000. Showers 900 / 1,400 / 2,500. Bathroom pods and bin store removed (bin store's old code 8.12 retired). Tea point renamed Staff kitchenette (non-domestic). Mezzanine offered on Fit-out, not Refurbishment. Kitchens: staff kitchenette is the default on non-domestic buildings, domestic kitchen on residential and student (Default option now takes building-use codes).</t>
   </si>
 </sst>
 </file>
@@ -5553,7 +5556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BBCD35-3C7D-4CAC-A46E-6C3CC3E31849}">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.7109375" style="8" customWidth="1"/>
@@ -5915,376 +5918,385 @@
       </c>
       <c r="C43" s="33"/>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A44" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" s="17" t="s">
+        <v>1633</v>
+      </c>
+      <c r="C44" s="33"/>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="17" t="s">
+      <c r="B45" s="17" t="s">
         <v>1594</v>
-      </c>
-      <c r="C44" s="33"/>
-    </row>
-    <row r="45" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A45" s="15" t="s">
-        <v>1595</v>
-      </c>
-      <c r="B45" s="17" t="s">
-        <v>1596</v>
       </c>
       <c r="C45" s="33"/>
     </row>
     <row r="46" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A46" s="15" t="s">
+        <v>1595</v>
+      </c>
+      <c r="B46" s="17" t="s">
+        <v>1596</v>
+      </c>
+      <c r="C46" s="33"/>
+    </row>
+    <row r="47" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A47" s="15" t="s">
         <v>1597</v>
       </c>
-      <c r="B46" s="17" t="s">
+      <c r="B47" s="17" t="s">
         <v>1598</v>
-      </c>
-      <c r="C46" s="33"/>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="15" t="s">
-        <v>1599</v>
-      </c>
-      <c r="B47" s="17" t="s">
-        <v>1600</v>
       </c>
       <c r="C47" s="33"/>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="15" t="s">
-        <v>1601</v>
+        <v>1599</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>1602</v>
+        <v>1600</v>
       </c>
       <c r="C48" s="33"/>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="15" t="s">
+        <v>1601</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>1602</v>
+      </c>
+      <c r="C49" s="33"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B50" s="17" t="s">
         <v>1603</v>
       </c>
-      <c r="C49" s="33"/>
-    </row>
-    <row r="50" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A50" s="15" t="s">
+      <c r="C50" s="33"/>
+    </row>
+    <row r="51" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A51" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B50" s="17" t="s">
+      <c r="B51" s="17" t="s">
         <v>1604</v>
-      </c>
-      <c r="C50" s="33"/>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="15" t="s">
-        <v>1605</v>
-      </c>
-      <c r="B51" s="17" t="s">
-        <v>1606</v>
       </c>
       <c r="C51" s="33"/>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="15" t="s">
-        <v>46</v>
+        <v>1605</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="C52" s="33"/>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="15" t="s">
-        <v>1608</v>
+        <v>46</v>
       </c>
       <c r="B53" s="17" t="s">
-        <v>1609</v>
+        <v>1607</v>
       </c>
       <c r="C53" s="33"/>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="15" t="s">
+        <v>1608</v>
+      </c>
+      <c r="B54" s="17" t="s">
+        <v>1609</v>
+      </c>
+      <c r="C54" s="33"/>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="B54" s="17" t="s">
+      <c r="B55" s="17" t="s">
         <v>1610</v>
       </c>
-      <c r="C54" s="33"/>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="15"/>
-      <c r="B55" s="17"/>
       <c r="C55" s="33"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="13" t="s">
+      <c r="A56" s="15"/>
+      <c r="B56" s="17"/>
+      <c r="C56" s="33"/>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B56" s="16"/>
-      <c r="C56" s="34"/>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="15" t="s">
+      <c r="B57" s="16"/>
+      <c r="C57" s="34"/>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="15" t="s">
         <v>1611</v>
       </c>
-      <c r="B57" s="17"/>
-      <c r="C57" s="33">
+      <c r="B58" s="17"/>
+      <c r="C58" s="33">
         <f>SUMPRODUCT(('2. Rates'!O6:O146&lt;&gt;"")*(COUNTIF('2. Rates'!O6:O146,'2. Rates'!O6:O146)&gt;1))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="15" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="15" t="s">
         <v>1612</v>
       </c>
-      <c r="B58" s="17"/>
-      <c r="C58" s="33">
+      <c r="B59" s="17"/>
+      <c r="C59" s="33">
         <f>SUMPRODUCT(('2. Rates'!O6:O146&lt;&gt;"")*(COUNTIF('4. Scope rules'!A91:A223,'2. Rates'!O6:O146)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="15" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="15" t="s">
         <v>1613</v>
       </c>
-      <c r="B59" s="17"/>
-      <c r="C59" s="33">
+      <c r="B60" s="17"/>
+      <c r="C60" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A91:A223&lt;&gt;"")*(COUNTIF('2. Rates'!O6:O146,'4. Scope rules'!A91:A223)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="15" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="15" t="s">
         <v>1614</v>
       </c>
-      <c r="B60" s="17"/>
-      <c r="C60" s="33">
+      <c r="B61" s="17"/>
+      <c r="C61" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A91:A223&lt;&gt;"")*(COUNTIF('4. Scope rules'!A6:A87,'4. Scope rules'!B91:B223)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="15" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="15" t="s">
         <v>1615</v>
       </c>
-      <c r="B61" s="17"/>
-      <c r="C61" s="33">
+      <c r="B62" s="17"/>
+      <c r="C62" s="33">
         <f>SUMPRODUCT(('2. Rates'!O6:O146&lt;&gt;"")*('2. Rates'!M6:M146=""))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="15" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="15" t="s">
         <v>1616</v>
       </c>
-      <c r="B62" s="17"/>
-      <c r="C62" s="33">
+      <c r="B63" s="17"/>
+      <c r="C63" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*(ROUND('4. Scope rules'!M6:M87+'4. Scope rules'!O6:O87,4)&lt;&gt;1))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="15" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B63" s="17"/>
-      <c r="C63" s="33">
+      <c r="B64" s="17"/>
+      <c r="C64" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*(COUNTIFS('4. Scope rules'!B91:B223,'4. Scope rules'!A6:A87,'4. Scope rules'!E91:E223,"Yes")=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="15" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="15" t="s">
         <v>1617</v>
       </c>
-      <c r="B64" s="17"/>
-      <c r="C64" s="33">
+      <c r="B65" s="17"/>
+      <c r="C65" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*('4. Scope rules'!F6:F87="One")*(COUNTIFS('4. Scope rules'!B91:B223,'4. Scope rules'!A6:A87,'4. Scope rules'!E91:E223,"Yes")&gt;1))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="15" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="15" t="s">
         <v>1618</v>
       </c>
-      <c r="B65" s="17"/>
-      <c r="C65" s="33">
+      <c r="B66" s="17"/>
+      <c r="C66" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*('4. Scope rules'!G6:G87=""))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="15" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="33">
+      <c r="B67" s="17"/>
+      <c r="C67" s="33">
         <f>SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('4. Scope rules'!H6:H87,"NB",""),"EX",""),"RF",""),"FO",""),"EW",""),"DM",""),"OM",""),"—","")))&gt;0))+SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('4. Scope rules'!I6:I87,"NB",""),"EX",""),"RF",""),"FO",""),"EW",""),"DM",""),"OM",""),"—","")))&gt;0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" s="15" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B67" s="17"/>
-      <c r="C67" s="33">
+      <c r="B68" s="17"/>
+      <c r="C68" s="33">
         <f>SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('4. Scope rules'!J6:J87,"RES",""),"STU",""),"OFF",""),"EDU",""),"HEA",""),"RET",""),"IND",""),"HOS",""),"MIX",""),"OTH",""),"ALL","")))&gt;0))+SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('2. Rates'!D6:D146,"RES",""),"STU",""),"OFF",""),"EDU",""),"HEA",""),"RET",""),"IND",""),"HOS",""),"MIX",""),"OTH",""),"ALL","")))&gt;0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="15" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B68" s="17"/>
-      <c r="C68" s="33">
+      <c r="B69" s="17"/>
+      <c r="C69" s="33">
         <f>SUMPRODUCT(('3. Settings'!A96:A123&lt;&gt;"")*(COUNTIFS('3. Settings'!A96:A123,'3. Settings'!A96:A123,'3. Settings'!B96:B123,"ALL")=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="15" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B69" s="17"/>
-      <c r="C69" s="33">
+      <c r="B70" s="17"/>
+      <c r="C70" s="33">
         <f>SUMPRODUCT(('3. Settings'!A96:A123&lt;&gt;"")*('3. Settings'!C96:C123=""))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="15"/>
-      <c r="B70" s="17"/>
-      <c r="C70" s="33"/>
-    </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="13" t="s">
+      <c r="A71" s="15"/>
+      <c r="B71" s="17"/>
+      <c r="C71" s="33"/>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B71" s="16"/>
-      <c r="C71" s="34"/>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="15" t="s">
+      <c r="B72" s="16"/>
+      <c r="C72" s="34"/>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B72" s="17"/>
-      <c r="C72" s="33">
+      <c r="B73" s="17"/>
+      <c r="C73" s="33">
         <f>COUNTA('4. Scope rules'!A6:A87)</f>
         <v>82</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A73" s="15" t="s">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="15" t="s">
         <v>1619</v>
       </c>
-      <c r="B73" s="17"/>
-      <c r="C73" s="33">
+      <c r="B74" s="17"/>
+      <c r="C74" s="33">
         <f>COUNTA('2. Rates'!O6:O146)</f>
         <v>133</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="15"/>
-      <c r="B74" s="17"/>
-      <c r="C74" s="33"/>
-    </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="13" t="s">
+      <c r="A75" s="15"/>
+      <c r="B75" s="17"/>
+      <c r="C75" s="33"/>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B75" s="16"/>
-      <c r="C75" s="34"/>
-    </row>
-    <row r="76" spans="1:3" s="54" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A76" s="17" t="s">
+      <c r="B76" s="16"/>
+      <c r="C76" s="34"/>
+    </row>
+    <row r="77" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A77" s="17" t="s">
         <v>1632</v>
       </c>
-      <c r="B76" s="17" t="s">
-        <v>1633</v>
-      </c>
-      <c r="C76" s="60"/>
-    </row>
-    <row r="77" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A77" s="15" t="s">
+      <c r="B77" s="17" t="s">
+        <v>1634</v>
+      </c>
+      <c r="C77" s="60"/>
+    </row>
+    <row r="78" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A78" s="15" t="s">
         <v>1620</v>
       </c>
-      <c r="B77" s="17" t="s">
+      <c r="B78" s="17" t="s">
         <v>1621</v>
       </c>
-      <c r="C77" s="33"/>
-    </row>
-    <row r="78" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A78" s="15" t="s">
+      <c r="C78" s="33"/>
+    </row>
+    <row r="79" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A79" s="15" t="s">
         <v>1060</v>
       </c>
-      <c r="B78" s="17" t="s">
+      <c r="B79" s="17" t="s">
         <v>1061</v>
       </c>
-      <c r="C78" s="33"/>
-    </row>
-    <row r="79" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A79" s="15" t="s">
+      <c r="C79" s="33"/>
+    </row>
+    <row r="80" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A80" s="15" t="s">
         <v>1051</v>
       </c>
-      <c r="B79" s="17" t="s">
+      <c r="B80" s="17" t="s">
         <v>1052</v>
       </c>
-      <c r="C79" s="33"/>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A80" s="15" t="s">
+      <c r="C80" s="33"/>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B80" s="17" t="s">
+      <c r="B81" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C80" s="33"/>
-    </row>
-    <row r="81" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A81" s="15" t="s">
+      <c r="C81" s="33"/>
+    </row>
+    <row r="82" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A82" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B82" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C81" s="33"/>
-    </row>
-    <row r="82" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A82" s="15" t="s">
+      <c r="C82" s="33"/>
+    </row>
+    <row r="83" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A83" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B82" s="17" t="s">
+      <c r="B83" s="17" t="s">
         <v>28</v>
-      </c>
-      <c r="C82" s="33"/>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B83" s="17" t="s">
-        <v>30</v>
       </c>
       <c r="C83" s="33"/>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B84" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C84" s="33"/>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B85" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C84" s="33"/>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A85" s="15"/>
-      <c r="B85" s="17"/>
       <c r="C85" s="33"/>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86" s="15"/>
+      <c r="B86" s="17"/>
+      <c r="C86" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20362,7 +20374,7 @@
         <v>274</v>
       </c>
       <c r="E123" s="15" t="s">
-        <v>66</v>
+        <v>456</v>
       </c>
       <c r="F123" s="15" t="s">
         <v>107</v>
@@ -20397,7 +20409,9 @@
       <c r="D124" s="15" t="s">
         <v>1627</v>
       </c>
-      <c r="E124" s="15"/>
+      <c r="E124" s="15" t="s">
+        <v>66</v>
+      </c>
       <c r="F124" s="15" t="s">
         <v>107</v>
       </c>

</xml_diff>

<commit_message>
NRM1 v5.8: add Computer Science decarbonisation tender evidence
Evidence only - no rate, option, rule or formula changed. Adds the
Computer Science Building decarbonisation tender returns (Harrabin and
Chiel, Mar 2024; mean of two bids x 1.07 / 0.94) to the Tender check
column for 2.5a, 2.6, 2.7, 5.1b, 5.26a and 7.1a. Updates the column
header and Instructions note, inserts an update-log line, bumps the
version to 5.8 and moves the version-pinned test.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrJDd1NaMQvzBf6wrGMvgx
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4211" uniqueCount="1713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4217" uniqueCount="1726">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5170,6 +5170,45 @@
   </si>
   <si>
     <t>Lakeside S&amp;F tender returns (29 Sept 2026): five bids, four used (median ÷ 0.94 West Midlands factor, on 3,306 m² measured floor area). Changed, Refurb &amp; Fit-out columns only: strip-out £45 → £55; bathrooms £900 / £2,000 / £3,500 → £1,150 / £2,500 / £4,400; domestic kitchens £3,500 / £6,000 / £10,000 → £3,100 / £5,300 / £8,850; residential power (5.7b) £70 / £108 / £185 → £95 / £150 / £255. Added: residential rows (RES STU) for floor finishes (3.2c £50), ceilings (3.3b £30), data incl. TV aerial (5.14b £25) and builder's work (5.26b £27); options Roof — Loft insulation only (2.5b, £32/m² roof) and Ventilation — Extract fans only (5.3b, £19). Ratios: m2_per_dwelling 80 → 66, bathrooms_per_dwelling 1.2 → 1.0. New 'Tender check' column on '2. Rates' and price source 'Tender – Lakeside S&amp;F (Sep 2026)'. Confirmed and kept: wall finishes, water (visible fittings), fire alarm, data, fire stopping (Basic).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loft insulation only: £32 — see 2.5b. CS: £313 (bids £288–£338) per m² of roof re-covered (699 m², less than the footprint) for a flat warm-roof overlay on the kept asphalt: AVCL, 120 mm PIR, two-layer felt, insulated upstands, new copings, ballast relaid. Scaffold extra (see 2.7). Claycroft pitched re-roof £627–£704.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £40 (bids £38–£43) for insulated render to part of the façade of an occupied 4-storey building. With the brick remedials under it (see 7.1a): £81 (bids £59–£102). Scaffold extra (see 2.7).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £176 (bids £161–£191) for triple-glazed windows, curtain walling and doors on a whole 4-storey building (openings ≈ 13% of GIFA, ≈ £1,330/m² of opening), incl. take-out, closers, fire barriers, reveals, boards and decs (≈ 30% on top of supply and fit). At High. The low bid left out the curtain walling. Scaffold for envelope works (in the bids' prelims): £35 (bids £29–£41) per m² GIFA, extra to 2.5a, 2.6 and 2.7.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £188 (bids £176–£200) for the whole M&amp;E package of an air source heat pump conversion of an occupied academic building: heat pumps replacing gas boilers, LTHW alterations, coils to 6 AHUs, radiators, BMS and ventilation (no breakdown). Std 5.1b + 5.5 = £93.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Residential rewire: £27 — see 5.26b. CS: £6.5 (bids £5–£8), 2.5–4.6% of M&amp;E, for a heat pump conversion (plant room, pipework and radiators).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £40 (bids £21–£60) for brick remedials before rendering: slab edges exposed, new stainless steel angles and cavity trays, remedial ties, movement joints, repointing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender check (this row's unit, on this workbook's basis. Unlabelled = Lakeside S&amp;F, Sep 2026: median of 4 bids ÷ 0.94. CS = Computer Science decarbonisation, Mar 2024: 2 bids × 1.07 ÷ 0.94)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.8 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lakeside Staff &amp; Family Flats tender returns (29 Sept 2026) converted to this workbook's basis: the median of the four credible bids (BSN, Chiel, Harrabin, William Gough with its kitchen error corrected; Watkin Jones excluded at twice the field) ÷ 0.94 West Midlands factor, per this row's unit, on 3,306 m² measured floor area (49 flats, the Warden's house and nine stair cores). Excludes the contractors' preliminaries and OH&amp;P. Lines starting 'CS:' are the Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; two bids, so the mean): tender × 1.07 (to Q3 2026) ÷ 0.94, on about 4,170 m² GIA measured from the tender plans and 699 m² of roof. Evidence only: no rate was changed for them in v5.8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v5.8 — 1 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence only, no rates changed. Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; mean of two bids × 1.07 ÷ 0.94, on about 4,170 m² GIA and 699 m² of roof) added to the Tender check column for 2.5a roof, 2.6 external walls, 2.7 windows (with the scaffold figure), 5.1b air source heat pump, 5.26a builder's work and 7.1a repairs. The Tender check header and its note above now cover more than one project. Suggested for the owner to decide: roof Std about £300 (Computer Science £313, Claycroft £627–£704); air source heat pump full system Std about £150; a scaffold item of about £35/m² GIFA for envelope works; triple glazing priced at High.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-01</t>
   </si>
 </sst>
 </file>
@@ -5790,7 +5829,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BBCD35-3C7D-4CAC-A46E-6C3CC3E31849}">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.7109375" style="8" customWidth="1"/>
@@ -5801,7 +5840,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1707</v>
+        <v>1720</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -5963,12 +6002,12 @@
       </c>
       <c r="C20" s="33"/>
     </row>
-    <row r="21" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" ht="51" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
         <v>1708</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>1709</v>
+        <v>1721</v>
       </c>
       <c r="C21" s="33"/>
     </row>
@@ -6466,98 +6505,107 @@
     </row>
     <row r="79" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A79" s="17" t="s">
-        <v>1711</v>
+        <v>1722</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>1712</v>
+        <v>1723</v>
       </c>
       <c r="C79" s="60"/>
     </row>
     <row r="80" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A80" s="17" t="s">
+        <v>1711</v>
+      </c>
+      <c r="B80" s="17" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C80" s="60"/>
+    </row>
+    <row r="81" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A81" s="17" t="s">
         <v>1632</v>
       </c>
-      <c r="B80" s="17" t="s">
+      <c r="B81" s="17" t="s">
         <v>1634</v>
       </c>
-      <c r="C80" s="60"/>
-    </row>
-    <row r="81" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A81" s="15" t="s">
+      <c r="C81" s="60"/>
+    </row>
+    <row r="82" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A82" s="15" t="s">
         <v>1620</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B82" s="17" t="s">
         <v>1621</v>
       </c>
-      <c r="C81" s="33"/>
-    </row>
-    <row r="82" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A82" s="15" t="s">
+      <c r="C82" s="33"/>
+    </row>
+    <row r="83" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A83" s="15" t="s">
         <v>1060</v>
       </c>
-      <c r="B82" s="17" t="s">
+      <c r="B83" s="17" t="s">
         <v>1061</v>
       </c>
-      <c r="C82" s="33"/>
-    </row>
-    <row r="83" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A83" s="15" t="s">
+      <c r="C83" s="33"/>
+    </row>
+    <row r="84" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A84" s="15" t="s">
         <v>1051</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B84" s="17" t="s">
         <v>1052</v>
       </c>
-      <c r="C83" s="33"/>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A84" s="15" t="s">
+      <c r="C84" s="33"/>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A85" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B85" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C84" s="33"/>
-    </row>
-    <row r="85" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A85" s="15" t="s">
+      <c r="C85" s="33"/>
+    </row>
+    <row r="86" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A86" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B86" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C85" s="33"/>
-    </row>
-    <row r="86" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A86" s="15" t="s">
+      <c r="C86" s="33"/>
+    </row>
+    <row r="87" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A87" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B87" s="17" t="s">
         <v>28</v>
-      </c>
-      <c r="C86" s="33"/>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A87" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B87" s="17" t="s">
-        <v>30</v>
       </c>
       <c r="C87" s="33"/>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B88" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C88" s="33"/>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B88" s="17" t="s">
+      <c r="B89" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C88" s="33"/>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A89" s="15"/>
-      <c r="B89" s="17"/>
       <c r="C89" s="33"/>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" s="15"/>
+      <c r="B90" s="17"/>
+      <c r="C90" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6651,7 +6699,7 @@
         <v>1623</v>
       </c>
       <c r="Q5" s="12" t="s">
-        <v>1690</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -7375,7 +7423,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A25" s="21" t="s">
         <v>1669</v>
       </c>
@@ -7422,7 +7470,7 @@
         <v>182</v>
       </c>
       <c r="Q25" s="22" t="s">
-        <v>1676</v>
+        <v>1713</v>
       </c>
     </row>
     <row r="26" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
@@ -7468,7 +7516,7 @@
         <v>1664</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A27" s="21" t="s">
         <v>197</v>
       </c>
@@ -7512,8 +7560,11 @@
       <c r="O27" s="24" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="Q27" s="22" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
       <c r="A28" s="21" t="s">
         <v>203</v>
       </c>
@@ -7556,6 +7607,9 @@
       </c>
       <c r="O28" s="24" t="s">
         <v>193</v>
+      </c>
+      <c r="Q28" s="22" t="s">
+        <v>1715</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -9068,7 +9122,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="64" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:17" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A64" s="55" t="s">
         <v>1027</v>
       </c>
@@ -9117,6 +9171,9 @@
       <c r="O64" s="59" t="s">
         <v>376</v>
       </c>
+      <c r="Q64" s="22" t="s">
+        <v>1716</v>
+      </c>
     </row>
     <row r="65" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A65" s="55" t="s">
@@ -11713,7 +11770,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="123" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A123" s="21" t="s">
         <v>1675</v>
       </c>
@@ -11756,7 +11813,7 @@
         <v>736</v>
       </c>
       <c r="Q123" s="22" t="s">
-        <v>1688</v>
+        <v>1717</v>
       </c>
     </row>
     <row r="124" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
@@ -11823,7 +11880,7 @@
       <c r="N125" s="26"/>
       <c r="O125" s="27"/>
     </row>
-    <row r="126" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A126" s="23" t="s">
         <v>1435</v>
       </c>
@@ -11866,6 +11923,9 @@
       <c r="N126" s="22"/>
       <c r="O126" s="24" t="s">
         <v>613</v>
+      </c>
+      <c r="Q126" s="22" t="s">
+        <v>1718</v>
       </c>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.2">
@@ -13041,7 +13101,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>428</v>
+        <v>1724</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -13052,7 +13112,7 @@
         <v>751</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>1705</v>
+        <v>1725</v>
       </c>
       <c r="C7" s="2"/>
     </row>

</xml_diff>

<commit_message>
NRM1 v5.8: add Computer Science final out-turn and heat pump sizes
Evidence only - no rate changed. Appends the final financial statement
(construction GBP 2.73m, +3.4% on contract; total GBP 3.13m excl. VAT)
and CPW's ASHP sizes (3 x 118 kW) to the CS Tender check lines on 2.7
and 5.1b, the Instructions note and the v5.8 log line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrJDd1NaMQvzBf6wrGMvgx
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4217" uniqueCount="1726">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4217" uniqueCount="1730">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5209,6 +5209,18 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £176 (bids £161–£191) for triple-glazed windows, curtain walling and doors on a whole 4-storey building (openings ≈ 13% of GIFA, ≈ £1,330/m² of opening), incl. take-out, closers, fire barriers, reveals, boards and decs (≈ 30% on top of supply and fit). At High. The low bid left out the curtain walling. Scaffold for envelope works (in the bids' prelims): £35 (bids £29–£41) per m² GIFA, extra to 2.5a, 2.6 and 2.7. Out-turn: window design development added £86k (3.3% of the contract sum) after award.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £188 (bids £176–£200) for the whole M&amp;E package of an air source heat pump conversion of an occupied academic building: heat pumps replacing gas boilers, LTHW alterations, coils to 6 AHUs, radiators, BMS and ventilation (no breakdown). Std 5.1b + 5.5 = £93. Heat pumps: 3 × 118 kW (N+1, about 240 kW duty, about 58 W/m² after the fabric works), so about £1,800–2,100 per kW installed for the whole M&amp;E package.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lakeside Staff &amp; Family Flats tender returns (29 Sept 2026) converted to this workbook's basis: the median of the four credible bids (BSN, Chiel, Harrabin, William Gough with its kitchen error corrected; Watkin Jones excluded at twice the field) ÷ 0.94 West Midlands factor, per this row's unit, on 3,306 m² measured floor area (49 flats, the Warden's house and nine stair cores). Excludes the contractors' preliminaries and OH&amp;P. Lines starting 'CS:' are the Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; two bids, so the mean): tender × 1.07 (to Q3 2026) ÷ 0.94, on about 4,170 m² GIA measured from the tender plans and 699 m² of roof. Evidence only: no rate was changed for them in v5.8. Final out-turn (financial statement, July 2026): construction £2.73m, +3.4% on a £2.64m contract; total project £3.13m excl. VAT.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence only, no rates changed. Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; mean of two bids × 1.07 ÷ 0.94, on about 4,170 m² GIA and 699 m² of roof) added to the Tender check column for 2.5a roof, 2.6 external walls, 2.7 windows (with the scaffold figure), 5.1b air source heat pump, 5.26a builder's work and 7.1a repairs. The Tender check header and its note above now cover more than one project. Suggested for the owner to decide: roof Std about £300 (Computer Science £313, Claycroft £627–£704); air source heat pump full system Std about £150; a scaffold item of about £35/m² GIFA for envelope works; triple glazing priced at High. Updated 2 Oct 2026 with the final out-turn and CPW's heat pump sizes.</t>
   </si>
 </sst>
 </file>
@@ -6007,7 +6019,7 @@
         <v>1708</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>1721</v>
+        <v>1728</v>
       </c>
       <c r="C21" s="33"/>
     </row>
@@ -6508,7 +6520,7 @@
         <v>1722</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>1723</v>
+        <v>1729</v>
       </c>
       <c r="C79" s="60"/>
     </row>
@@ -7564,7 +7576,7 @@
         <v>1714</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:17" ht="165.75" x14ac:dyDescent="0.2">
       <c r="A28" s="21" t="s">
         <v>203</v>
       </c>
@@ -7609,7 +7621,7 @@
         <v>193</v>
       </c>
       <c r="Q28" s="22" t="s">
-        <v>1715</v>
+        <v>1726</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -9122,7 +9134,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="64" spans="1:17" ht="89.25" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
       <c r="A64" s="55" t="s">
         <v>1027</v>
       </c>
@@ -9172,7 +9184,7 @@
         <v>376</v>
       </c>
       <c r="Q64" s="22" t="s">
-        <v>1716</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="65" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
NRM1 v5.8: recalculate CS evidence on the Estates GIA (3,495 m2)
Evidence only - no rate changed. The UoW Estates CAD plans give a GIA of
3,495 m2 (the 4,170 m2 measured from the tender plans counted roofs and
voids), so the CS per-m2 GIFA figures on 2.6, 2.7, 5.1b, 5.26a and 7.1a
rise by 19%. Instructions note and the v5.8 log line updated, including
the suggested rates for the owner (ASHP ~190, scaffold ~40, triple
glazing ~210).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrJDd1NaMQvzBf6wrGMvgx
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4217" uniqueCount="1730">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4217" uniqueCount="1738">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5221,6 +5221,30 @@
   </si>
   <si>
     <t xml:space="preserve">Evidence only, no rates changed. Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; mean of two bids × 1.07 ÷ 0.94, on about 4,170 m² GIA and 699 m² of roof) added to the Tender check column for 2.5a roof, 2.6 external walls, 2.7 windows (with the scaffold figure), 5.1b air source heat pump, 5.26a builder's work and 7.1a repairs. The Tender check header and its note above now cover more than one project. Suggested for the owner to decide: roof Std about £300 (Computer Science £313, Claycroft £627–£704); air source heat pump full system Std about £150; a scaffold item of about £35/m² GIFA for envelope works; triple glazing priced at High. Updated 2 Oct 2026 with the final out-turn and CPW's heat pump sizes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £48 (bids £45–£51) for insulated render to part of the façade of an occupied 4-storey building. With the brick remedials under it (see 7.1a): £97 (bids £70–£122). Scaffold extra (see 2.7).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £210 (bids £192–£228) for triple-glazed windows, curtain walling and doors on a whole 4-storey building (openings ≈ 16% of GIFA, ≈ £1,330/m² of opening), incl. take-out, closers, fire barriers, reveals, boards and decs (≈ 30% on top of supply and fit). 17% above High. The low bid left out the curtain walling. Scaffold for envelope works (in the bids' prelims): £42 (bids £35–£49) per m² GIFA, extra to 2.5a, 2.6 and 2.7. Out-turn: window design development added £86k (3.3% of the contract sum) after award.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £224 (bids £210–£238) for the whole M&amp;E package of an air source heat pump conversion of an occupied academic building: heat pumps replacing gas boilers, LTHW alterations, coils to 6 AHUs, about 160 radiators, BMS and ventilation (no breakdown). Std 5.1b + 5.5 = £93. Heat pumps: 3 × 118 kW (N+1, about 240 kW duty, about 69 W/m² after the fabric works), so about £1,800–2,100 per kW installed for the whole M&amp;E package.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Residential rewire: £27 — see 5.26b. CS: £8 (bids £6–£10), 2.5–4.6% of M&amp;E, for a heat pump conversion (plant room, pipework and radiators).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CS: £48 (bids £25–£71) for brick remedials before rendering: slab edges exposed, new stainless steel angles and cavity trays, remedial ties, movement joints, repointing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lakeside Staff &amp; Family Flats tender returns (29 Sept 2026) converted to this workbook's basis: the median of the four credible bids (BSN, Chiel, Harrabin, William Gough with its kitchen error corrected; Watkin Jones excluded at twice the field) ÷ 0.94 West Midlands factor, per this row's unit, on 3,306 m² measured floor area (49 flats, the Warden's house and nine stair cores). Excludes the contractors' preliminaries and OH&amp;P. Lines starting 'CS:' are the Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; two bids, so the mean): tender × 1.07 (to Q3 2026) ÷ 0.94, on 3,495 m² GIA (UoW Estates CAD outlines) and 699 m² of roof. Evidence only: no rate was changed for them in v5.8. Final out-turn (financial statement, July 2026): construction £2.73m, +3.4% on a £2.64m contract; total project £3.13m excl. VAT.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence only, no rates changed. Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; mean of two bids × 1.07 ÷ 0.94, on 3,495 m² GIA and 699 m² of roof) added to the Tender check column for 2.5a roof, 2.6 external walls, 2.7 windows (with the scaffold figure), 5.1b air source heat pump, 5.26a builder's work and 7.1a repairs. The Tender check header and its note above now cover more than one project. Suggested for the owner to decide: roof Std about £300 (Computer Science £313, Claycroft £627–£704); air source heat pump full system Std about £150; a scaffold item of about £35/m² GIFA for envelope works; triple glazing priced at High. Updated 2 Oct 2026 with the final out-turn and CPW's heat pump sizes, and the per-m² figures recalculated on the Estates GIA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence only, no rates changed. Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; mean of two bids × 1.07 ÷ 0.94, on 3,495 m² GIA and 699 m² of roof) added to the Tender check column for 2.5a roof, 2.6 external walls, 2.7 windows (with the scaffold figure), 5.1b air source heat pump, 5.26a builder's work and 7.1a repairs, with the final out-turn (July 2026) and CPW's heat pump sizes. The Tender check header and its note above now cover more than one project. Suggested for the owner to decide: roof Std about £300 (Computer Science £313, Claycroft £627–£704); air source heat pump full system Std about £190; a scaffold item of about £40/m² GIFA for envelope works; triple glazing about £210/m² GIFA (an option, or High).</t>
   </si>
 </sst>
 </file>
@@ -6019,7 +6043,7 @@
         <v>1708</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>1728</v>
+        <v>1735</v>
       </c>
       <c r="C21" s="33"/>
     </row>
@@ -6520,7 +6544,7 @@
         <v>1722</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>1729</v>
+        <v>1737</v>
       </c>
       <c r="C79" s="60"/>
     </row>
@@ -7573,7 +7597,7 @@
         <v>188</v>
       </c>
       <c r="Q27" s="22" t="s">
-        <v>1714</v>
+        <v>1730</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="165.75" x14ac:dyDescent="0.2">
@@ -7621,7 +7645,7 @@
         <v>193</v>
       </c>
       <c r="Q28" s="22" t="s">
-        <v>1726</v>
+        <v>1731</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -9134,7 +9158,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="64" spans="1:17" ht="127.5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:17" ht="140.25" x14ac:dyDescent="0.2">
       <c r="A64" s="55" t="s">
         <v>1027</v>
       </c>
@@ -9184,7 +9208,7 @@
         <v>376</v>
       </c>
       <c r="Q64" s="22" t="s">
-        <v>1727</v>
+        <v>1732</v>
       </c>
     </row>
     <row r="65" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -11825,7 +11849,7 @@
         <v>736</v>
       </c>
       <c r="Q123" s="22" t="s">
-        <v>1717</v>
+        <v>1733</v>
       </c>
     </row>
     <row r="124" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
@@ -11937,7 +11961,7 @@
         <v>613</v>
       </c>
       <c r="Q126" s="22" t="s">
-        <v>1718</v>
+        <v>1734</v>
       </c>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
NRM1 v5.9: add Whitefields demolition rate column (evidence only)
New column R 'Whitefields rate' on '2. Rates' with the Whitefields
demolition contract (Total Reclaims, GBP 525,676; AFC GBP 532,445 at
FS 16, Jul 2026) on the workbook basis (x 1.014 / 0.94, excl. the
contractor's prelims and OH&P): 0.1 asbestos 10.1, 0.2 demolition incl.
service disconnections 91.4, 0.7 service diversions 40.2, 8.10 soft
landscaping 2.2. WF lines added to Tender check, an Instructions note
for column R, the v5.9 log line and version. No rate, option, rule or
formula changed; the app does not read the new column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ThEE8jqhmBASGLx3pT6ipD
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4217" uniqueCount="1730">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4226" uniqueCount="1744">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5221,6 +5221,48 @@
   </si>
   <si>
     <t xml:space="preserve">Evidence only, no rates changed. Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; mean of two bids × 1.07 ÷ 0.94, on about 4,170 m² GIA and 699 m² of roof) added to the Tender check column for 2.5a roof, 2.6 external walls, 2.7 windows (with the scaffold figure), 5.1b air source heat pump, 5.26a builder's work and 7.1a repairs. The Tender check header and its note above now cover more than one project. Suggested for the owner to decide: roof Std about £300 (Computer Science £313, Claycroft £627–£704); air source heat pump full system Std about £150; a scaffold item of about £35/m² GIFA for envelope works; triple glazing priced at High. Updated 2 Oct 2026 with the final out-turn and CPW's heat pump sizes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender check (this row's unit, on this workbook's basis. Unlabelled = Lakeside S&amp;F, Sep 2026: median of 4 bids ÷ 0.94. CS = Computer Science decarbonisation, Mar 2024: 2 bids × 1.07 ÷ 0.94. WF = Whitefields demolition, Total Reclaims contract 2026: line items × 1.014 ÷ 0.94 — the figure is also in column R)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whitefields rate (£ per this row's unit, this workbook's basis: Total Reclaims contract 2026, excl. the contractor's prelims and OH&amp;P, ÷ 0.94 × 1.014. Evidence only — the app does not read it)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WF: £10.1 on the contract (Total Reclaims, £28,050 to the asbestos BoQ) over 3,000 m² GIA assumed (1,995 m² measured footprint × 1.5 storeys). Five bids on the same BoQ: £10.1–£53, median £15.8. The R&amp;D survey (£9,400) was a fee.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WF: £91 per m² demolished on the contract, 3,000 m² GIA assumed (1,995 m² measured footprint × 1.5 storeys): soft strip, demolish, slabs and foundations £43; disconnecting and cutting back drainage, water, gas, electrical and telecoms, plus Trinity / Honeywell fire alarm, security and metering removal, £49. Core demolition across five bids £43–£87 (median £57). Excludes the water-main replacement (0.7) and the contractor's own £15k provisional sums for the Trinity / Honeywell work, which those quotes replace.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WF: £40 per m² footprint on the contract (1,995 m² footprint): replacing the ductile iron water main that crosses the site in MDPE, with temporary water, trenching, stone surround and tarmac reinstatement (£74k). £49 with the changes pending at FS 16, Jul 2026 (trial pits on the district heating and water mains, out-of-hours water works: £16.7k).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WF: £2.2 per m² over the 7,715 m² red line (contract £15.4k): topsoil and grass seed to the UoW Grounds specification only — no planting or maintenance. Five bids £2.2–£11.7, median £3.4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.9 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lakeside Staff &amp; Family Flats tender returns (29 Sept 2026) converted to this workbook's basis: the median of the four credible bids (BSN, Chiel, Harrabin, William Gough with its kitchen error corrected; Watkin Jones excluded at twice the field) ÷ 0.94 West Midlands factor, per this row's unit, on 3,306 m² measured floor area (49 flats, the Warden's house and nine stair cores). Excludes the contractors' preliminaries and OH&amp;P. Lines starting 'CS:' are the Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; two bids, so the mean): tender × 1.07 (to Q3 2026) ÷ 0.94, on about 4,170 m² GIA measured from the tender plans and 699 m² of roof. Evidence only: no rate was changed for them in v5.8. Final out-turn (financial statement, July 2026): construction £2.73m, +3.4% on a £2.64m contract; total project £3.13m excl. VAT. WF lines: Whitefields demolition (17 blocks, UoW main campus), the Total Reclaims contract (tendered Feb 2026, Option 2) — the figure is also in column R, Whitefields rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whitefields rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column R on '2. Rates': the Whitefields demolition contract figure for that row (Total Reclaims, £525,676; AFC £532,445 at FS 16, Jul 2026), in the row's unit and on this workbook's basis — line items without the contractor's prelims and OH&amp;P, ÷ 0.94 West Midlands factor, × 1.014 to Q3 2026. m² GIFA and m² demolished use 3,000 m² GIA (assumed: 1,995 m² measured footprint × 1.5 storeys); m² footprint uses 1,995 m²; soft landscaping uses the 7,715 m² red line. Evidence only: the app does not read this column and no rate changed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v5.9 — 2 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence only, no rates changed. New column R 'Whitefields rate' on '2. Rates' and WF lines in Tender check, from the Whitefields demolition contract (Total Reclaims £525,676; AFC £532,445 at FS 16, Jul 2026; 3,000 m² GIA assumed): 0.1 asbestos £10.1/m² GIFA; 0.2 demolition incl. disconnections £91/m² demolished; 0.7 service diversions £40/m² footprint (water-main replacement); 8.10 topsoil and seed £2.2/m². Not on '2. Rates': the contractor's prelims incl. hoarding were 16.8% of works and OH&amp;P 15%; professional fees 28% of construction (ecology and environmental monitoring £67k), UoW Estates fees 4%, contingency 7%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-02</t>
   </si>
 </sst>
 </file>
@@ -5841,7 +5883,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BBCD35-3C7D-4CAC-A46E-6C3CC3E31849}">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.7109375" style="8" customWidth="1"/>
@@ -5852,7 +5894,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1720</v>
+        <v>1736</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -6019,13 +6061,17 @@
         <v>1708</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>1728</v>
+        <v>1737</v>
       </c>
       <c r="C21" s="33"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="15"/>
-      <c r="B22" s="17"/>
+    <row r="22" spans="1:3" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="15" t="s">
+        <v>1738</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>1739</v>
+      </c>
       <c r="C22" s="33"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -6515,109 +6561,118 @@
       <c r="B78" s="16"/>
       <c r="C78" s="34"/>
     </row>
-    <row r="79" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="17" t="s">
-        <v>1722</v>
+        <v>1740</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>1729</v>
+        <v>1741</v>
       </c>
       <c r="C79" s="60"/>
     </row>
     <row r="80" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A80" s="17" t="s">
-        <v>1711</v>
+        <v>1722</v>
       </c>
       <c r="B80" s="17" t="s">
-        <v>1712</v>
+        <v>1729</v>
       </c>
       <c r="C80" s="60"/>
     </row>
     <row r="81" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A81" s="17" t="s">
+        <v>1711</v>
+      </c>
+      <c r="B81" s="17" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C81" s="60"/>
+    </row>
+    <row r="82" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A82" s="17" t="s">
         <v>1632</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B82" s="17" t="s">
         <v>1634</v>
       </c>
-      <c r="C81" s="60"/>
-    </row>
-    <row r="82" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A82" s="15" t="s">
+      <c r="C82" s="60"/>
+    </row>
+    <row r="83" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A83" s="15" t="s">
         <v>1620</v>
       </c>
-      <c r="B82" s="17" t="s">
+      <c r="B83" s="17" t="s">
         <v>1621</v>
       </c>
-      <c r="C82" s="33"/>
-    </row>
-    <row r="83" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A83" s="15" t="s">
+      <c r="C83" s="33"/>
+    </row>
+    <row r="84" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A84" s="15" t="s">
         <v>1060</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B84" s="17" t="s">
         <v>1061</v>
       </c>
-      <c r="C83" s="33"/>
-    </row>
-    <row r="84" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A84" s="15" t="s">
+      <c r="C84" s="33"/>
+    </row>
+    <row r="85" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A85" s="15" t="s">
         <v>1051</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B85" s="17" t="s">
         <v>1052</v>
       </c>
-      <c r="C84" s="33"/>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A85" s="15" t="s">
+      <c r="C85" s="33"/>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B86" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C85" s="33"/>
-    </row>
-    <row r="86" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A86" s="15" t="s">
+      <c r="C86" s="33"/>
+    </row>
+    <row r="87" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A87" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B87" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C86" s="33"/>
-    </row>
-    <row r="87" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A87" s="15" t="s">
+      <c r="C87" s="33"/>
+    </row>
+    <row r="88" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A88" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B87" s="17" t="s">
+      <c r="B88" s="17" t="s">
         <v>28</v>
-      </c>
-      <c r="C87" s="33"/>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A88" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B88" s="17" t="s">
-        <v>30</v>
       </c>
       <c r="C88" s="33"/>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B89" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C89" s="33"/>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="B90" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C89" s="33"/>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A90" s="15"/>
-      <c r="B90" s="17"/>
       <c r="C90" s="33"/>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" s="15"/>
+      <c r="B91" s="17"/>
+      <c r="C91" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6626,7 +6681,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61613224-FE41-4C03-8B46-4109509C3076}">
-  <dimension ref="A1:Q152"/>
+  <dimension ref="A1:R152"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.7109375" style="8" customWidth="1"/>
@@ -6643,7 +6698,8 @@
     <col min="15" max="15" width="11.7109375" style="8" customWidth="1"/>
     <col min="16" max="16" width="25.85546875" style="8" customWidth="1"/>
     <col min="17" max="17" width="44.7109375" style="8" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="8"/>
+    <col min="18" max="18" width="16.7109375" style="8" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="18" x14ac:dyDescent="0.25">
@@ -6661,7 +6717,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>756</v>
       </c>
@@ -6711,7 +6767,10 @@
         <v>1623</v>
       </c>
       <c r="Q5" s="12" t="s">
-        <v>1719</v>
+        <v>1730</v>
+      </c>
+      <c r="R5" s="12" t="s">
+        <v>1731</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -6733,7 +6792,7 @@
       <c r="N6" s="19"/>
       <c r="O6" s="20"/>
     </row>
-    <row r="7" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
         <v>72</v>
       </c>
@@ -6771,8 +6830,14 @@
       <c r="O7" s="24" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="Q7" s="22" t="s">
+        <v>1732</v>
+      </c>
+      <c r="R7" s="22">
+        <v>10.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
         <v>82</v>
       </c>
@@ -6810,6 +6875,12 @@
       <c r="O8" s="24" t="s">
         <v>73</v>
       </c>
+      <c r="Q8" s="22" t="s">
+        <v>1733</v>
+      </c>
+      <c r="R8" s="22">
+        <v>91.4</v>
+      </c>
     </row>
     <row r="9" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
@@ -6968,7 +7039,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
         <v>119</v>
       </c>
@@ -7003,6 +7074,12 @@
       <c r="N13" s="22"/>
       <c r="O13" s="24" t="s">
         <v>113</v>
+      </c>
+      <c r="Q13" s="22" t="s">
+        <v>1734</v>
+      </c>
+      <c r="R13" s="22">
+        <v>40.2</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -12692,7 +12769,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="145" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:18" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A145" s="21" t="s">
         <v>696</v>
       </c>
@@ -12735,6 +12812,12 @@
       </c>
       <c r="O145" s="24" t="s">
         <v>697</v>
+      </c>
+      <c r="Q145" s="22" t="s">
+        <v>1735</v>
+      </c>
+      <c r="R145" s="22">
+        <v>2.2</v>
       </c>
     </row>
     <row r="146" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -13113,7 +13196,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>1724</v>
+        <v>1742</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -13124,7 +13207,7 @@
         <v>751</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>1725</v>
+        <v>1743</v>
       </c>
       <c r="C7" s="2"/>
     </row>

</xml_diff>

<commit_message>
NRM1 v5.10: Claycroft refurbishment rate column (evidence only)
New column S "Claycroft rate" on '2. Rates' with the Claycroft student
residences refurbishment figures (Morgan Sindall G4 contract, May 2025)
on the workbook basis: sub-contract packages excl. MS prelims, risk, fee
and design, x 1.034 / 0.94, on 17,172 m2 GIA measured from the Estates
fire plans. 2.10 fire stopping uses the Mace Val 16 forecast out-turn.
18 rows filled, matching "CC:" lines in Tender check, an Instructions
row for column S and a v5.10 log line. Version 5.10 on workbook_info.

No rate, option, rule or formula changed; the app ignores column S.
Self-checks all 0 after LibreOffice recalculation; 82 items, 139 rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MHuyNRuSD5TFNxmRibMe2
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4226" uniqueCount="1752">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4236" uniqueCount="1782">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5287,6 +5287,96 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender check (this row's unit, on this workbook's basis. Unlabelled = Lakeside S&amp;F, Sep 2026: median of 4 bids ÷ 0.94. CS = Computer Science decarbonisation, Mar 2024: 2 bids × 1.07 ÷ 0.94. WF = Whitefields demolition, Total Reclaims contract 2026: line items × 1.014 ÷ 0.94 — the figure is also in column R. CC = Claycroft refurbishment, Morgan Sindall G4 contract May 2025: packages × 1.034 ÷ 0.94 — the figure is also in column S)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claycroft rate (£ per this row's unit, this workbook's basis: Morgan Sindall G4 contract, May 2025 — sub-contract packages excl. Morgan Sindall's prelims, risk, fee and design, × 1.034 ÷ 0.94, on 17,172 m² GIA measured. 2.10 fire stopping is the forecast out-turn (Mace Val 16, Sep 2026). Evidence only — the app does not read it)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£54 (bids £36–£56) for a partial strip-out: finishes, fittings, redundant electrics and protection CC: £51.4 on the Claycroft G4 contract (Cawarden, £801,990): full strip-out of three occupied student blocks, 17,172 m² GIA. Three bids £802k–£928k.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loft insulation only: £32 — see 2.5b. CS: £313 (bids £288–£338) per m² of roof re-covered (699 m², less than the footprint) for a flat warm-roof overlay on the kept asphalt: AVCL, 120 mm PIR, two-layer felt, insulated upstands, new copings, ballast relaid. Scaffold extra (see 2.7). Claycroft pitched re-roof £627–£704. CC: £517 per m² of roof plan (5,747 m² footprint) on the G4 contract: strip concrete tiles, top-hat spacers, Euroclad secret-fix metal over-roof, hips and verges, new eaves, gutters and soffits (£596 per m of eaves), incl. Metclad's design and prelims; excl. the bay-window cladding and scaffold (scaffold £99 per m² of plan). Forecast out-turn with roof timber remedials £601. Tiled like-for-like alternative about £460 (Stage 3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£13.5 (bids £7–£32) for local fire stopping only — in line with Basic £15 CC: £96 forecast out-turn (Mace Val 16, Sep 2026; £88 if the Claycroft 2 CE replaces its provisional sum), against £22 for the £350k provisional sum in the G4 contract. By block: Claycroft 1 £53 (final); Claycroft 3 £76 (measured: about 18 seals per bed at about £42 each; access 22% of the cost); Claycroft 2 £135–£155 (under review). Excludes £1.30m of compartment-wall head remediation on Claycroft 3, which included a 16-week delay.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£72 (bids £60–£84) incl. bathroom wall cladding, kitchen tiling and full redecoration — confirms £75 CC: £99 on the G4 contract: decoration (RE Martin, £1.02m; three bids £1.02m–£1.16m), making good (£274k) and PVC hygienic wall cladding (£251k). Includes painting ceilings and doors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£51 (bids £48–£59). New build columns copied from 3.2a CC: £38 on the G4 contract: carpet and vinyl (Active, £506k; three bids £506k–£660k), Claycroft 2 corridor and lobby floors (£88k) and screed (£4.5k).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£30 (bids £21–£36). New build columns copied from 3.3a CC: £70 on the G4 contract: ceilings and partitions package (Ace, £1.10m; three bids £1.10m–£1.23m) — replacement plasterboard ceilings (two layers of fire-line board on top floors), stair soffits and some partitions, not split. Claycroft replaced its ceilings, so compare with 3.3a.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£2,563 per bathroom (bids £2,322–£4,440); standard suite alone £2,460. New build columns not changed CC: £3,869 per bathroom on the G4 contract, Claycroft 1 (135 bathroom units): IPS and vanity (Inscape) plus WC, basin and bath with taps, incl. assisted-bathroom changes. Water and drainage connections are in 5.2a; PVC wall cladding is in 3.1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC: £64 on the G4 contract: joinery package (Mansard, £994k; two bids £994k–£1.04m) — bathroom joinery (boxings, bath panels, shelves) 67%, bedroom joinery (wardrobe alterations, shelving) 21%, other incl. signage 12%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC: £39 on the G4 contract: domestic hot and cold water (riser pipework and valves, bathroom connections, DHW plate heat exchangers and pumps) and drainage (bathroom connections to stacks, SVP terminations). A partial replacement, not a full installation. Sanitaryware is in 4.2a.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Residential extract-only scope: £18.5 — see 5.3b CC: forecast out-turn £92 (Mace Val 16) for bathroom extract incl. new ductwork and roof-mounted fans added by CE in Claycroft 1 (£182k) and Claycroft 2 (£865k). The contract figure is on 5.3b.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£18.5 (bids £13–£23), incl. the electrical connection to each fan CC: £28 on the G4 contract: new branch connections, dampers and grilles to the existing bathroom extract, duct cleaning and flow checks, plus fire dampers (£124k). Forecast out-turn £92 once new ductwork and roof fans were added — see 5.3a.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC: £4.3 on the G4 contract: interfaces from the existing BEMS to the new fire alarm and DHW controls only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power + lighting £186 (bids £157–£253) less lighting 5.8a £33 = £153; incl. landlord panels and sub-mains per block. New build columns not changed CC: £158 on the G4 contract: full rewire — LV switch panels and distribution boards (£1.10m), containment (£366k), small power (£669k), isolation and strip-out of the old installation (£158k) and earthing. Electrical total with lighting, fire alarm and data: £355.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not separable in the tender — checked together with 5.7b CC: £113 on the G4 contract for general, emergency and external lighting together (£1.66m, not split) — compare with 5.8a + 5.9 (£33 + £10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£18.6 (bids £18–£21), residential — confirms £18 CC: £65 on the G4 contract: new fire alarm throughout three blocks of student flats (£949k). Disabled refuge and assisted-WC alarms add £8.5 (not in this figure).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£24.5 incl. TV aerial system (bids £22–£39). New build columns copied from 5.14a CC: £19 on the G4 contract: voice and data (£284k); no TV aerial system.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not comparable: the tender only had doorbells and door-entry infrastructure CC: £4.5 on the G4 contract: access control (£52k) and CCTV (£14k) only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC: £112,850 per lift on the G4 contract: one passenger lift removed and replaced in Claycroft 3 (Morris Vermaport, £102,588 incl. design).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£27 (bids £18–£55): chasing and making good for a full rewire of occupied flats. New build columns copied from 5.26a CC: £11 on the G4 contract: builder's work assessed by Morgan Sindall at 2.2% of M&amp;E (£172k); more builder's work is priced inside the M&amp;E lines.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC: no contract figure. The forecast out-turn (Mace Val 16) adds £2.65m of structural and fabric defect remediation, £164 on this basis — mostly a £2.14m budget for Claycroft 2, found only as each block was opened up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.10 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lakeside Staff &amp; Family Flats tender returns (29 Sept 2026) converted to this workbook's basis: the median of the four credible bids (BSN, Chiel, Harrabin, William Gough with its kitchen error corrected; Watkin Jones excluded at twice the field) ÷ 0.94 West Midlands factor, per this row's unit, on 3,306 m² measured floor area (49 flats, the Warden's house and nine stair cores). Excludes the contractors' preliminaries and OH&amp;P. Lines starting 'CS:' are the Computer Science Building decarbonisation tender returns (Harrabin and Chiel, March 2024; two bids, so the mean): tender × 1.07 (to Q3 2026) ÷ 0.94, on 3,495 m² GIA (UoW Estates CAD outlines) and 699 m² of roof. Evidence only: no rate was changed for them in v5.8. Final out-turn (financial statement, July 2026): construction £2.73m, +3.4% on a £2.64m contract; total project £3.13m excl. VAT. WF lines: Whitefields demolition (17 blocks, UoW main campus), the Total Reclaims contract (tendered Feb 2026, Option 2) — the figure is also in column R, Whitefields rate. CC lines: the Claycroft student residences refurbishment (679 beds, three occupied blocks, UoW main campus), Morgan Sindall G4 contract (May 2025, SCAPE) — the figure is also in column S, Claycroft rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claycroft rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column S on '2. Rates': the Claycroft student residences refurbishment figure for that row (Morgan Sindall, Tier 1, SCAPE Lot 4, NEC ECC; G4 contract £20,955,523, May 2025), in the row's unit and on this workbook's basis — sub-contract package values without Morgan Sindall's prelims, risk, fee and design, × 1.034 to Q3 2026, ÷ 0.94 West Midlands factor. m² GIFA uses 17,172 m² GIA and m² roof the 5,747 m² footprint, both measured from the UoW Estates fire plans; bathrooms use Claycroft 1 (135 bathroom units). M&amp;E rows include their share (6.5%) of the M&amp;E design, prelims and testing. 2.10 fire stopping is the forecast out-turn (Mace Val 16, Sep 2026; ÷ 0.94, not rebased), because the contract held only a £350k provisional sum. Evidence only: the app does not read this column and no rate changed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v5.10 — 3 Oct 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence only, no rates changed. New column S 'Claycroft rate' on '2. Rates' and CC lines in Tender check, from the Claycroft refurbishment (Morgan Sindall G4 contract £20.96m, May 2025; Mace Val 16 forecast final account £27.96m, +33%; 17,172 m² GIA measured, 679 beds): strip-out £51; metal over-roof £517/m² roof; fire stopping £96 (out-turn); wall finishes £99; floor finishes £38; ceilings £70; bathrooms £3,869 each; fixed joinery £64; water and drainage £39; extract £28; power £158; lighting incl. emergency £113; fire alarm £65; data £19; passenger lift £112,850; BWIC £11. Not on '2. Rates': scaffold £33/m² GIA; Morgan Sindall prelims 11.3% of works, fee 2.2%, risk 2.8%, design 2.1%; client risk and contingency 21.5% of contract, exceeded by the forecast growth (structural and fabric defects £2.65m, fire stopping incl. compartment-wall heads £2.63m, M&amp;E £1.40m, roof £0.55m).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-03</t>
   </si>
 </sst>
 </file>
@@ -5907,7 +5997,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BBCD35-3C7D-4CAC-A46E-6C3CC3E31849}">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.7109375" style="8" customWidth="1"/>
@@ -5918,7 +6008,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1744</v>
+        <v>1774</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -6080,12 +6170,12 @@
       </c>
       <c r="C20" s="33"/>
     </row>
-    <row r="21" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" ht="142.25" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
         <v>1708</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>1745</v>
+        <v>1775</v>
       </c>
       <c r="C21" s="33"/>
     </row>
@@ -6098,605 +6188,623 @@
       </c>
       <c r="C22" s="33"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="13" t="s">
+    <row r="23" spans="1:3" ht="91.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="15" t="s">
+        <v>1776</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>1777</v>
+      </c>
+      <c r="C23" s="33"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="13" t="s">
         <v>1568</v>
       </c>
-      <c r="B23" s="16"/>
-      <c r="C23" s="34"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="15" t="s">
-        <v>1076</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>1569</v>
-      </c>
-      <c r="C24" s="33"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="34"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="15" t="s">
-        <v>1098</v>
+        <v>1076</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>1570</v>
+        <v>1569</v>
       </c>
       <c r="C25" s="33"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="15" t="s">
-        <v>1118</v>
+        <v>1098</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>1571</v>
+        <v>1570</v>
       </c>
       <c r="C26" s="33"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="15" t="s">
-        <v>1179</v>
+        <v>1118</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>1572</v>
+        <v>1571</v>
       </c>
       <c r="C27" s="33"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="15" t="s">
-        <v>1174</v>
+        <v>1179</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>1573</v>
+        <v>1572</v>
       </c>
       <c r="C28" s="33"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="15" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>1573</v>
+      </c>
+      <c r="C29" s="33"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="15" t="s">
         <v>1637</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B30" s="17" t="s">
         <v>1710</v>
       </c>
-      <c r="C29" s="33"/>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="15"/>
-      <c r="B30" s="17"/>
       <c r="C30" s="33"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="15"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="33"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="16"/>
-      <c r="C31" s="34"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="15" t="s">
-        <v>1574</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>1575</v>
-      </c>
-      <c r="C32" s="33"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="34"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="15" t="s">
-        <v>8</v>
+        <v>1574</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>1576</v>
+        <v>1575</v>
       </c>
       <c r="C33" s="33"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="15" t="s">
-        <v>1577</v>
+        <v>8</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>1578</v>
+        <v>1576</v>
       </c>
       <c r="C34" s="33"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="15" t="s">
-        <v>1579</v>
-      </c>
-      <c r="B35" s="32" t="s">
-        <v>1580</v>
+        <v>1577</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>1578</v>
       </c>
       <c r="C35" s="33"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="15" t="s">
-        <v>1581</v>
+        <v>1579</v>
       </c>
       <c r="B36" s="32" t="s">
-        <v>1582</v>
+        <v>1580</v>
       </c>
       <c r="C36" s="33"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="B37" s="17" t="s">
-        <v>1583</v>
+        <v>1581</v>
+      </c>
+      <c r="B37" s="32" t="s">
+        <v>1582</v>
       </c>
       <c r="C37" s="33"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>1583</v>
+      </c>
+      <c r="C38" s="33"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="B39" s="17" t="s">
         <v>1584</v>
       </c>
-      <c r="C38" s="33"/>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="15"/>
-      <c r="B39" s="17"/>
       <c r="C39" s="33"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="13" t="s">
+      <c r="A40" s="15"/>
+      <c r="B40" s="17"/>
+      <c r="C40" s="33"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="13" t="s">
         <v>1585</v>
       </c>
-      <c r="B40" s="16"/>
-      <c r="C40" s="34"/>
-    </row>
-    <row r="41" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A41" s="15" t="s">
-        <v>1586</v>
-      </c>
-      <c r="B41" s="17" t="s">
-        <v>1587</v>
-      </c>
-      <c r="C41" s="33"/>
+      <c r="B41" s="16"/>
+      <c r="C41" s="34"/>
     </row>
     <row r="42" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A42" s="15" t="s">
+        <v>1586</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>1587</v>
+      </c>
+      <c r="C42" s="33"/>
+    </row>
+    <row r="43" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A43" s="15" t="s">
         <v>1588</v>
       </c>
-      <c r="B42" s="17" t="s">
+      <c r="B43" s="17" t="s">
         <v>3</v>
-      </c>
-      <c r="C42" s="33"/>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="15" t="s">
-        <v>1589</v>
-      </c>
-      <c r="B43" s="17" t="s">
-        <v>1590</v>
       </c>
       <c r="C43" s="33"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="15" t="s">
-        <v>1591</v>
+        <v>1589</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>1592</v>
+        <v>1590</v>
       </c>
       <c r="C44" s="33"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="15" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B45" s="17" t="s">
+        <v>1592</v>
+      </c>
+      <c r="C45" s="33"/>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="B45" s="17" t="s">
+      <c r="B46" s="17" t="s">
         <v>1593</v>
       </c>
-      <c r="C45" s="33"/>
-    </row>
-    <row r="46" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A46" s="15" t="s">
+      <c r="C46" s="33"/>
+    </row>
+    <row r="47" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A47" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="B46" s="17" t="s">
+      <c r="B47" s="17" t="s">
         <v>1633</v>
       </c>
-      <c r="C46" s="33"/>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="15" t="s">
+      <c r="C47" s="33"/>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B48" s="17" t="s">
         <v>1594</v>
-      </c>
-      <c r="C47" s="33"/>
-    </row>
-    <row r="48" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A48" s="15" t="s">
-        <v>1595</v>
-      </c>
-      <c r="B48" s="17" t="s">
-        <v>1596</v>
       </c>
       <c r="C48" s="33"/>
     </row>
     <row r="49" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A49" s="15" t="s">
+        <v>1595</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>1596</v>
+      </c>
+      <c r="C49" s="33"/>
+    </row>
+    <row r="50" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A50" s="15" t="s">
         <v>1597</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B50" s="17" t="s">
         <v>1598</v>
-      </c>
-      <c r="C49" s="33"/>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="15" t="s">
-        <v>1599</v>
-      </c>
-      <c r="B50" s="17" t="s">
-        <v>1600</v>
       </c>
       <c r="C50" s="33"/>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="15" t="s">
-        <v>1601</v>
+        <v>1599</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>1602</v>
+        <v>1600</v>
       </c>
       <c r="C51" s="33"/>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="15" t="s">
+        <v>1601</v>
+      </c>
+      <c r="B52" s="17" t="s">
+        <v>1602</v>
+      </c>
+      <c r="C52" s="33"/>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B52" s="17" t="s">
+      <c r="B53" s="17" t="s">
         <v>1603</v>
       </c>
-      <c r="C52" s="33"/>
-    </row>
-    <row r="53" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A53" s="15" t="s">
+      <c r="C53" s="33"/>
+    </row>
+    <row r="54" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A54" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B53" s="17" t="s">
+      <c r="B54" s="17" t="s">
         <v>1604</v>
-      </c>
-      <c r="C53" s="33"/>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" s="15" t="s">
-        <v>1605</v>
-      </c>
-      <c r="B54" s="17" t="s">
-        <v>1606</v>
       </c>
       <c r="C54" s="33"/>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="15" t="s">
-        <v>46</v>
+        <v>1605</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="C55" s="33"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="15" t="s">
-        <v>1608</v>
+        <v>46</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>1609</v>
+        <v>1607</v>
       </c>
       <c r="C56" s="33"/>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="15" t="s">
+        <v>1608</v>
+      </c>
+      <c r="B57" s="17" t="s">
+        <v>1609</v>
+      </c>
+      <c r="C57" s="33"/>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="B57" s="17" t="s">
+      <c r="B58" s="17" t="s">
         <v>1610</v>
       </c>
-      <c r="C57" s="33"/>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="15"/>
-      <c r="B58" s="17"/>
       <c r="C58" s="33"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="13" t="s">
+      <c r="A59" s="15"/>
+      <c r="B59" s="17"/>
+      <c r="C59" s="33"/>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B59" s="16"/>
-      <c r="C59" s="34"/>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="15" t="s">
+      <c r="B60" s="16"/>
+      <c r="C60" s="34"/>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="15" t="s">
         <v>1611</v>
       </c>
-      <c r="B60" s="17"/>
-      <c r="C60" s="33">
+      <c r="B61" s="17"/>
+      <c r="C61" s="33">
         <f>SUMPRODUCT(('2. Rates'!O6:O152&lt;&gt;"")*(COUNTIF('2. Rates'!O6:O152,'2. Rates'!O6:O152)&gt;1))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="15" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="15" t="s">
         <v>1612</v>
       </c>
-      <c r="B61" s="17"/>
-      <c r="C61" s="33">
+      <c r="B62" s="17"/>
+      <c r="C62" s="33">
         <f>SUMPRODUCT(('2. Rates'!O6:O152&lt;&gt;"")*(COUNTIF('4. Scope rules'!A91:A229,'2. Rates'!O6:O152)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="15" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="15" t="s">
         <v>1613</v>
       </c>
-      <c r="B62" s="17"/>
-      <c r="C62" s="33">
+      <c r="B63" s="17"/>
+      <c r="C63" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A91:A229&lt;&gt;"")*(COUNTIF('2. Rates'!O6:O152,'4. Scope rules'!A91:A229)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="15" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="15" t="s">
         <v>1614</v>
       </c>
-      <c r="B63" s="17"/>
-      <c r="C63" s="33">
+      <c r="B64" s="17"/>
+      <c r="C64" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A91:A229&lt;&gt;"")*(COUNTIF('4. Scope rules'!A6:A87,'4. Scope rules'!B91:B229)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="15" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="15" t="s">
         <v>1615</v>
       </c>
-      <c r="B64" s="17"/>
-      <c r="C64" s="33">
+      <c r="B65" s="17"/>
+      <c r="C65" s="33">
         <f>SUMPRODUCT(('2. Rates'!O6:O152&lt;&gt;"")*('2. Rates'!M6:M152=""))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="15" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="15" t="s">
         <v>1616</v>
       </c>
-      <c r="B65" s="17"/>
-      <c r="C65" s="33">
+      <c r="B66" s="17"/>
+      <c r="C66" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*(ROUND('4. Scope rules'!M6:M87+'4. Scope rules'!O6:O87,4)&lt;&gt;1))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="15" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="33">
+      <c r="B67" s="17"/>
+      <c r="C67" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*(COUNTIFS('4. Scope rules'!B91:B229,'4. Scope rules'!A6:A87,'4. Scope rules'!E91:E229,"Yes")=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" s="15" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="15" t="s">
         <v>1617</v>
       </c>
-      <c r="B67" s="17"/>
-      <c r="C67" s="33">
+      <c r="B68" s="17"/>
+      <c r="C68" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*('4. Scope rules'!F6:F87="One")*(COUNTIFS('4. Scope rules'!B91:B229,'4. Scope rules'!A6:A87,'4. Scope rules'!E91:E229,"Yes")&gt;1))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="15" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="15" t="s">
         <v>1618</v>
       </c>
-      <c r="B68" s="17"/>
-      <c r="C68" s="33">
+      <c r="B69" s="17"/>
+      <c r="C69" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*('4. Scope rules'!G6:G87=""))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="15" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B69" s="17"/>
-      <c r="C69" s="33">
+      <c r="B70" s="17"/>
+      <c r="C70" s="33">
         <f>SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('4. Scope rules'!H6:H87,"NB",""),"EX",""),"RF",""),"FO",""),"EW",""),"DM",""),"OM",""),"—","")))&gt;0))+SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('4. Scope rules'!I6:I87,"NB",""),"EX",""),"RF",""),"FO",""),"EW",""),"DM",""),"OM",""),"—","")))&gt;0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="15" t="s">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B70" s="17"/>
-      <c r="C70" s="33">
+      <c r="B71" s="17"/>
+      <c r="C71" s="33">
         <f>SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('4. Scope rules'!J6:J87,"RES",""),"STU",""),"OFF",""),"EDU",""),"HEA",""),"RET",""),"IND",""),"HOS",""),"MIX",""),"OTH",""),"ALL","")))&gt;0))+SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('2. Rates'!D6:D152,"RES",""),"STU",""),"OFF",""),"EDU",""),"HEA",""),"RET",""),"IND",""),"HOS",""),"MIX",""),"OTH",""),"ALL","")))&gt;0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="15" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B71" s="17"/>
-      <c r="C71" s="33">
+      <c r="B72" s="17"/>
+      <c r="C72" s="33">
         <f>SUMPRODUCT(('3. Settings'!A96:A123&lt;&gt;"")*(COUNTIFS('3. Settings'!A96:A123,'3. Settings'!A96:A123,'3. Settings'!B96:B123,"ALL")=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="15" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B72" s="17"/>
-      <c r="C72" s="33">
+      <c r="B73" s="17"/>
+      <c r="C73" s="33">
         <f>SUMPRODUCT(('3. Settings'!A96:A123&lt;&gt;"")*('3. Settings'!C96:C123=""))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A73" s="15"/>
-      <c r="B73" s="17"/>
-      <c r="C73" s="33"/>
-    </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="13" t="s">
+      <c r="A74" s="15"/>
+      <c r="B74" s="17"/>
+      <c r="C74" s="33"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B74" s="16"/>
-      <c r="C74" s="34"/>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="15" t="s">
+      <c r="B75" s="16"/>
+      <c r="C75" s="34"/>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B75" s="17"/>
-      <c r="C75" s="33">
+      <c r="B76" s="17"/>
+      <c r="C76" s="33">
         <f>COUNTA('4. Scope rules'!A6:A87)</f>
         <v>82</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" s="15" t="s">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="15" t="s">
         <v>1619</v>
       </c>
-      <c r="B76" s="17"/>
-      <c r="C76" s="33">
+      <c r="B77" s="17"/>
+      <c r="C77" s="33">
         <f>COUNTA('2. Rates'!O6:O152)</f>
         <v>139</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="15"/>
-      <c r="B77" s="17"/>
-      <c r="C77" s="33"/>
-    </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A78" s="13" t="s">
+      <c r="A78" s="15"/>
+      <c r="B78" s="17"/>
+      <c r="C78" s="33"/>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B78" s="16"/>
-      <c r="C78" s="34"/>
-    </row>
-    <row r="79" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="17" t="s">
+      <c r="B79" s="16"/>
+      <c r="C79" s="34"/>
+    </row>
+    <row r="80" spans="1:3" s="54" customFormat="1" ht="104.0" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="17" t="s">
+        <v>1778</v>
+      </c>
+      <c r="B80" s="17" t="s">
+        <v>1779</v>
+      </c>
+      <c r="C80" s="60"/>
+    </row>
+    <row r="81" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="17" t="s">
         <v>1748</v>
       </c>
-      <c r="B79" s="17" t="s">
+      <c r="B81" s="17" t="s">
         <v>1749</v>
-      </c>
-      <c r="C79" s="60"/>
-    </row>
-    <row r="80" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A80" s="17" t="s">
-        <v>1722</v>
-      </c>
-      <c r="B80" s="17" t="s">
-        <v>1737</v>
-      </c>
-      <c r="C80" s="60"/>
-    </row>
-    <row r="81" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A81" s="17" t="s">
-        <v>1711</v>
-      </c>
-      <c r="B81" s="17" t="s">
-        <v>1712</v>
       </c>
       <c r="C81" s="60"/>
     </row>
     <row r="82" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A82" s="17" t="s">
+        <v>1722</v>
+      </c>
+      <c r="B82" s="17" t="s">
+        <v>1737</v>
+      </c>
+      <c r="C82" s="60"/>
+    </row>
+    <row r="83" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A83" s="17" t="s">
+        <v>1711</v>
+      </c>
+      <c r="B83" s="17" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C83" s="60"/>
+    </row>
+    <row r="84" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A84" s="17" t="s">
         <v>1632</v>
       </c>
-      <c r="B82" s="17" t="s">
+      <c r="B84" s="17" t="s">
         <v>1634</v>
       </c>
-      <c r="C82" s="60"/>
-    </row>
-    <row r="83" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A83" s="15" t="s">
+      <c r="C84" s="60"/>
+    </row>
+    <row r="85" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A85" s="15" t="s">
         <v>1620</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B85" s="17" t="s">
         <v>1621</v>
       </c>
-      <c r="C83" s="33"/>
-    </row>
-    <row r="84" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A84" s="15" t="s">
+      <c r="C85" s="33"/>
+    </row>
+    <row r="86" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A86" s="15" t="s">
         <v>1060</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B86" s="17" t="s">
         <v>1061</v>
-      </c>
-      <c r="C84" s="33"/>
-    </row>
-    <row r="85" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A85" s="15" t="s">
-        <v>1051</v>
-      </c>
-      <c r="B85" s="17" t="s">
-        <v>1052</v>
-      </c>
-      <c r="C85" s="33"/>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A86" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="B86" s="17" t="s">
-        <v>24</v>
       </c>
       <c r="C86" s="33"/>
     </row>
     <row r="87" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A87" s="15" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B87" s="17" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C87" s="33"/>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B88" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C88" s="33"/>
+    </row>
+    <row r="89" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A89" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B87" s="17" t="s">
+      <c r="B89" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C87" s="33"/>
-    </row>
-    <row r="88" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A88" s="15" t="s">
+      <c r="C89" s="33"/>
+    </row>
+    <row r="90" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A90" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B88" s="17" t="s">
+      <c r="B90" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C88" s="33"/>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A89" s="15" t="s">
+      <c r="C90" s="33"/>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="B91" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C89" s="33"/>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A90" s="15" t="s">
+      <c r="C91" s="33"/>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B90" s="17" t="s">
+      <c r="B92" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C90" s="33"/>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A91" s="15"/>
-      <c r="B91" s="17"/>
-      <c r="C91" s="33"/>
+      <c r="C92" s="33"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93" s="15"/>
+      <c r="B93" s="17"/>
+      <c r="C93" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6705,7 +6813,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61613224-FE41-4C03-8B46-4109509C3076}">
-  <dimension ref="A1:R152"/>
+  <dimension ref="A1:S152"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.7109375" style="8" customWidth="1"/>
@@ -6723,7 +6831,8 @@
     <col min="16" max="16" width="25.85546875" style="8" customWidth="1"/>
     <col min="17" max="17" width="44.7109375" style="8" customWidth="1"/>
     <col min="18" max="18" width="16.7109375" style="8" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="8"/>
+    <col min="19" max="19" width="16.7109375" style="8" customWidth="1"/>
+    <col min="20" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="18" x14ac:dyDescent="0.25">
@@ -6741,7 +6850,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>756</v>
       </c>
@@ -6791,10 +6900,13 @@
         <v>1623</v>
       </c>
       <c r="Q5" s="12" t="s">
-        <v>1738</v>
+        <v>1752</v>
       </c>
       <c r="R5" s="12" t="s">
         <v>1739</v>
+      </c>
+      <c r="S5" s="12" t="s">
+        <v>1753</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -6906,7 +7018,7 @@
         <v>91.4</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" ht="78.5" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
         <v>96</v>
       </c>
@@ -6945,7 +7057,10 @@
         <v>83</v>
       </c>
       <c r="Q9" s="22" t="s">
-        <v>1665</v>
+        <v>1754</v>
+      </c>
+      <c r="S9" s="22">
+        <v>51.4</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
@@ -7536,7 +7651,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="102" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" ht="218.75" x14ac:dyDescent="0.2">
       <c r="A25" s="21" t="s">
         <v>1669</v>
       </c>
@@ -7583,7 +7698,10 @@
         <v>182</v>
       </c>
       <c r="Q25" s="22" t="s">
-        <v>1713</v>
+        <v>1755</v>
+      </c>
+      <c r="S25" s="22">
+        <v>516.9</v>
       </c>
     </row>
     <row r="26" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
@@ -7815,7 +7933,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:19" ht="155.0" x14ac:dyDescent="0.2">
       <c r="A31" s="21" t="s">
         <v>1146</v>
       </c>
@@ -7858,7 +7976,10 @@
         <v>209</v>
       </c>
       <c r="Q31" s="22" t="s">
-        <v>1677</v>
+        <v>1756</v>
+      </c>
+      <c r="S31" s="22">
+        <v>95.8</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
@@ -7880,7 +8001,7 @@
       <c r="N32" s="26"/>
       <c r="O32" s="27"/>
     </row>
-    <row r="33" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:19" ht="91.25" x14ac:dyDescent="0.2">
       <c r="A33" s="21" t="s">
         <v>221</v>
       </c>
@@ -7925,7 +8046,10 @@
         <v>216</v>
       </c>
       <c r="Q33" s="22" t="s">
-        <v>1678</v>
+        <v>1757</v>
+      </c>
+      <c r="S33" s="22">
+        <v>99.3</v>
       </c>
     </row>
     <row r="34" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
@@ -8025,7 +8149,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:19" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A36" s="23" t="s">
         <v>1655</v>
       </c>
@@ -8071,7 +8195,10 @@
       </c>
       <c r="P36"/>
       <c r="Q36" s="22" t="s">
-        <v>1658</v>
+        <v>1758</v>
+      </c>
+      <c r="S36" s="22">
+        <v>38.4</v>
       </c>
     </row>
     <row r="37" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
@@ -8122,7 +8249,7 @@
         <v>1680</v>
       </c>
     </row>
-    <row r="38" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:19" ht="104.0" x14ac:dyDescent="0.2">
       <c r="A38" s="21" t="s">
         <v>1650</v>
       </c>
@@ -8166,7 +8293,10 @@
       </c>
       <c r="P38"/>
       <c r="Q38" s="22" t="s">
-        <v>1654</v>
+        <v>1759</v>
+      </c>
+      <c r="S38" s="22">
+        <v>70.4</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.2">
@@ -8324,7 +8454,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="43" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:19" ht="104.0" x14ac:dyDescent="0.2">
       <c r="A43" s="48" t="s">
         <v>1175</v>
       </c>
@@ -8370,8 +8500,11 @@
       <c r="O43" s="52" t="s">
         <v>257</v>
       </c>
-      <c r="Q43" s="49" t="s">
-        <v>1666</v>
+      <c r="Q43" s="22" t="s">
+        <v>1760</v>
+      </c>
+      <c r="S43" s="22">
+        <v>3869</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
@@ -8563,7 +8696,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="48" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:19" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A48" s="21" t="s">
         <v>292</v>
       </c>
@@ -8606,6 +8739,12 @@
       </c>
       <c r="O48" s="24" t="s">
         <v>281</v>
+      </c>
+      <c r="Q48" s="22" t="s">
+        <v>1761</v>
+      </c>
+      <c r="S48" s="22">
+        <v>63.7</v>
       </c>
     </row>
     <row r="49" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
@@ -9938,7 +10077,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="78" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:19" ht="91.25" x14ac:dyDescent="0.2">
       <c r="A78" s="23" t="s">
         <v>1299</v>
       </c>
@@ -9983,6 +10122,12 @@
       </c>
       <c r="O78" s="24" t="s">
         <v>415</v>
+      </c>
+      <c r="Q78" s="22" t="s">
+        <v>1762</v>
+      </c>
+      <c r="S78" s="22">
+        <v>38.9</v>
       </c>
     </row>
     <row r="79" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
@@ -10038,7 +10183,7 @@
         <v>1681</v>
       </c>
     </row>
-    <row r="80" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:19" ht="78.5" x14ac:dyDescent="0.2">
       <c r="A80" s="21" t="s">
         <v>1672</v>
       </c>
@@ -10085,10 +10230,10 @@
         <v>424</v>
       </c>
       <c r="Q80" s="22" t="s">
-        <v>1682</v>
-      </c>
-    </row>
-    <row r="81" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+        <v>1763</v>
+      </c>
+    </row>
+    <row r="81" spans="1:19" ht="91.25" x14ac:dyDescent="0.2">
       <c r="A81" s="21" t="s">
         <v>1644</v>
       </c>
@@ -10132,7 +10277,10 @@
       </c>
       <c r="P81"/>
       <c r="Q81" s="22" t="s">
-        <v>1649</v>
+        <v>1764</v>
+      </c>
+      <c r="S81" s="22">
+        <v>28.2</v>
       </c>
     </row>
     <row r="82" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -10180,7 +10328,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="83" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:19" ht="40.25" x14ac:dyDescent="0.2">
       <c r="A83" s="21" t="s">
         <v>373</v>
       </c>
@@ -10224,6 +10372,12 @@
       <c r="O83" s="24" t="s">
         <v>433</v>
       </c>
+      <c r="Q83" s="22" t="s">
+        <v>1765</v>
+      </c>
+      <c r="S83" s="22">
+        <v>4.3</v>
+      </c>
     </row>
     <row r="84" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A84" s="55" t="s">
@@ -10393,7 +10547,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="88" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:19" ht="116.75" x14ac:dyDescent="0.2">
       <c r="A88" s="23" t="s">
         <v>1332</v>
       </c>
@@ -10440,7 +10594,10 @@
         <v>455</v>
       </c>
       <c r="Q88" s="22" t="s">
-        <v>1668</v>
+        <v>1766</v>
+      </c>
+      <c r="S88" s="22">
+        <v>157.7</v>
       </c>
     </row>
     <row r="89" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -10486,7 +10643,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="90" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:19" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A90" s="23" t="s">
         <v>1338</v>
       </c>
@@ -10533,7 +10690,10 @@
         <v>461</v>
       </c>
       <c r="Q90" s="22" t="s">
-        <v>1683</v>
+        <v>1767</v>
+      </c>
+      <c r="S90" s="22">
+        <v>113.2</v>
       </c>
     </row>
     <row r="91" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -10868,7 +11028,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="99" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:19" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A99" s="21" t="s">
         <v>507</v>
       </c>
@@ -10913,7 +11073,10 @@
         <v>496</v>
       </c>
       <c r="Q99" s="22" t="s">
-        <v>1685</v>
+        <v>1768</v>
+      </c>
+      <c r="S99" s="22">
+        <v>64.7</v>
       </c>
     </row>
     <row r="100" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -11050,7 +11213,7 @@
         <v>1686</v>
       </c>
     </row>
-    <row r="103" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:19" ht="53.0" x14ac:dyDescent="0.2">
       <c r="A103" s="21" t="s">
         <v>1640</v>
       </c>
@@ -11094,10 +11257,13 @@
       </c>
       <c r="P103"/>
       <c r="Q103" s="22" t="s">
-        <v>1643</v>
-      </c>
-    </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.2">
+        <v>1769</v>
+      </c>
+      <c r="S103" s="22">
+        <v>19.3</v>
+      </c>
+    </row>
+    <row r="104" spans="1:19" x14ac:dyDescent="0.2" ht="53.0" customHeight="1">
       <c r="A104" s="21" t="s">
         <v>563</v>
       </c>
@@ -11142,10 +11308,13 @@
         <v>524</v>
       </c>
       <c r="Q104" s="22" t="s">
-        <v>1687</v>
-      </c>
-    </row>
-    <row r="105" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+        <v>1770</v>
+      </c>
+      <c r="S104" s="22">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="105" spans="1:19" ht="53.0" x14ac:dyDescent="0.2">
       <c r="A105" s="23" t="s">
         <v>1381</v>
       </c>
@@ -11190,6 +11359,12 @@
       </c>
       <c r="O105" s="24" t="s">
         <v>529</v>
+      </c>
+      <c r="Q105" s="22" t="s">
+        <v>1771</v>
+      </c>
+      <c r="S105" s="22">
+        <v>112847</v>
       </c>
     </row>
     <row r="106" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -11929,7 +12104,7 @@
         <v>1733</v>
       </c>
     </row>
-    <row r="124" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:19" ht="78.5" x14ac:dyDescent="0.2">
       <c r="A124" s="21" t="s">
         <v>1635</v>
       </c>
@@ -11971,7 +12146,10 @@
       </c>
       <c r="P124"/>
       <c r="Q124" s="22" t="s">
-        <v>1639</v>
+        <v>1772</v>
+      </c>
+      <c r="S124" s="22">
+        <v>11.0</v>
       </c>
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.2">
@@ -12091,7 +12269,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="128" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:19" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A128" s="23" t="s">
         <v>1443</v>
       </c>
@@ -12139,6 +12317,9 @@
       <c r="N128" s="22"/>
       <c r="O128" s="24" t="s">
         <v>625</v>
+      </c>
+      <c r="Q128" s="22" t="s">
+        <v>1773</v>
       </c>
     </row>
     <row r="129" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
@@ -13220,7 +13401,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>1750</v>
+        <v>1780</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -13231,7 +13412,7 @@
         <v>751</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>1751</v>
+        <v>1781</v>
       </c>
       <c r="C7" s="2"/>
     </row>

</xml_diff>

<commit_message>
NRM1 v5.9: Whitefields rates on the owner's quantities
The owner confirmed 17 blocks, about 3,740 m2 GIA (220 m2 each),
2,210 m2 footprint (130 m2 each) and an 8,000 m2 site, replacing the
3,000 m2 GIA assumption. Column R: 0.1 asbestos 8.1, 0.2 demolition
73.3, 0.7 service diversions 36.3 (254 m water main, from Mace's
pre-tender estimate), 8.10 soft landscaping 2.1. WF lines, the
Instructions note and the v5.9 log line updated. Evidence only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ThEE8jqhmBASGLx3pT6ipD
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4226" uniqueCount="1752">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4226" uniqueCount="1758">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5287,6 +5287,24 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WF: £8.1 on the contract (Total Reclaims, £28,050 to the asbestos BoQ) over 3,740 m² GIA (17 blocks × about 220 m², owner's figures). Five bids on the same BoQ: £8.1–£42.5, median £12.7. Mace's pre-tender allowance was £85,000 (£24.5). The R&amp;D survey (£9,400) was a fee.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WF: £73 per m² demolished on the contract, 3,740 m² GIA (17 blocks × about 220 m², owner's figures): soft strip, demolish, slabs and foundations £34; disconnecting and cutting back drainage, water, gas, electrical and telecoms, plus Trinity / Honeywell fire alarm, security and metering removal, £39. Core demolition across five bids £34–£70 (median £46). About £15k per block. Excludes the water-main replacement (0.7) and the contractor's own £15k provisional sums for the Trinity / Honeywell work, which those quotes replace.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WF: £36 per m² footprint on the contract (17 × about 130 m² = 2,210 m² footprint): replacing 254 m of ductile iron water main across the site in MDPE, with temporary water, trenching, stone surround and tarmac reinstatement (£74k; about £315/m of main). £44 with the changes pending at FS 16, Jul 2026 (trial pits on the district heating and water mains, out-of-hours water works: £16.7k).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WF: £2.1 per m² over the 8,000 m² site (contract £15.4k): topsoil and grass seed to the UoW Grounds specification only — no planting or maintenance. Five bids £2.1–£11.2, median £3.2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column R on '2. Rates': the Whitefields demolition contract figure for that row (Total Reclaims, £525,676; AFC £532,445 at FS 16, Jul 2026), in the row's unit and on this workbook's basis — line items without the contractor's prelims and OH&amp;P, ÷ 0.94 West Midlands factor, × 1.014 to Q3 2026. Quantities from the owner: 17 blocks, 3,740 m² GIA (about 220 m² each over ground and first floors), 2,210 m² footprint (about 130 m² each), 8,000 m² site. Evidence only: the app does not read this column and no rate changed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence only, no rates changed. New column R 'Whitefields rate' on '2. Rates' and WF lines in Tender check, from the Whitefields demolition contract (Total Reclaims £525,676; AFC £532,445 at FS 16, Jul 2026; 3,740 m² GIA, 2,210 m² footprint, 8,000 m² site): 0.1 asbestos £8.1/m² GIFA; 0.2 demolition incl. disconnections £73/m² demolished; 0.7 service diversions £36/m² footprint (254 m water-main replacement); 8.10 topsoil and seed £2.1/m². Not on '2. Rates': the contractor's prelims incl. hoarding were 16.8% of works and OH&amp;P 15%; professional fees 28% of construction (asbestos surveys £43k, ecology £33k), UoW Estates fees 4%, contingency 7%; construction 15–16 weeks on site.</t>
   </si>
 </sst>
 </file>
@@ -6094,7 +6112,7 @@
         <v>1746</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>1747</v>
+        <v>1756</v>
       </c>
       <c r="C22" s="33"/>
     </row>
@@ -6590,7 +6608,7 @@
         <v>1748</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>1749</v>
+        <v>1757</v>
       </c>
       <c r="C79" s="60"/>
     </row>
@@ -6855,10 +6873,10 @@
         <v>58</v>
       </c>
       <c r="Q7" s="22" t="s">
-        <v>1740</v>
+        <v>1752</v>
       </c>
       <c r="R7" s="22">
-        <v>10.1</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="38.25" x14ac:dyDescent="0.2">
@@ -6900,10 +6918,10 @@
         <v>73</v>
       </c>
       <c r="Q8" s="22" t="s">
-        <v>1741</v>
+        <v>1753</v>
       </c>
       <c r="R8" s="22">
-        <v>91.4</v>
+        <v>73.3</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
@@ -7100,10 +7118,10 @@
         <v>113</v>
       </c>
       <c r="Q13" s="22" t="s">
-        <v>1742</v>
+        <v>1754</v>
       </c>
       <c r="R13" s="22">
-        <v>40.2</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -12838,10 +12856,10 @@
         <v>697</v>
       </c>
       <c r="Q145" s="22" t="s">
-        <v>1743</v>
+        <v>1755</v>
       </c>
       <c r="R145" s="22">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="146" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
NRM1 v5.11: one rate column per real project, plus an average
'2. Rates' gains plain number columns beside Whitefields (R) and
Claycroft (S): T Lakeside, U Computer Science, V Scarman toilets (high
spec), W Co-op store, X IBRB cafe, Y Riley Court (signed contract CSA),
and Z = AVERAGE(R:Y) on the 47 rows with a figure. Each is in the row's
unit on the workbook basis. Instructions row 24 explains the columns
and the evidence with no row; v5.11 log line at row 81.

Evidence only: the loader reads columns by header text, so no estimate
changes. 557 tests pass; version pin moved to v5.11.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QB69m6diVrBfvTZaLwAazz
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4236" uniqueCount="1788">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4236" uniqueCount="1790">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5395,6 +5395,12 @@
   </si>
   <si>
     <t xml:space="preserve">WF: £2.1 per m² over the 8,000 m² site (contract £15.4k): topsoil and grass seed to the UoW Grounds specification only — no planting or maintenance. Five bids £2.1–£11.2, median £3.2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.11 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-04</t>
   </si>
 </sst>
 </file>
@@ -6015,7 +6021,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BBCD35-3C7D-4CAC-A46E-6C3CC3E31849}">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.7109375" style="8" customWidth="1"/>
@@ -6026,7 +6032,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1774</v>
+        <v>1788</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -6216,613 +6222,637 @@
       <c r="C23" s="33"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Project rate columns (T–Z)</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Columns T–Y on '2. Rates' hold the other real projects' figures in the row's unit and on this workbook's basis, beside Whitefields (R) and Claycroft (S): T Lakeside S&amp;F (tender Sep 2026, median of 4 bids); U Computer Science decarbonisation (tender Mar 2024, mean of 2 bids); V Scarman Public Toilets Phase 2 (HIGH spec, tender Apr 2026, median of 6 bids; per m² over the 71 m² toilet area); W Co-op grocery store fit-out (Kingfisher contract Aug 2025, 885 m²); X IBRB café servery (Senevo winning bid 2025, 72 m² café, 28 m² servery); Y Riley Court Psychology full refurbishment (Maris signed contract £9.15m, GMP Nov 2024, GIFA 3,850 m²). Each excludes the contractor's prelims, OH&amp;P and design, rebased to Q3 2026 and ÷ 0.94 West Midlands. Column Z is the average of R–Y for the row. Projects differ in scope and specification, so expect spread. Not on '2. Rates': scaffold for envelope works £42 (CS) and £33 (Claycroft) per m² GIFA; retail refrigeration £379 and retailer equipment £373 per m² (Co-op); preliminaries Lakeside ~9%, Whitefields 16.8%, Claycroft 11.3%, Scarman 14%, Co-op 7.2%, IBRB 17.7%, Riley Court 5.5% (+4% contractor PM and design). Evidence only: the app does not read these columns and no rate changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="13" t="s">
         <v>1568</v>
       </c>
-      <c r="B24" s="16"/>
-      <c r="C24" s="34"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="15" t="s">
-        <v>1076</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>1569</v>
-      </c>
-      <c r="C25" s="33"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="34"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="15" t="s">
-        <v>1098</v>
+        <v>1076</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>1570</v>
+        <v>1569</v>
       </c>
       <c r="C26" s="33"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="15" t="s">
-        <v>1118</v>
+        <v>1098</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>1571</v>
+        <v>1570</v>
       </c>
       <c r="C27" s="33"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="15" t="s">
-        <v>1179</v>
+        <v>1118</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>1572</v>
+        <v>1571</v>
       </c>
       <c r="C28" s="33"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="15" t="s">
-        <v>1174</v>
+        <v>1179</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>1573</v>
+        <v>1572</v>
       </c>
       <c r="C29" s="33"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="15" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>1573</v>
+      </c>
+      <c r="C30" s="33"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="15" t="s">
         <v>1637</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B31" s="17" t="s">
         <v>1710</v>
       </c>
-      <c r="C30" s="33"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="15"/>
-      <c r="B31" s="17"/>
       <c r="C31" s="33"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="15"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="33"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B32" s="16"/>
-      <c r="C32" s="34"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="15" t="s">
-        <v>1574</v>
-      </c>
-      <c r="B33" s="17" t="s">
-        <v>1575</v>
-      </c>
-      <c r="C33" s="33"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="34"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="15" t="s">
-        <v>8</v>
+        <v>1574</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>1576</v>
+        <v>1575</v>
       </c>
       <c r="C34" s="33"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="15" t="s">
-        <v>1577</v>
+        <v>8</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>1578</v>
+        <v>1576</v>
       </c>
       <c r="C35" s="33"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="15" t="s">
-        <v>1579</v>
-      </c>
-      <c r="B36" s="32" t="s">
-        <v>1580</v>
+        <v>1577</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>1578</v>
       </c>
       <c r="C36" s="33"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="15" t="s">
-        <v>1581</v>
+        <v>1579</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>1582</v>
+        <v>1580</v>
       </c>
       <c r="C37" s="33"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>1583</v>
+        <v>1581</v>
+      </c>
+      <c r="B38" s="32" t="s">
+        <v>1582</v>
       </c>
       <c r="C38" s="33"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>1583</v>
+      </c>
+      <c r="C39" s="33"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B39" s="17" t="s">
+      <c r="B40" s="17" t="s">
         <v>1584</v>
       </c>
-      <c r="C39" s="33"/>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="15"/>
-      <c r="B40" s="17"/>
       <c r="C40" s="33"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="13" t="s">
+      <c r="A41" s="15"/>
+      <c r="B41" s="17"/>
+      <c r="C41" s="33"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="13" t="s">
         <v>1585</v>
       </c>
-      <c r="B41" s="16"/>
-      <c r="C41" s="34"/>
-    </row>
-    <row r="42" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A42" s="15" t="s">
-        <v>1586</v>
-      </c>
-      <c r="B42" s="17" t="s">
-        <v>1587</v>
-      </c>
-      <c r="C42" s="33"/>
+      <c r="B42" s="16"/>
+      <c r="C42" s="34"/>
     </row>
     <row r="43" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A43" s="15" t="s">
+        <v>1586</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>1587</v>
+      </c>
+      <c r="C43" s="33"/>
+    </row>
+    <row r="44" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A44" s="15" t="s">
         <v>1588</v>
       </c>
-      <c r="B43" s="17" t="s">
+      <c r="B44" s="17" t="s">
         <v>3</v>
-      </c>
-      <c r="C43" s="33"/>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="15" t="s">
-        <v>1589</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>1590</v>
       </c>
       <c r="C44" s="33"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="15" t="s">
-        <v>1591</v>
+        <v>1589</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>1592</v>
+        <v>1590</v>
       </c>
       <c r="C45" s="33"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="15" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B46" s="17" t="s">
+        <v>1592</v>
+      </c>
+      <c r="C46" s="33"/>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="B46" s="17" t="s">
+      <c r="B47" s="17" t="s">
         <v>1593</v>
       </c>
-      <c r="C46" s="33"/>
-    </row>
-    <row r="47" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A47" s="15" t="s">
+      <c r="C47" s="33"/>
+    </row>
+    <row r="48" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A48" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B48" s="17" t="s">
         <v>1633</v>
       </c>
-      <c r="C47" s="33"/>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="15" t="s">
+      <c r="C48" s="33"/>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="B49" s="17" t="s">
         <v>1594</v>
-      </c>
-      <c r="C48" s="33"/>
-    </row>
-    <row r="49" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A49" s="15" t="s">
-        <v>1595</v>
-      </c>
-      <c r="B49" s="17" t="s">
-        <v>1596</v>
       </c>
       <c r="C49" s="33"/>
     </row>
     <row r="50" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A50" s="15" t="s">
+        <v>1595</v>
+      </c>
+      <c r="B50" s="17" t="s">
+        <v>1596</v>
+      </c>
+      <c r="C50" s="33"/>
+    </row>
+    <row r="51" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A51" s="15" t="s">
         <v>1597</v>
       </c>
-      <c r="B50" s="17" t="s">
+      <c r="B51" s="17" t="s">
         <v>1598</v>
-      </c>
-      <c r="C50" s="33"/>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="15" t="s">
-        <v>1599</v>
-      </c>
-      <c r="B51" s="17" t="s">
-        <v>1600</v>
       </c>
       <c r="C51" s="33"/>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="15" t="s">
-        <v>1601</v>
+        <v>1599</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>1602</v>
+        <v>1600</v>
       </c>
       <c r="C52" s="33"/>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="15" t="s">
+        <v>1601</v>
+      </c>
+      <c r="B53" s="17" t="s">
+        <v>1602</v>
+      </c>
+      <c r="C53" s="33"/>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B53" s="17" t="s">
+      <c r="B54" s="17" t="s">
         <v>1603</v>
       </c>
-      <c r="C53" s="33"/>
-    </row>
-    <row r="54" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A54" s="15" t="s">
+      <c r="C54" s="33"/>
+    </row>
+    <row r="55" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A55" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B54" s="17" t="s">
+      <c r="B55" s="17" t="s">
         <v>1604</v>
-      </c>
-      <c r="C54" s="33"/>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="15" t="s">
-        <v>1605</v>
-      </c>
-      <c r="B55" s="17" t="s">
-        <v>1606</v>
       </c>
       <c r="C55" s="33"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="15" t="s">
-        <v>46</v>
+        <v>1605</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="C56" s="33"/>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="15" t="s">
-        <v>1608</v>
+        <v>46</v>
       </c>
       <c r="B57" s="17" t="s">
-        <v>1609</v>
+        <v>1607</v>
       </c>
       <c r="C57" s="33"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="15" t="s">
+        <v>1608</v>
+      </c>
+      <c r="B58" s="17" t="s">
+        <v>1609</v>
+      </c>
+      <c r="C58" s="33"/>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="17" t="s">
+      <c r="B59" s="17" t="s">
         <v>1610</v>
       </c>
-      <c r="C58" s="33"/>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="15"/>
-      <c r="B59" s="17"/>
       <c r="C59" s="33"/>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="13" t="s">
+      <c r="A60" s="15"/>
+      <c r="B60" s="17"/>
+      <c r="C60" s="33"/>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B60" s="16"/>
-      <c r="C60" s="34"/>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="15" t="s">
+      <c r="B61" s="16"/>
+      <c r="C61" s="34"/>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="15" t="s">
         <v>1611</v>
       </c>
-      <c r="B61" s="17"/>
-      <c r="C61" s="33">
+      <c r="B62" s="17"/>
+      <c r="C62" s="33">
         <f>SUMPRODUCT(('2. Rates'!O6:O152&lt;&gt;"")*(COUNTIF('2. Rates'!O6:O152,'2. Rates'!O6:O152)&gt;1))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="15" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="15" t="s">
         <v>1612</v>
       </c>
-      <c r="B62" s="17"/>
-      <c r="C62" s="33">
+      <c r="B63" s="17"/>
+      <c r="C63" s="33">
         <f>SUMPRODUCT(('2. Rates'!O6:O152&lt;&gt;"")*(COUNTIF('4. Scope rules'!A91:A229,'2. Rates'!O6:O152)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="15" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="15" t="s">
         <v>1613</v>
       </c>
-      <c r="B63" s="17"/>
-      <c r="C63" s="33">
+      <c r="B64" s="17"/>
+      <c r="C64" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A91:A229&lt;&gt;"")*(COUNTIF('2. Rates'!O6:O152,'4. Scope rules'!A91:A229)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="15" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="15" t="s">
         <v>1614</v>
       </c>
-      <c r="B64" s="17"/>
-      <c r="C64" s="33">
+      <c r="B65" s="17"/>
+      <c r="C65" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A91:A229&lt;&gt;"")*(COUNTIF('4. Scope rules'!A6:A87,'4. Scope rules'!B91:B229)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="15" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="15" t="s">
         <v>1615</v>
       </c>
-      <c r="B65" s="17"/>
-      <c r="C65" s="33">
+      <c r="B66" s="17"/>
+      <c r="C66" s="33">
         <f>SUMPRODUCT(('2. Rates'!O6:O152&lt;&gt;"")*('2. Rates'!M6:M152=""))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="15" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="15" t="s">
         <v>1616</v>
       </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="33">
+      <c r="B67" s="17"/>
+      <c r="C67" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*(ROUND('4. Scope rules'!M6:M87+'4. Scope rules'!O6:O87,4)&lt;&gt;1))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" s="15" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B67" s="17"/>
-      <c r="C67" s="33">
+      <c r="B68" s="17"/>
+      <c r="C68" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*(COUNTIFS('4. Scope rules'!B91:B229,'4. Scope rules'!A6:A87,'4. Scope rules'!E91:E229,"Yes")=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="15" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="15" t="s">
         <v>1617</v>
       </c>
-      <c r="B68" s="17"/>
-      <c r="C68" s="33">
+      <c r="B69" s="17"/>
+      <c r="C69" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*('4. Scope rules'!F6:F87="One")*(COUNTIFS('4. Scope rules'!B91:B229,'4. Scope rules'!A6:A87,'4. Scope rules'!E91:E229,"Yes")&gt;1))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="15" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="15" t="s">
         <v>1618</v>
       </c>
-      <c r="B69" s="17"/>
-      <c r="C69" s="33">
+      <c r="B70" s="17"/>
+      <c r="C70" s="33">
         <f>SUMPRODUCT(('4. Scope rules'!A6:A87&lt;&gt;"")*('4. Scope rules'!G6:G87=""))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="15" t="s">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B70" s="17"/>
-      <c r="C70" s="33">
+      <c r="B71" s="17"/>
+      <c r="C71" s="33">
         <f>SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('4. Scope rules'!H6:H87,"NB",""),"EX",""),"RF",""),"FO",""),"EW",""),"DM",""),"OM",""),"—","")))&gt;0))+SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('4. Scope rules'!I6:I87,"NB",""),"EX",""),"RF",""),"FO",""),"EW",""),"DM",""),"OM",""),"—","")))&gt;0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="15" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B71" s="17"/>
-      <c r="C71" s="33">
+      <c r="B72" s="17"/>
+      <c r="C72" s="33">
         <f>SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('4. Scope rules'!J6:J87,"RES",""),"STU",""),"OFF",""),"EDU",""),"HEA",""),"RET",""),"IND",""),"HOS",""),"MIX",""),"OTH",""),"ALL","")))&gt;0))+SUMPRODUCT(--(LEN(TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE('2. Rates'!D6:D152,"RES",""),"STU",""),"OFF",""),"EDU",""),"HEA",""),"RET",""),"IND",""),"HOS",""),"MIX",""),"OTH",""),"ALL","")))&gt;0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="15" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B72" s="17"/>
-      <c r="C72" s="33">
+      <c r="B73" s="17"/>
+      <c r="C73" s="33">
         <f>SUMPRODUCT(('3. Settings'!A96:A123&lt;&gt;"")*(COUNTIFS('3. Settings'!A96:A123,'3. Settings'!A96:A123,'3. Settings'!B96:B123,"ALL")=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A73" s="15" t="s">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B73" s="17"/>
-      <c r="C73" s="33">
+      <c r="B74" s="17"/>
+      <c r="C74" s="33">
         <f>SUMPRODUCT(('3. Settings'!A96:A123&lt;&gt;"")*('3. Settings'!C96:C123=""))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="15"/>
-      <c r="B74" s="17"/>
-      <c r="C74" s="33"/>
-    </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="13" t="s">
+      <c r="A75" s="15"/>
+      <c r="B75" s="17"/>
+      <c r="C75" s="33"/>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B75" s="16"/>
-      <c r="C75" s="34"/>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" s="15" t="s">
+      <c r="B76" s="16"/>
+      <c r="C76" s="34"/>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B76" s="17"/>
-      <c r="C76" s="33">
+      <c r="B77" s="17"/>
+      <c r="C77" s="33">
         <f>COUNTA('4. Scope rules'!A6:A87)</f>
         <v>82</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="15" t="s">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78" s="15" t="s">
         <v>1619</v>
       </c>
-      <c r="B77" s="17"/>
-      <c r="C77" s="33">
+      <c r="B78" s="17"/>
+      <c r="C78" s="33">
         <f>COUNTA('2. Rates'!O6:O152)</f>
         <v>139</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A78" s="15"/>
-      <c r="B78" s="17"/>
-      <c r="C78" s="33"/>
-    </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A79" s="13" t="s">
+      <c r="A79" s="15"/>
+      <c r="B79" s="17"/>
+      <c r="C79" s="33"/>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B79" s="16"/>
-      <c r="C79" s="34"/>
-    </row>
-    <row r="80" spans="1:3" s="54" customFormat="1" ht="104.0" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="17" t="s">
+      <c r="B80" s="16"/>
+      <c r="C80" s="34"/>
+    </row>
+    <row r="81" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="17" t="inlineStr">
+        <is>
+          <t>v5.11 — 4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B81" s="17" t="inlineStr">
+        <is>
+          <t>Evidence only, no rates changed. Six more project columns on '2. Rates' beside Whitefields (R) and Claycroft (S), each a plain figure in the row's unit on this workbook's basis: T Lakeside S&amp;F (15 rows), U Computer Science (6), V Scarman Public Toilets Phase 2, high spec (12), W Co-op store fit-out (19), X IBRB café (7), Y Riley Court Psychology refurbishment (27, from the signed contract CSA). Column Z averages R–Y on 47 rows. Row 24 explains the columns and lists the evidence that has no row (scaffold, retail refrigeration and equipment, preliminaries %).</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:3" s="54" customFormat="1" ht="104.0" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="17" t="s">
         <v>1778</v>
       </c>
-      <c r="B80" s="17" t="s">
+      <c r="B82" s="17" t="s">
         <v>1779</v>
       </c>
-      <c r="C80" s="60"/>
-    </row>
-    <row r="81" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="17" t="s">
+      <c r="C82" s="60"/>
+    </row>
+    <row r="83" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="17" t="s">
         <v>1748</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B83" s="17" t="s">
         <v>1783</v>
-      </c>
-      <c r="C81" s="60"/>
-    </row>
-    <row r="82" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A82" s="17" t="s">
-        <v>1722</v>
-      </c>
-      <c r="B82" s="17" t="s">
-        <v>1737</v>
-      </c>
-      <c r="C82" s="60"/>
-    </row>
-    <row r="83" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A83" s="17" t="s">
-        <v>1711</v>
-      </c>
-      <c r="B83" s="17" t="s">
-        <v>1712</v>
       </c>
       <c r="C83" s="60"/>
     </row>
     <row r="84" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A84" s="17" t="s">
+        <v>1722</v>
+      </c>
+      <c r="B84" s="17" t="s">
+        <v>1737</v>
+      </c>
+      <c r="C84" s="60"/>
+    </row>
+    <row r="85" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A85" s="17" t="s">
+        <v>1711</v>
+      </c>
+      <c r="B85" s="17" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C85" s="60"/>
+    </row>
+    <row r="86" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A86" s="17" t="s">
         <v>1632</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B86" s="17" t="s">
         <v>1634</v>
       </c>
-      <c r="C84" s="60"/>
-    </row>
-    <row r="85" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A85" s="15" t="s">
+      <c r="C86" s="60"/>
+    </row>
+    <row r="87" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A87" s="15" t="s">
         <v>1620</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B87" s="17" t="s">
         <v>1621</v>
       </c>
-      <c r="C85" s="33"/>
-    </row>
-    <row r="86" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A86" s="15" t="s">
+      <c r="C87" s="33"/>
+    </row>
+    <row r="88" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A88" s="15" t="s">
         <v>1060</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B88" s="17" t="s">
         <v>1061</v>
-      </c>
-      <c r="C86" s="33"/>
-    </row>
-    <row r="87" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A87" s="15" t="s">
-        <v>1051</v>
-      </c>
-      <c r="B87" s="17" t="s">
-        <v>1052</v>
-      </c>
-      <c r="C87" s="33"/>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A88" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="B88" s="17" t="s">
-        <v>24</v>
       </c>
       <c r="C88" s="33"/>
     </row>
     <row r="89" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A89" s="15" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B89" s="17" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C89" s="33"/>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B90" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C90" s="33"/>
+    </row>
+    <row r="91" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A91" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="B91" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C89" s="33"/>
-    </row>
-    <row r="90" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A90" s="15" t="s">
+      <c r="C91" s="33"/>
+    </row>
+    <row r="92" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A92" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B90" s="17" t="s">
+      <c r="B92" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C90" s="33"/>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A91" s="15" t="s">
+      <c r="C92" s="33"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B91" s="17" t="s">
+      <c r="B93" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C91" s="33"/>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A92" s="15" t="s">
+      <c r="C93" s="33"/>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B92" s="17" t="s">
+      <c r="B94" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C92" s="33"/>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A93" s="15"/>
-      <c r="B93" s="17"/>
-      <c r="C93" s="33"/>
+      <c r="C94" s="33"/>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95" s="15"/>
+      <c r="B95" s="17"/>
+      <c r="C95" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6831,7 +6861,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61613224-FE41-4C03-8B46-4109509C3076}">
-  <dimension ref="A1:S152"/>
+  <dimension ref="A1:Z152"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.7109375" style="8" customWidth="1"/>
@@ -6850,7 +6880,9 @@
     <col min="17" max="17" width="44.7109375" style="8" customWidth="1"/>
     <col min="18" max="18" width="16.7109375" style="8" customWidth="1"/>
     <col min="19" max="19" width="16.7109375" style="8" customWidth="1"/>
-    <col min="20" max="16384" width="9.140625" style="8"/>
+    <col min="20" max="25" width="16.7109375" style="8" customWidth="1"/>
+    <col min="26" max="26" width="14.7109375" style="8" customWidth="1"/>
+    <col min="27" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="18" x14ac:dyDescent="0.25">
@@ -6868,7 +6900,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>756</v>
       </c>
@@ -6925,6 +6957,41 @@
       </c>
       <c r="S5" s="12" t="s">
         <v>1753</v>
+      </c>
+      <c r="T5" s="12" t="inlineStr">
+        <is>
+          <t>Lakeside rate (£ per this row's unit, this workbook's basis: Lakeside Staff &amp; Family Flats refurbishment, tender Sep 2026, median of 4 bids ÷ 0.94. Evidence only — the app does not read it)</t>
+        </is>
+      </c>
+      <c r="U5" s="12" t="inlineStr">
+        <is>
+          <t>Computer Science rate (£ per this row's unit, this workbook's basis: CS Building decarbonisation, tender Mar 2024, mean of 2 bids × 1.07 ÷ 0.94; roof per m² footprint; 5.1b is the whole M&amp;E package. Evidence only)</t>
+        </is>
+      </c>
+      <c r="V5" s="12" t="inlineStr">
+        <is>
+          <t>Scarman rate (£ per this row's unit, this workbook's basis: Scarman Public Toilets Phase 2, HIGH specification, tender Apr 2026, median of 6 bids × 1.007 ÷ 0.94; per m² figures over the 71 m² toilet area only. Evidence only)</t>
+        </is>
+      </c>
+      <c r="W5" s="12" t="inlineStr">
+        <is>
+          <t>Co-op rate (£ per this row's unit, this workbook's basis: Co-op grocery store fit-out, Kingfisher CSA, contract Aug 2025 × 1.03 ÷ 0.94, over 885 m². Evidence only)</t>
+        </is>
+      </c>
+      <c r="X5" s="12" t="inlineStr">
+        <is>
+          <t>IBRB café rate (£ per this row's unit, this workbook's basis: IBRB café servery fit-out, Senevo winning bid 2025 × 1.035 ÷ 0.94, over 72 m² (catering kitchen per 28 m² servery). Evidence only)</t>
+        </is>
+      </c>
+      <c r="Y5" s="12" t="inlineStr">
+        <is>
+          <t>Riley Court rate (£ per this row's unit, this workbook's basis: Psychology building full refurbishment, Maris signed contract CSA £9.15m, GMP Nov 2024 × 1.05 ÷ 0.94, GIFA 3,850 m². Evidence only)</t>
+        </is>
+      </c>
+      <c r="Z5" s="12" t="inlineStr">
+        <is>
+          <t>Average of project rates (mean of columns R–Y that hold a figure for this row. Projects differ in scope and specification, so read it with the column notes. Evidence only — the app does not read it)</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -6946,7 +7013,7 @@
       <c r="N6" s="19"/>
       <c r="O6" s="20"/>
     </row>
-    <row r="7" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
         <v>72</v>
       </c>
@@ -6990,8 +7057,12 @@
       <c r="R7" s="22" t="n">
         <v>8.1</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="Z7" s="40">
+        <f>AVERAGE(R7:Y7)</f>
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
         <v>82</v>
       </c>
@@ -7035,8 +7106,12 @@
       <c r="R8" s="22" t="n">
         <v>73.3</v>
       </c>
-    </row>
-    <row r="9" spans="1:19" ht="78.5" x14ac:dyDescent="0.2">
+      <c r="Z8" s="40">
+        <f>AVERAGE(R8:Y8)</f>
+        <v>73.3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="78.5" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
         <v>96</v>
       </c>
@@ -7080,6 +7155,25 @@
       <c r="S9" s="22">
         <v>51.4</v>
       </c>
+      <c r="T9" s="22">
+        <v>54</v>
+      </c>
+      <c r="V9" s="22">
+        <v>217</v>
+      </c>
+      <c r="W9" s="22">
+        <v>48.8</v>
+      </c>
+      <c r="X9" s="22">
+        <v>11.5</v>
+      </c>
+      <c r="Y9" s="22">
+        <v>54.9</v>
+      </c>
+      <c r="Z9" s="40">
+        <f>AVERAGE(R9:Y9)</f>
+        <v>72.933333</v>
+      </c>
     </row>
     <row r="10" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
@@ -7196,7 +7290,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
         <v>119</v>
       </c>
@@ -7236,6 +7330,10 @@
         <v>1786</v>
       </c>
       <c r="R13" s="22" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="Z13" s="40">
+        <f>AVERAGE(R13:Y13)</f>
         <v>36.3</v>
       </c>
     </row>
@@ -7669,7 +7767,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="218.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:26" ht="218.75" x14ac:dyDescent="0.2">
       <c r="A25" s="21" t="s">
         <v>1669</v>
       </c>
@@ -7721,8 +7819,15 @@
       <c r="S25" s="22">
         <v>516.9</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="U25" s="22">
+        <v>182</v>
+      </c>
+      <c r="Z25" s="40">
+        <f>AVERAGE(R25:Y25)</f>
+        <v>349.45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A26" s="21" t="s">
         <v>1659</v>
       </c>
@@ -7764,8 +7869,15 @@
       <c r="Q26" s="22" t="s">
         <v>1664</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="T26" s="22">
+        <v>32</v>
+      </c>
+      <c r="Z26" s="40">
+        <f>AVERAGE(R26:Y26)</f>
+        <v>32.0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:26" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A27" s="21" t="s">
         <v>197</v>
       </c>
@@ -7812,8 +7924,18 @@
       <c r="Q27" s="22" t="s">
         <v>1730</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" ht="165.75" x14ac:dyDescent="0.2">
+      <c r="U27" s="22">
+        <v>48</v>
+      </c>
+      <c r="Y27" s="22">
+        <v>170.5</v>
+      </c>
+      <c r="Z27" s="40">
+        <f>AVERAGE(R27:Y27)</f>
+        <v>109.25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:26" ht="165.75" x14ac:dyDescent="0.2">
       <c r="A28" s="21" t="s">
         <v>203</v>
       </c>
@@ -7860,8 +7982,21 @@
       <c r="Q28" s="22" t="s">
         <v>1731</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="U28" s="22">
+        <v>210</v>
+      </c>
+      <c r="W28" s="22">
+        <v>24.4</v>
+      </c>
+      <c r="Y28" s="22">
+        <v>146.7</v>
+      </c>
+      <c r="Z28" s="40">
+        <f>AVERAGE(R28:Y28)</f>
+        <v>127.033333</v>
+      </c>
+    </row>
+    <row r="29" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A29" s="21" t="s">
         <v>208</v>
       </c>
@@ -7905,8 +8040,18 @@
       <c r="O29" s="24" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="W29" s="22">
+        <v>26.4</v>
+      </c>
+      <c r="Y29" s="22">
+        <v>246.9</v>
+      </c>
+      <c r="Z29" s="40">
+        <f>AVERAGE(R29:Y29)</f>
+        <v>136.65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A30" s="21" t="s">
         <v>1142</v>
       </c>
@@ -7950,8 +8095,21 @@
       <c r="O30" s="24" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="31" spans="1:19" ht="155.0" x14ac:dyDescent="0.2">
+      <c r="V30" s="22">
+        <v>99</v>
+      </c>
+      <c r="W30" s="22">
+        <v>9.1</v>
+      </c>
+      <c r="Y30" s="22">
+        <v>163.7</v>
+      </c>
+      <c r="Z30" s="40">
+        <f>AVERAGE(R30:Y30)</f>
+        <v>90.6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:26" ht="155.0" x14ac:dyDescent="0.2">
       <c r="A31" s="21" t="s">
         <v>1146</v>
       </c>
@@ -7998,6 +8156,22 @@
       </c>
       <c r="S31" s="22">
         <v>95.8</v>
+      </c>
+      <c r="T31" s="22">
+        <v>13.5</v>
+      </c>
+      <c r="V31" s="22">
+        <v>24</v>
+      </c>
+      <c r="W31" s="22">
+        <v>3.4</v>
+      </c>
+      <c r="Y31" s="22">
+        <v>15.6</v>
+      </c>
+      <c r="Z31" s="40">
+        <f>AVERAGE(R31:Y31)</f>
+        <v>30.46</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
@@ -8019,7 +8193,7 @@
       <c r="N32" s="26"/>
       <c r="O32" s="27"/>
     </row>
-    <row r="33" spans="1:19" ht="91.25" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:26" ht="91.25" x14ac:dyDescent="0.2">
       <c r="A33" s="21" t="s">
         <v>221</v>
       </c>
@@ -8069,8 +8243,27 @@
       <c r="S33" s="22">
         <v>99.3</v>
       </c>
-    </row>
-    <row r="34" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="T33" s="22">
+        <v>72</v>
+      </c>
+      <c r="V33" s="22">
+        <v>304</v>
+      </c>
+      <c r="W33" s="22">
+        <v>26.6</v>
+      </c>
+      <c r="X33" s="22">
+        <v>49</v>
+      </c>
+      <c r="Y33" s="22">
+        <v>39.4</v>
+      </c>
+      <c r="Z33" s="40">
+        <f>AVERAGE(R33:Y33)</f>
+        <v>98.383333</v>
+      </c>
+    </row>
+    <row r="34" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A34" s="23" t="s">
         <v>1153</v>
       </c>
@@ -8118,6 +8311,19 @@
       </c>
       <c r="Q34" s="22" t="s">
         <v>1679</v>
+      </c>
+      <c r="V34" s="22">
+        <v>177</v>
+      </c>
+      <c r="W34" s="22">
+        <v>21.5</v>
+      </c>
+      <c r="Y34" s="22">
+        <v>95.3</v>
+      </c>
+      <c r="Z34" s="40">
+        <f>AVERAGE(R34:Y34)</f>
+        <v>97.933333</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
@@ -8167,7 +8373,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="65.75" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:26" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A36" s="23" t="s">
         <v>1655</v>
       </c>
@@ -8218,8 +8424,15 @@
       <c r="S36" s="22">
         <v>38.4</v>
       </c>
-    </row>
-    <row r="37" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="T36" s="22">
+        <v>51</v>
+      </c>
+      <c r="Z36" s="40">
+        <f>AVERAGE(R36:Y36)</f>
+        <v>44.7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A37" s="21" t="s">
         <v>1671</v>
       </c>
@@ -8266,8 +8479,21 @@
       <c r="Q37" s="22" t="s">
         <v>1680</v>
       </c>
-    </row>
-    <row r="38" spans="1:19" ht="104.0" x14ac:dyDescent="0.2">
+      <c r="V37" s="22">
+        <v>129</v>
+      </c>
+      <c r="W37" s="22">
+        <v>21.0</v>
+      </c>
+      <c r="Y37" s="22">
+        <v>109.6</v>
+      </c>
+      <c r="Z37" s="40">
+        <f>AVERAGE(R37:Y37)</f>
+        <v>86.533333</v>
+      </c>
+    </row>
+    <row r="38" spans="1:26" ht="104.0" x14ac:dyDescent="0.2">
       <c r="A38" s="21" t="s">
         <v>1650</v>
       </c>
@@ -8315,6 +8541,13 @@
       </c>
       <c r="S38" s="22">
         <v>70.4</v>
+      </c>
+      <c r="T38" s="22">
+        <v>30</v>
+      </c>
+      <c r="Z38" s="40">
+        <f>AVERAGE(R38:Y38)</f>
+        <v>50.2</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.2">
@@ -8336,7 +8569,7 @@
       <c r="N39" s="26"/>
       <c r="O39" s="27"/>
     </row>
-    <row r="40" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A40" s="48" t="s">
         <v>1164</v>
       </c>
@@ -8383,8 +8616,18 @@
         <v>238</v>
       </c>
       <c r="P40" s="54"/>
-    </row>
-    <row r="41" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="V40" s="22">
+        <v>7653</v>
+      </c>
+      <c r="Y40" s="22">
+        <v>14573</v>
+      </c>
+      <c r="Z40" s="40">
+        <f>AVERAGE(R40:Y40)</f>
+        <v>11113.0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A41" s="48" t="s">
         <v>1169</v>
       </c>
@@ -8428,6 +8671,13 @@
       <c r="O41" s="52" t="s">
         <v>251</v>
       </c>
+      <c r="Y41" s="22">
+        <v>16025</v>
+      </c>
+      <c r="Z41" s="40">
+        <f>AVERAGE(R41:Y41)</f>
+        <v>16025.0</v>
+      </c>
     </row>
     <row r="42" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A42" s="43" t="s">
@@ -8472,7 +8722,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="104.0" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:26" ht="104.0" x14ac:dyDescent="0.2">
       <c r="A43" s="48" t="s">
         <v>1175</v>
       </c>
@@ -8523,6 +8773,13 @@
       </c>
       <c r="S43" s="22">
         <v>3869</v>
+      </c>
+      <c r="T43" s="22">
+        <v>2563</v>
+      </c>
+      <c r="Z43" s="40">
+        <f>AVERAGE(R43:Y43)</f>
+        <v>3216.0</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
@@ -8617,7 +8874,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="46" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A46" s="48" t="s">
         <v>1188</v>
       </c>
@@ -8666,8 +8923,15 @@
       <c r="Q46" s="49" t="s">
         <v>1667</v>
       </c>
-    </row>
-    <row r="47" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="T46" s="22">
+        <v>5296</v>
+      </c>
+      <c r="Z46" s="40">
+        <f>AVERAGE(R46:Y46)</f>
+        <v>5296.0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A47" s="48" t="s">
         <v>1194</v>
       </c>
@@ -8713,8 +8977,15 @@
       <c r="O47" s="52" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="48" spans="1:19" ht="65.75" x14ac:dyDescent="0.2">
+      <c r="Y47" s="22">
+        <v>10276</v>
+      </c>
+      <c r="Z47" s="40">
+        <f>AVERAGE(R47:Y47)</f>
+        <v>10276.0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:26" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A48" s="21" t="s">
         <v>292</v>
       </c>
@@ -8764,8 +9035,18 @@
       <c r="S48" s="22">
         <v>63.7</v>
       </c>
-    </row>
-    <row r="49" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="W48" s="22">
+        <v>7.0</v>
+      </c>
+      <c r="Y48" s="22">
+        <v>41.8</v>
+      </c>
+      <c r="Z48" s="40">
+        <f>AVERAGE(R48:Y48)</f>
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A49" s="21" t="s">
         <v>1199</v>
       </c>
@@ -8809,6 +9090,16 @@
       <c r="O49" s="24" t="s">
         <v>287</v>
       </c>
+      <c r="W49" s="22">
+        <v>16.4</v>
+      </c>
+      <c r="Y49" s="22">
+        <v>12.2</v>
+      </c>
+      <c r="Z49" s="40">
+        <f>AVERAGE(R49:Y49)</f>
+        <v>14.3</v>
+      </c>
     </row>
     <row r="50" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A50" s="21" t="s">
@@ -9035,7 +9326,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="55" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A55" s="21" t="s">
         <v>1216</v>
       </c>
@@ -9076,6 +9367,13 @@
       <c r="N55" s="22"/>
       <c r="O55" s="24" t="s">
         <v>312</v>
+      </c>
+      <c r="X55" s="22">
+        <v>1438</v>
+      </c>
+      <c r="Z55" s="40">
+        <f>AVERAGE(R55:Y55)</f>
+        <v>1438.0</v>
       </c>
     </row>
     <row r="56" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -9392,7 +9690,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="64" spans="1:17" ht="140.25" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:26" ht="140.25" x14ac:dyDescent="0.2">
       <c r="A64" s="55" t="s">
         <v>1027</v>
       </c>
@@ -9444,6 +9742,13 @@
       <c r="Q64" s="22" t="s">
         <v>1732</v>
       </c>
+      <c r="U64" s="22">
+        <v>224</v>
+      </c>
+      <c r="Z64" s="40">
+        <f>AVERAGE(R64:Y64)</f>
+        <v>224.0</v>
+      </c>
     </row>
     <row r="65" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A65" s="55" t="s">
@@ -9495,7 +9800,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="66" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A66" s="55" t="s">
         <v>1252</v>
       </c>
@@ -9544,6 +9849,13 @@
       <c r="O66" s="59" t="s">
         <v>383</v>
       </c>
+      <c r="Y66" s="22">
+        <v>134.7</v>
+      </c>
+      <c r="Z66" s="40">
+        <f>AVERAGE(R66:Y66)</f>
+        <v>134.7</v>
+      </c>
     </row>
     <row r="67" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A67" s="55" t="s">
@@ -10095,7 +10407,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="78" spans="1:19" ht="91.25" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:26" ht="91.25" x14ac:dyDescent="0.2">
       <c r="A78" s="23" t="s">
         <v>1299</v>
       </c>
@@ -10147,8 +10459,24 @@
       <c r="S78" s="22">
         <v>38.9</v>
       </c>
-    </row>
-    <row r="79" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="V78" s="22">
+        <v>209</v>
+      </c>
+      <c r="W78" s="22">
+        <v>18.2</v>
+      </c>
+      <c r="X78" s="22">
+        <v>124</v>
+      </c>
+      <c r="Y78" s="22">
+        <v>104.5</v>
+      </c>
+      <c r="Z78" s="40">
+        <f>AVERAGE(R78:Y78)</f>
+        <v>98.92</v>
+      </c>
+    </row>
+    <row r="79" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A79" s="23" t="s">
         <v>1304</v>
       </c>
@@ -10200,8 +10528,15 @@
       <c r="Q79" s="22" t="s">
         <v>1681</v>
       </c>
-    </row>
-    <row r="80" spans="1:19" ht="78.5" x14ac:dyDescent="0.2">
+      <c r="T79" s="22">
+        <v>20</v>
+      </c>
+      <c r="Z79" s="40">
+        <f>AVERAGE(R79:Y79)</f>
+        <v>20.0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:26" ht="78.5" x14ac:dyDescent="0.2">
       <c r="A80" s="21" t="s">
         <v>1672</v>
       </c>
@@ -10250,8 +10585,18 @@
       <c r="Q80" s="22" t="s">
         <v>1763</v>
       </c>
-    </row>
-    <row r="81" spans="1:19" ht="91.25" x14ac:dyDescent="0.2">
+      <c r="W80" s="22">
+        <v>73.1</v>
+      </c>
+      <c r="Y80" s="22">
+        <v>172.4</v>
+      </c>
+      <c r="Z80" s="40">
+        <f>AVERAGE(R80:Y80)</f>
+        <v>122.75</v>
+      </c>
+    </row>
+    <row r="81" spans="1:26" ht="91.25" x14ac:dyDescent="0.2">
       <c r="A81" s="21" t="s">
         <v>1644</v>
       </c>
@@ -10300,8 +10645,18 @@
       <c r="S81" s="22">
         <v>28.2</v>
       </c>
-    </row>
-    <row r="82" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="T81" s="22">
+        <v>18.5</v>
+      </c>
+      <c r="V81" s="22">
+        <v>62</v>
+      </c>
+      <c r="Z81" s="40">
+        <f>AVERAGE(R81:Y81)</f>
+        <v>36.233333</v>
+      </c>
+    </row>
+    <row r="82" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A82" s="21" t="s">
         <v>420</v>
       </c>
@@ -10345,8 +10700,18 @@
       <c r="O82" s="24" t="s">
         <v>429</v>
       </c>
-    </row>
-    <row r="83" spans="1:19" ht="40.25" x14ac:dyDescent="0.2">
+      <c r="W82" s="22">
+        <v>39.5</v>
+      </c>
+      <c r="Y82" s="22">
+        <v>34.1</v>
+      </c>
+      <c r="Z82" s="40">
+        <f>AVERAGE(R82:Y82)</f>
+        <v>36.8</v>
+      </c>
+    </row>
+    <row r="83" spans="1:26" ht="40.25" x14ac:dyDescent="0.2">
       <c r="A83" s="21" t="s">
         <v>373</v>
       </c>
@@ -10396,6 +10761,16 @@
       <c r="S83" s="22">
         <v>4.3</v>
       </c>
+      <c r="W83" s="22">
+        <v>11.5</v>
+      </c>
+      <c r="Y83" s="22">
+        <v>59.1</v>
+      </c>
+      <c r="Z83" s="40">
+        <f>AVERAGE(R83:Y83)</f>
+        <v>24.966667</v>
+      </c>
     </row>
     <row r="84" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A84" s="55" t="s">
@@ -10518,7 +10893,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="87" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A87" s="23" t="s">
         <v>1328</v>
       </c>
@@ -10564,8 +10939,24 @@
       <c r="O87" s="24" t="s">
         <v>449</v>
       </c>
-    </row>
-    <row r="88" spans="1:19" ht="116.75" x14ac:dyDescent="0.2">
+      <c r="V87" s="22">
+        <v>97</v>
+      </c>
+      <c r="W87" s="22">
+        <v>88.5</v>
+      </c>
+      <c r="X87" s="22">
+        <v>218</v>
+      </c>
+      <c r="Y87" s="22">
+        <v>130.6</v>
+      </c>
+      <c r="Z87" s="40">
+        <f>AVERAGE(R87:Y87)</f>
+        <v>133.525</v>
+      </c>
+    </row>
+    <row r="88" spans="1:26" ht="116.75" x14ac:dyDescent="0.2">
       <c r="A88" s="23" t="s">
         <v>1332</v>
       </c>
@@ -10616,6 +11007,13 @@
       </c>
       <c r="S88" s="22">
         <v>157.7</v>
+      </c>
+      <c r="T88" s="22">
+        <v>153</v>
+      </c>
+      <c r="Z88" s="40">
+        <f>AVERAGE(R88:Y88)</f>
+        <v>155.35</v>
       </c>
     </row>
     <row r="89" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -10661,7 +11059,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="90" spans="1:19" ht="65.75" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:26" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A90" s="23" t="s">
         <v>1338</v>
       </c>
@@ -10712,6 +11110,22 @@
       </c>
       <c r="S90" s="22">
         <v>113.2</v>
+      </c>
+      <c r="V90" s="22">
+        <v>84</v>
+      </c>
+      <c r="W90" s="22">
+        <v>80.6</v>
+      </c>
+      <c r="X90" s="22">
+        <v>51</v>
+      </c>
+      <c r="Y90" s="22">
+        <v>198.0</v>
+      </c>
+      <c r="Z90" s="40">
+        <f>AVERAGE(R90:Y90)</f>
+        <v>105.36</v>
       </c>
     </row>
     <row r="91" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -11046,7 +11460,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="99" spans="1:19" ht="65.75" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:26" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A99" s="21" t="s">
         <v>507</v>
       </c>
@@ -11096,6 +11510,22 @@
       <c r="S99" s="22">
         <v>64.7</v>
       </c>
+      <c r="T99" s="22">
+        <v>18.6</v>
+      </c>
+      <c r="V99" s="22">
+        <v>77</v>
+      </c>
+      <c r="W99" s="22">
+        <v>28.4</v>
+      </c>
+      <c r="Y99" s="22">
+        <v>43.5</v>
+      </c>
+      <c r="Z99" s="40">
+        <f>AVERAGE(R99:Y99)</f>
+        <v>46.44</v>
+      </c>
     </row>
     <row r="100" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A100" s="21" t="s">
@@ -11183,7 +11613,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="102" spans="1:17" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A102" s="21" t="s">
         <v>1674</v>
       </c>
@@ -11230,8 +11660,21 @@
       <c r="Q102" s="22" t="s">
         <v>1686</v>
       </c>
-    </row>
-    <row r="103" spans="1:19" ht="53.0" x14ac:dyDescent="0.2">
+      <c r="T102" s="22">
+        <v>19.4</v>
+      </c>
+      <c r="X102" s="22">
+        <v>5.3</v>
+      </c>
+      <c r="Y102" s="22">
+        <v>33.6</v>
+      </c>
+      <c r="Z102" s="40">
+        <f>AVERAGE(R102:Y102)</f>
+        <v>19.433333</v>
+      </c>
+    </row>
+    <row r="103" spans="1:26" ht="53.0" x14ac:dyDescent="0.2">
       <c r="A103" s="21" t="s">
         <v>1640</v>
       </c>
@@ -11280,8 +11723,15 @@
       <c r="S103" s="22">
         <v>19.3</v>
       </c>
-    </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.2" ht="53.0" customHeight="1">
+      <c r="T103" s="22">
+        <v>24.5</v>
+      </c>
+      <c r="Z103" s="40">
+        <f>AVERAGE(R103:Y103)</f>
+        <v>21.9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:26" x14ac:dyDescent="0.2" ht="53.0" customHeight="1">
       <c r="A104" s="21" t="s">
         <v>563</v>
       </c>
@@ -11331,8 +11781,18 @@
       <c r="S104" s="22">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="105" spans="1:19" ht="53.0" x14ac:dyDescent="0.2">
+      <c r="W104" s="22">
+        <v>57.8</v>
+      </c>
+      <c r="Y104" s="22">
+        <v>22.0</v>
+      </c>
+      <c r="Z104" s="40">
+        <f>AVERAGE(R104:Y104)</f>
+        <v>28.1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:26" ht="53.0" x14ac:dyDescent="0.2">
       <c r="A105" s="23" t="s">
         <v>1381</v>
       </c>
@@ -11383,6 +11843,10 @@
       </c>
       <c r="S105" s="22">
         <v>112847</v>
+      </c>
+      <c r="Z105" s="40">
+        <f>AVERAGE(R105:Y105)</f>
+        <v>112847.0</v>
       </c>
     </row>
     <row r="106" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -12076,7 +12540,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="123" spans="1:17" ht="51" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:26" ht="51" x14ac:dyDescent="0.2">
       <c r="A123" s="21" t="s">
         <v>1675</v>
       </c>
@@ -12121,8 +12585,18 @@
       <c r="Q123" s="22" t="s">
         <v>1733</v>
       </c>
-    </row>
-    <row r="124" spans="1:19" ht="78.5" x14ac:dyDescent="0.2">
+      <c r="U123" s="22">
+        <v>8</v>
+      </c>
+      <c r="W123" s="22">
+        <v>3.1</v>
+      </c>
+      <c r="Z123" s="40">
+        <f>AVERAGE(R123:Y123)</f>
+        <v>5.55</v>
+      </c>
+    </row>
+    <row r="124" spans="1:26" ht="78.5" x14ac:dyDescent="0.2">
       <c r="A124" s="21" t="s">
         <v>1635</v>
       </c>
@@ -12168,6 +12642,13 @@
       </c>
       <c r="S124" s="22">
         <v>11.0</v>
+      </c>
+      <c r="T124" s="22">
+        <v>27</v>
+      </c>
+      <c r="Z124" s="40">
+        <f>AVERAGE(R124:Y124)</f>
+        <v>19.0</v>
       </c>
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.2">
@@ -12189,7 +12670,7 @@
       <c r="N125" s="26"/>
       <c r="O125" s="27"/>
     </row>
-    <row r="126" spans="1:17" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:26" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A126" s="23" t="s">
         <v>1435</v>
       </c>
@@ -12236,6 +12717,13 @@
       <c r="Q126" s="22" t="s">
         <v>1734</v>
       </c>
+      <c r="U126" s="22">
+        <v>48</v>
+      </c>
+      <c r="Z126" s="40">
+        <f>AVERAGE(R126:Y126)</f>
+        <v>48.0</v>
+      </c>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A127" s="23" t="s">
@@ -12340,7 +12828,7 @@
         <v>1773</v>
       </c>
     </row>
-    <row r="129" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A129" s="21" t="s">
         <v>1447</v>
       </c>
@@ -12383,6 +12871,13 @@
       </c>
       <c r="O129" s="24" t="s">
         <v>628</v>
+      </c>
+      <c r="Y129" s="22">
+        <v>53.7</v>
+      </c>
+      <c r="Z129" s="40">
+        <f>AVERAGE(R129:Y129)</f>
+        <v>53.7</v>
       </c>
     </row>
     <row r="130" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -12537,7 +13032,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="134" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A134" s="21" t="s">
         <v>691</v>
       </c>
@@ -12581,8 +13076,15 @@
       <c r="O134" s="24" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="135" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="Y134" s="22">
+        <v>35.4</v>
+      </c>
+      <c r="Z134" s="40">
+        <f>AVERAGE(R134:Y134)</f>
+        <v>35.4</v>
+      </c>
+    </row>
+    <row r="135" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A135" s="21" t="s">
         <v>656</v>
       </c>
@@ -12626,6 +13128,13 @@
       <c r="O135" s="24" t="s">
         <v>662</v>
       </c>
+      <c r="Y135" s="22">
+        <v>67.6</v>
+      </c>
+      <c r="Z135" s="40">
+        <f>AVERAGE(R135:Y135)</f>
+        <v>67.6</v>
+      </c>
     </row>
     <row r="136" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A136" s="23" t="s">
@@ -12992,7 +13501,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="145" spans="1:18" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A145" s="21" t="s">
         <v>696</v>
       </c>
@@ -13040,6 +13549,10 @@
         <v>1787</v>
       </c>
       <c r="R145" s="22" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="Z145" s="40">
+        <f>AVERAGE(R145:Y145)</f>
         <v>2.1</v>
       </c>
     </row>
@@ -13419,7 +13932,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>1780</v>
+        <v>507</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -13430,7 +13943,7 @@
         <v>751</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>1781</v>
+        <v>1789</v>
       </c>
       <c r="C7" s="2"/>
     </row>

</xml_diff>

<commit_message>
NRM1 v5.11: add suggested Std rate and reason columns (AA-AB)
For each of the 47 rows with project evidence, column AA holds a
suggested Refurb & Fit-out Standard rate and AB a one-line reason
(25 raise, 2 lower, 20 keep). Suggestions only: the loader reads no
new column and no rate column changed. Instructions row 24 and the
v5.11 log line mention the columns. 557 tests pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QB69m6diVrBfvTZaLwAazz
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -6229,7 +6229,7 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>Columns T–Y on '2. Rates' hold the other real projects' figures in the row's unit and on this workbook's basis, beside Whitefields (R) and Claycroft (S): T Lakeside S&amp;F (tender Sep 2026, median of 4 bids); U Computer Science decarbonisation (tender Mar 2024, mean of 2 bids); V Scarman Public Toilets Phase 2 (HIGH spec, tender Apr 2026, median of 6 bids; per m² over the 71 m² toilet area); W Co-op grocery store fit-out (Kingfisher contract Aug 2025, 885 m²); X IBRB café servery (Senevo winning bid 2025, 72 m² café, 28 m² servery); Y Riley Court Psychology full refurbishment (Maris signed contract £9.15m, GMP Nov 2024, GIFA 3,850 m²). Each excludes the contractor's prelims, OH&amp;P and design, rebased to Q3 2026 and ÷ 0.94 West Midlands. Column Z is the average of R–Y for the row. Projects differ in scope and specification, so expect spread. Not on '2. Rates': scaffold for envelope works £42 (CS) and £33 (Claycroft) per m² GIFA; retail refrigeration £379 and retailer equipment £373 per m² (Co-op); preliminaries Lakeside ~9%, Whitefields 16.8%, Claycroft 11.3%, Scarman 14%, Co-op 7.2%, IBRB 17.7%, Riley Court 5.5% (+4% contractor PM and design). Evidence only: the app does not read these columns and no rate changed.</t>
+          <t>Columns T–Y on '2. Rates' hold the other real projects' figures in the row's unit and on this workbook's basis, beside Whitefields (R) and Claycroft (S): T Lakeside S&amp;F (tender Sep 2026, median of 4 bids); U Computer Science decarbonisation (tender Mar 2024, mean of 2 bids); V Scarman Public Toilets Phase 2 (HIGH spec, tender Apr 2026, median of 6 bids; per m² over the 71 m² toilet area); W Co-op grocery store fit-out (Kingfisher contract Aug 2025, 885 m²); X IBRB café servery (Senevo winning bid 2025, 72 m² café, 28 m² servery); Y Riley Court Psychology full refurbishment (Maris signed contract £9.15m, GMP Nov 2024, GIFA 3,850 m²). Each excludes the contractor's prelims, OH&amp;P and design, rebased to Q3 2026 and ÷ 0.94 West Midlands. Column Z is the average of R–Y for the row. Projects differ in scope and specification, so expect spread. Not on '2. Rates': scaffold for envelope works £42 (CS) and £33 (Claycroft) per m² GIFA; retail refrigeration £379 and retailer equipment £373 per m² (Co-op); preliminaries Lakeside ~9%, Whitefields 16.8%, Claycroft 11.3%, Scarman 14%, Co-op 7.2%, IBRB 17.7%, Riley Court 5.5% (+4% contractor PM and design). Evidence only: the app does not read these columns and no rate changed. Column AA is Claude's suggested Refurb &amp; Fit-out Standard rate for each row with evidence, and AB the reason (Raise / Lower / Keep). They are suggestions for the owner only: the app does not read them, and a rate changes only when the owner edits the rate columns.</t>
         </is>
       </c>
     </row>
@@ -6728,7 +6728,7 @@
       </c>
       <c r="B81" s="17" t="inlineStr">
         <is>
-          <t>Evidence only, no rates changed. Six more project columns on '2. Rates' beside Whitefields (R) and Claycroft (S), each a plain figure in the row's unit on this workbook's basis: T Lakeside S&amp;F (15 rows), U Computer Science (6), V Scarman Public Toilets Phase 2, high spec (12), W Co-op store fit-out (19), X IBRB café (7), Y Riley Court Psychology refurbishment (27, from the signed contract CSA). Column Z averages R–Y on 47 rows. Row 24 explains the columns and lists the evidence that has no row (scaffold, retail refrigeration and equipment, preliminaries %).</t>
+          <t>Evidence only, no rates changed. Six more project columns on '2. Rates' beside Whitefields (R) and Claycroft (S), each a plain figure in the row's unit on this workbook's basis: T Lakeside S&amp;F (15 rows), U Computer Science (6), V Scarman Public Toilets Phase 2, high spec (12), W Co-op store fit-out (19), X IBRB café (7), Y Riley Court Psychology refurbishment (27, from the signed contract CSA). Column Z averages R–Y on 47 rows. Row 24 explains the columns and lists the evidence that has no row (scaffold, retail refrigeration and equipment, preliminaries %). Columns AA–AB: Claude's suggested Refurb &amp; Fit-out Std rate and the reason, on all 47 rows (25 raise, 2 lower, 20 keep).</t>
         </is>
       </c>
     </row>
@@ -6861,7 +6861,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61613224-FE41-4C03-8B46-4109509C3076}">
-  <dimension ref="A1:Z152"/>
+  <dimension ref="A1:AB152"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.7109375" style="8" customWidth="1"/>
@@ -6882,7 +6882,9 @@
     <col min="19" max="19" width="16.7109375" style="8" customWidth="1"/>
     <col min="20" max="25" width="16.7109375" style="8" customWidth="1"/>
     <col min="26" max="26" width="14.7109375" style="8" customWidth="1"/>
-    <col min="27" max="16384" width="9.140625" style="8"/>
+    <col min="27" max="27" width="14.7109375" style="8" customWidth="1"/>
+    <col min="28" max="28" width="60.7109375" style="8" customWidth="1"/>
+    <col min="29" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="18" x14ac:dyDescent="0.25">
@@ -6900,7 +6902,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:28" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>756</v>
       </c>
@@ -6991,6 +6993,16 @@
       <c r="Z5" s="12" t="inlineStr">
         <is>
           <t>Average of project rates (mean of columns R–Y that hold a figure for this row. Projects differ in scope and specification, so read it with the column notes. Evidence only — the app does not read it)</t>
+        </is>
+      </c>
+      <c r="AA5" s="12" t="inlineStr">
+        <is>
+          <t>Suggested Refurb &amp; Fit-out Std rate (Claude's suggestion from the project columns R–Y, 4 Oct 2026, for the owner to accept, change or ignore. Evidence only — the app does not read it)</t>
+        </is>
+      </c>
+      <c r="AB5" s="12" t="inlineStr">
+        <is>
+          <t>Reason for the suggestion</t>
         </is>
       </c>
     </row>
@@ -7013,7 +7025,7 @@
       <c r="N6" s="19"/>
       <c r="O6" s="20"/>
     </row>
-    <row r="7" spans="1:26" ht="51" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:28" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
         <v>72</v>
       </c>
@@ -7061,8 +7073,16 @@
         <f>AVERAGE(R7:Y7)</f>
         <v>8.1</v>
       </c>
-    </row>
-    <row r="8" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="AA7" s="40">
+        <v>25</v>
+      </c>
+      <c r="AB7" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Matches Mace pre-tender allowance (£24.5); one low tender (£8) is not enough to cut it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:28" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
         <v>82</v>
       </c>
@@ -7110,8 +7130,16 @@
         <f>AVERAGE(R8:Y8)</f>
         <v>73.3</v>
       </c>
-    </row>
-    <row r="9" spans="1:26" ht="78.5" x14ac:dyDescent="0.2">
+      <c r="AA8" s="40">
+        <v>100</v>
+      </c>
+      <c r="AB8" s="22" t="inlineStr">
+        <is>
+          <t>Lower. Whitefields £73 on simple 2-storey masonry; £100 leaves room for framed or taller buildings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="78.5" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
         <v>96</v>
       </c>
@@ -7174,6 +7202,14 @@
         <f>AVERAGE(R9:Y9)</f>
         <v>72.933333</v>
       </c>
+      <c r="AA9" s="40">
+        <v>55</v>
+      </c>
+      <c r="AB9" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside, Claycroft, Co-op and Riley Court all £49–55. Scarman and IBRB are tiny jobs.</t>
+        </is>
+      </c>
     </row>
     <row r="10" spans="1:16" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
@@ -7290,7 +7326,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:28" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
         <v>119</v>
       </c>
@@ -7335,6 +7371,14 @@
       <c r="Z13" s="40">
         <f>AVERAGE(R13:Y13)</f>
         <v>36.3</v>
+      </c>
+      <c r="AA13" s="40">
+        <v>100</v>
+      </c>
+      <c r="AB13" s="22" t="inlineStr">
+        <is>
+          <t>Keep. One water-main job (£36); diversions are too site-specific to move the rate.</t>
+        </is>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -7767,7 +7811,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="25" spans="1:26" ht="218.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:28" ht="218.75" x14ac:dyDescent="0.2">
       <c r="A25" s="21" t="s">
         <v>1669</v>
       </c>
@@ -7826,8 +7870,16 @@
         <f>AVERAGE(R25:Y25)</f>
         <v>349.45</v>
       </c>
-    </row>
-    <row r="26" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="AA25" s="40">
+        <v>190</v>
+      </c>
+      <c r="AB25" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Computer Science £182 per m² footprint. Claycroft metal over-roof £517 is a High case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:28" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A26" s="21" t="s">
         <v>1659</v>
       </c>
@@ -7876,8 +7928,16 @@
         <f>AVERAGE(R26:Y26)</f>
         <v>32.0</v>
       </c>
-    </row>
-    <row r="27" spans="1:26" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="AA26" s="40">
+        <v>32</v>
+      </c>
+      <c r="AB26" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside tender.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:28" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A27" s="21" t="s">
         <v>197</v>
       </c>
@@ -7934,8 +7994,16 @@
         <f>AVERAGE(R27:Y27)</f>
         <v>109.25</v>
       </c>
-    </row>
-    <row r="28" spans="1:26" ht="165.75" x14ac:dyDescent="0.2">
+      <c r="AA27" s="40">
+        <v>100</v>
+      </c>
+      <c r="AB27" s="22" t="inlineStr">
+        <is>
+          <t>Raise. CS part render £48; Riley Court full envelope upgrade £171 (cladding, insulated linings).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="1:28" ht="165.75" x14ac:dyDescent="0.2">
       <c r="A28" s="21" t="s">
         <v>203</v>
       </c>
@@ -7995,8 +8063,16 @@
         <f>AVERAGE(R28:Y28)</f>
         <v>127.033333</v>
       </c>
-    </row>
-    <row r="29" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="AA28" s="40">
+        <v>140</v>
+      </c>
+      <c r="AB28" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court new windows £147; CS triple glazing £210 (High). Co-op was refinish only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A29" s="21" t="s">
         <v>208</v>
       </c>
@@ -8050,8 +8126,16 @@
         <f>AVERAGE(R29:Y29)</f>
         <v>136.65</v>
       </c>
-    </row>
-    <row r="30" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="AA29" s="40">
+        <v>150</v>
+      </c>
+      <c r="AB29" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £247 (acoustic academic partitions); Co-op £26 was a light shop fit-out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A30" s="21" t="s">
         <v>1142</v>
       </c>
@@ -8108,8 +8192,16 @@
         <f>AVERAGE(R30:Y30)</f>
         <v>90.6</v>
       </c>
-    </row>
-    <row r="31" spans="1:26" ht="155.0" x14ac:dyDescent="0.2">
+      <c r="AA30" s="40">
+        <v>100</v>
+      </c>
+      <c r="AB30" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £164, Scarman £99; Co-op £9 reused most doors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" spans="1:28" ht="155.0" x14ac:dyDescent="0.2">
       <c r="A31" s="21" t="s">
         <v>1146</v>
       </c>
@@ -8172,6 +8264,14 @@
       <c r="Z31" s="40">
         <f>AVERAGE(R31:Y31)</f>
         <v>30.46</v>
+      </c>
+      <c r="AA31" s="40">
+        <v>30</v>
+      </c>
+      <c r="AB31" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Most projects £3–24; Claycroft £96 out-turn (surveyed occupied residential) is a High case.</t>
+        </is>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
@@ -8193,7 +8293,7 @@
       <c r="N32" s="26"/>
       <c r="O32" s="27"/>
     </row>
-    <row r="33" spans="1:26" ht="91.25" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:28" ht="91.25" x14ac:dyDescent="0.2">
       <c r="A33" s="21" t="s">
         <v>221</v>
       </c>
@@ -8262,8 +8362,16 @@
         <f>AVERAGE(R33:Y33)</f>
         <v>98.383333</v>
       </c>
-    </row>
-    <row r="34" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="AA33" s="40">
+        <v>75</v>
+      </c>
+      <c r="AB33" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside £72, Claycroft £99, Riley Court £39 (decoration only). Scarman is toilet-area only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A34" s="23" t="s">
         <v>1153</v>
       </c>
@@ -8325,6 +8433,14 @@
         <f>AVERAGE(R34:Y34)</f>
         <v>97.933333</v>
       </c>
+      <c r="AA34" s="40">
+        <v>85</v>
+      </c>
+      <c r="AB34" s="22" t="inlineStr">
+        <is>
+          <t>Raise slightly. Riley Court £95 full replacement; Co-op £22 kept its floor. Scarman is toilet-area only.</t>
+        </is>
+      </c>
     </row>
     <row r="35" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A35" s="23" t="s">
@@ -8373,7 +8489,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="36" spans="1:26" ht="65.75" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:28" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A36" s="23" t="s">
         <v>1655</v>
       </c>
@@ -8431,8 +8547,16 @@
         <f>AVERAGE(R36:Y36)</f>
         <v>44.7</v>
       </c>
-    </row>
-    <row r="37" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="AA36" s="40">
+        <v>50</v>
+      </c>
+      <c r="AB36" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside £51, Claycroft £38.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A37" s="21" t="s">
         <v>1671</v>
       </c>
@@ -8492,8 +8616,16 @@
         <f>AVERAGE(R37:Y37)</f>
         <v>86.533333</v>
       </c>
-    </row>
-    <row r="38" spans="1:26" ht="104.0" x14ac:dyDescent="0.2">
+      <c r="AA37" s="40">
+        <v>80</v>
+      </c>
+      <c r="AB37" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £110 new suspended ceilings; Co-op £21 painted soffits only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:28" ht="104.0" x14ac:dyDescent="0.2">
       <c r="A38" s="21" t="s">
         <v>1650</v>
       </c>
@@ -8548,6 +8680,14 @@
       <c r="Z38" s="40">
         <f>AVERAGE(R38:Y38)</f>
         <v>50.2</v>
+      </c>
+      <c r="AA38" s="40">
+        <v>30</v>
+      </c>
+      <c r="AB38" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside £30; Claycroft £70 was full replacement (High case).</t>
+        </is>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.2">
@@ -8569,7 +8709,7 @@
       <c r="N39" s="26"/>
       <c r="O39" s="27"/>
     </row>
-    <row r="40" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:28" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A40" s="48" t="s">
         <v>1164</v>
       </c>
@@ -8626,8 +8766,16 @@
         <f>AVERAGE(R40:Y40)</f>
         <v>11113.0</v>
       </c>
-    </row>
-    <row r="41" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="AA40" s="40">
+        <v>7000</v>
+      </c>
+      <c r="AB40" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Scarman £7,650 (high spec) and Riley Court £14,600 incl. tiling both far above £3,950.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:28" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A41" s="48" t="s">
         <v>1169</v>
       </c>
@@ -8678,6 +8826,14 @@
         <f>AVERAGE(R41:Y41)</f>
         <v>16025.0</v>
       </c>
+      <c r="AA41" s="40">
+        <v>9000</v>
+      </c>
+      <c r="AB41" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £16,000 per accessible WC incl. tiling and shower; £5,500 too low.</t>
+        </is>
+      </c>
     </row>
     <row r="42" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A42" s="43" t="s">
@@ -8722,7 +8878,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="43" spans="1:26" ht="104.0" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:28" ht="104.0" x14ac:dyDescent="0.2">
       <c r="A43" s="48" t="s">
         <v>1175</v>
       </c>
@@ -8781,6 +8937,14 @@
         <f>AVERAGE(R43:Y43)</f>
         <v>3216.0</v>
       </c>
+      <c r="AA43" s="40">
+        <v>2500</v>
+      </c>
+      <c r="AB43" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside £2,563; Claycroft £3,869 sits between Std and High.</t>
+        </is>
+      </c>
     </row>
     <row r="44" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A44" s="48" t="s">
@@ -8874,7 +9038,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="46" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A46" s="48" t="s">
         <v>1188</v>
       </c>
@@ -8930,8 +9094,16 @@
         <f>AVERAGE(R46:Y46)</f>
         <v>5296.0</v>
       </c>
-    </row>
-    <row r="47" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="AA46" s="40">
+        <v>5300</v>
+      </c>
+      <c r="AB46" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside tender £5,296.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:28" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A47" s="48" t="s">
         <v>1194</v>
       </c>
@@ -8984,8 +9156,16 @@
         <f>AVERAGE(R47:Y47)</f>
         <v>10276.0</v>
       </c>
-    </row>
-    <row r="48" spans="1:26" ht="65.75" x14ac:dyDescent="0.2">
+      <c r="AA47" s="40">
+        <v>6000</v>
+      </c>
+      <c r="AB47" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court about £10,300 per tea point (8 assumed); your own review said £5,500.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="1:28" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A48" s="21" t="s">
         <v>292</v>
       </c>
@@ -9045,8 +9225,16 @@
         <f>AVERAGE(R48:Y48)</f>
         <v>37.5</v>
       </c>
-    </row>
-    <row r="49" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="AA48" s="40">
+        <v>45</v>
+      </c>
+      <c r="AB48" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Riley Court £42, Claycroft £64, Co-op £7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A49" s="21" t="s">
         <v>1199</v>
       </c>
@@ -9100,6 +9288,14 @@
         <f>AVERAGE(R49:Y49)</f>
         <v>14.3</v>
       </c>
+      <c r="AA49" s="40">
+        <v>12</v>
+      </c>
+      <c r="AB49" s="22" t="inlineStr">
+        <is>
+          <t>Raise slightly. Riley Court £12, Co-op £16 (incl. graphics).</t>
+        </is>
+      </c>
     </row>
     <row r="50" spans="1:16" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A50" s="21" t="s">
@@ -9326,7 +9522,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="55" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:28" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A55" s="21" t="s">
         <v>1216</v>
       </c>
@@ -9374,6 +9570,14 @@
       <c r="Z55" s="40">
         <f>AVERAGE(R55:Y55)</f>
         <v>1438.0</v>
+      </c>
+      <c r="AA55" s="40">
+        <v>1000</v>
+      </c>
+      <c r="AB55" s="22" t="inlineStr">
+        <is>
+          <t>Raise. IBRB café servery £1,438 (bespoke stainless) = High; your own review said Std £1,000.</t>
+        </is>
       </c>
     </row>
     <row r="56" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -9690,7 +9894,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="64" spans="1:26" ht="140.25" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:28" ht="140.25" x14ac:dyDescent="0.2">
       <c r="A64" s="55" t="s">
         <v>1027</v>
       </c>
@@ -9749,6 +9953,14 @@
         <f>AVERAGE(R64:Y64)</f>
         <v>224.0</v>
       </c>
+      <c r="AA64" s="40">
+        <v>190</v>
+      </c>
+      <c r="AB64" s="22" t="inlineStr">
+        <is>
+          <t>Raise. CS whole heat pump M&amp;E package £224; enter as a figure, not = 5.1a × factor.</t>
+        </is>
+      </c>
     </row>
     <row r="65" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A65" s="55" t="s">
@@ -9800,7 +10012,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="66" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A66" s="55" t="s">
         <v>1252</v>
       </c>
@@ -9856,6 +10068,14 @@
         <f>AVERAGE(R66:Y66)</f>
         <v>134.7</v>
       </c>
+      <c r="AA66" s="40">
+        <v>120</v>
+      </c>
+      <c r="AB66" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £135 incl. new LTHW pipework, radiators and pumps off district heating.</t>
+        </is>
+      </c>
     </row>
     <row r="67" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A67" s="55" t="s">
@@ -10407,7 +10627,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="78" spans="1:26" ht="91.25" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:28" ht="91.25" x14ac:dyDescent="0.2">
       <c r="A78" s="23" t="s">
         <v>1299</v>
       </c>
@@ -10475,8 +10695,16 @@
         <f>AVERAGE(R78:Y78)</f>
         <v>98.92</v>
       </c>
-    </row>
-    <row r="79" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="AA78" s="40">
+        <v>80</v>
+      </c>
+      <c r="AB78" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £105, IBRB £124 (small café); Claycroft £39 and Co-op £18 were partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A79" s="23" t="s">
         <v>1304</v>
       </c>
@@ -10535,8 +10763,16 @@
         <f>AVERAGE(R79:Y79)</f>
         <v>20.0</v>
       </c>
-    </row>
-    <row r="80" spans="1:26" ht="78.5" x14ac:dyDescent="0.2">
+      <c r="AA79" s="40">
+        <v>19.5</v>
+      </c>
+      <c r="AB79" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside £20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:28" ht="78.5" x14ac:dyDescent="0.2">
       <c r="A80" s="21" t="s">
         <v>1672</v>
       </c>
@@ -10595,8 +10831,16 @@
         <f>AVERAGE(R80:Y80)</f>
         <v>122.75</v>
       </c>
-    </row>
-    <row r="81" spans="1:26" ht="91.25" x14ac:dyDescent="0.2">
+      <c r="AA80" s="40">
+        <v>100</v>
+      </c>
+      <c r="AB80" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court MVHR £172, Co-op £73, Claycroft out-turn £92.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:28" ht="91.25" x14ac:dyDescent="0.2">
       <c r="A81" s="21" t="s">
         <v>1644</v>
       </c>
@@ -10655,8 +10899,16 @@
         <f>AVERAGE(R81:Y81)</f>
         <v>36.233333</v>
       </c>
-    </row>
-    <row r="82" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="AA81" s="40">
+        <v>22</v>
+      </c>
+      <c r="AB81" s="22" t="inlineStr">
+        <is>
+          <t>Raise slightly. Lakeside £18.5, Claycroft £28; Scarman £62 is toilet-area only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A82" s="21" t="s">
         <v>420</v>
       </c>
@@ -10710,8 +10962,16 @@
         <f>AVERAGE(R82:Y82)</f>
         <v>36.8</v>
       </c>
-    </row>
-    <row r="83" spans="1:26" ht="40.25" x14ac:dyDescent="0.2">
+      <c r="AA82" s="40">
+        <v>75</v>
+      </c>
+      <c r="AB82" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Riley Court £34 and Co-op £40 cooled only some rooms; no whole-building evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" spans="1:28" ht="40.25" x14ac:dyDescent="0.2">
       <c r="A83" s="21" t="s">
         <v>373</v>
       </c>
@@ -10771,6 +11031,14 @@
         <f>AVERAGE(R83:Y83)</f>
         <v>24.966667</v>
       </c>
+      <c r="AA83" s="40">
+        <v>25</v>
+      </c>
+      <c r="AB83" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £59 (full BMS budget); Co-op £11.5; Claycroft £4 interfaces only.</t>
+        </is>
+      </c>
     </row>
     <row r="84" spans="1:15" ht="51" x14ac:dyDescent="0.2">
       <c r="A84" s="55" t="s">
@@ -10893,7 +11161,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="87" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:28" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A87" s="23" t="s">
         <v>1328</v>
       </c>
@@ -10955,8 +11223,16 @@
         <f>AVERAGE(R87:Y87)</f>
         <v>133.525</v>
       </c>
-    </row>
-    <row r="88" spans="1:26" ht="116.75" x14ac:dyDescent="0.2">
+      <c r="AA87" s="40">
+        <v>126</v>
+      </c>
+      <c r="AB87" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Riley Court £131, Scarman £97, Co-op £89. IBRB £218 is one supply on a small room.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" spans="1:28" ht="116.75" x14ac:dyDescent="0.2">
       <c r="A88" s="23" t="s">
         <v>1332</v>
       </c>
@@ -11015,6 +11291,14 @@
         <f>AVERAGE(R88:Y88)</f>
         <v>155.35</v>
       </c>
+      <c r="AA88" s="40">
+        <v>150</v>
+      </c>
+      <c r="AB88" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside £153, Claycroft £158.</t>
+        </is>
+      </c>
     </row>
     <row r="89" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A89" s="23" t="s">
@@ -11059,7 +11343,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="90" spans="1:26" ht="65.75" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:28" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A90" s="23" t="s">
         <v>1338</v>
       </c>
@@ -11127,6 +11411,14 @@
         <f>AVERAGE(R90:Y90)</f>
         <v>105.36</v>
       </c>
+      <c r="AA90" s="40">
+        <v>80</v>
+      </c>
+      <c r="AB90" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Five projects £51–198 (median £84); £33 is far too low.</t>
+        </is>
+      </c>
     </row>
     <row r="91" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A91" s="23" t="s">
@@ -11460,7 +11752,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="99" spans="1:26" ht="65.75" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:28" ht="65.75" x14ac:dyDescent="0.2">
       <c r="A99" s="21" t="s">
         <v>507</v>
       </c>
@@ -11526,6 +11818,14 @@
         <f>AVERAGE(R99:Y99)</f>
         <v>46.44</v>
       </c>
+      <c r="AA99" s="40">
+        <v>35</v>
+      </c>
+      <c r="AB99" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £44, Claycroft £65, Scarman £77 for new systems; Lakeside £19 was partial.</t>
+        </is>
+      </c>
     </row>
     <row r="100" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A100" s="21" t="s">
@@ -11613,7 +11913,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="102" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A102" s="21" t="s">
         <v>1674</v>
       </c>
@@ -11673,8 +11973,16 @@
         <f>AVERAGE(R102:Y102)</f>
         <v>19.433333</v>
       </c>
-    </row>
-    <row r="103" spans="1:26" ht="53.0" x14ac:dyDescent="0.2">
+      <c r="AA102" s="40">
+        <v>20</v>
+      </c>
+      <c r="AB102" s="22" t="inlineStr">
+        <is>
+          <t>Raise slightly. Lakeside £19, Riley Court £34, IBRB £5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" spans="1:28" ht="53.0" x14ac:dyDescent="0.2">
       <c r="A103" s="21" t="s">
         <v>1640</v>
       </c>
@@ -11730,8 +12038,16 @@
         <f>AVERAGE(R103:Y103)</f>
         <v>21.9</v>
       </c>
-    </row>
-    <row r="104" spans="1:26" x14ac:dyDescent="0.2" ht="53.0" customHeight="1">
+      <c r="AA103" s="40">
+        <v>25</v>
+      </c>
+      <c r="AB103" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside £24.5, Claycroft £19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" spans="1:28" x14ac:dyDescent="0.2" ht="53.0" customHeight="1">
       <c r="A104" s="21" t="s">
         <v>563</v>
       </c>
@@ -11791,8 +12107,16 @@
         <f>AVERAGE(R104:Y104)</f>
         <v>28.1</v>
       </c>
-    </row>
-    <row r="105" spans="1:26" ht="53.0" x14ac:dyDescent="0.2">
+      <c r="AA104" s="40">
+        <v>20</v>
+      </c>
+      <c r="AB104" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £22, Co-op £58 (retail CCTV and alarm); Claycroft £4.5 minimal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" spans="1:28" ht="53.0" x14ac:dyDescent="0.2">
       <c r="A105" s="23" t="s">
         <v>1381</v>
       </c>
@@ -11848,6 +12172,14 @@
         <f>AVERAGE(R105:Y105)</f>
         <v>112847.0</v>
       </c>
+      <c r="AA105" s="40">
+        <v>100000</v>
+      </c>
+      <c r="AB105" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Claycroft £112,850 for a replacement passenger lift; £40,000 is a third of that.</t>
+        </is>
+      </c>
     </row>
     <row r="106" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A106" s="23" t="s">
@@ -12540,7 +12872,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="123" spans="1:26" ht="51" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:28" ht="51" x14ac:dyDescent="0.2">
       <c r="A123" s="21" t="s">
         <v>1675</v>
       </c>
@@ -12595,8 +12927,16 @@
         <f>AVERAGE(R123:Y123)</f>
         <v>5.55</v>
       </c>
-    </row>
-    <row r="124" spans="1:26" ht="78.5" x14ac:dyDescent="0.2">
+      <c r="AA123" s="40">
+        <v>12</v>
+      </c>
+      <c r="AB123" s="22" t="inlineStr">
+        <is>
+          <t>Lower. CS £8, Co-op £3; most builder's work sits inside the M&amp;E prices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" spans="1:28" ht="78.5" x14ac:dyDescent="0.2">
       <c r="A124" s="21" t="s">
         <v>1635</v>
       </c>
@@ -12649,6 +12989,14 @@
       <c r="Z124" s="40">
         <f>AVERAGE(R124:Y124)</f>
         <v>19.0</v>
+      </c>
+      <c r="AA124" s="40">
+        <v>27</v>
+      </c>
+      <c r="AB124" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Lakeside £27 (rewire of occupied flats); Claycroft £11.</t>
+        </is>
       </c>
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.2">
@@ -12670,7 +13018,7 @@
       <c r="N125" s="26"/>
       <c r="O125" s="27"/>
     </row>
-    <row r="126" spans="1:26" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:28" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A126" s="23" t="s">
         <v>1435</v>
       </c>
@@ -12724,6 +13072,14 @@
         <f>AVERAGE(R126:Y126)</f>
         <v>48.0</v>
       </c>
+      <c r="AA126" s="40">
+        <v>45</v>
+      </c>
+      <c r="AB126" s="22" t="inlineStr">
+        <is>
+          <t>Keep. CS brick remedials £48.</t>
+        </is>
+      </c>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A127" s="23" t="s">
@@ -12828,7 +13184,7 @@
         <v>1773</v>
       </c>
     </row>
-    <row r="129" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:28" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A129" s="21" t="s">
         <v>1447</v>
       </c>
@@ -12878,6 +13234,14 @@
       <c r="Z129" s="40">
         <f>AVERAGE(R129:Y129)</f>
         <v>53.7</v>
+      </c>
+      <c r="AA129" s="40">
+        <v>60</v>
+      </c>
+      <c r="AB129" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Riley Court £54.</t>
+        </is>
       </c>
     </row>
     <row r="130" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">
@@ -13032,7 +13396,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="134" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A134" s="21" t="s">
         <v>691</v>
       </c>
@@ -13083,8 +13447,16 @@
         <f>AVERAGE(R134:Y134)</f>
         <v>35.4</v>
       </c>
-    </row>
-    <row r="135" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="AA134" s="40">
+        <v>15</v>
+      </c>
+      <c r="AB134" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £35 for new internal below-ground drainage (one project).</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A135" s="21" t="s">
         <v>656</v>
       </c>
@@ -13135,6 +13507,14 @@
         <f>AVERAGE(R135:Y135)</f>
         <v>67.6</v>
       </c>
+      <c r="AA135" s="40">
+        <v>25</v>
+      </c>
+      <c r="AB135" s="22" t="inlineStr">
+        <is>
+          <t>Raise. Riley Court £68 for new district heating and water mains (one project; site-specific).</t>
+        </is>
+      </c>
     </row>
     <row r="136" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A136" s="23" t="s">
@@ -13501,7 +13881,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="145" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:28" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A145" s="21" t="s">
         <v>696</v>
       </c>
@@ -13554,6 +13934,14 @@
       <c r="Z145" s="40">
         <f>AVERAGE(R145:Y145)</f>
         <v>2.1</v>
+      </c>
+      <c r="AA145" s="40">
+        <v>30</v>
+      </c>
+      <c r="AB145" s="22" t="inlineStr">
+        <is>
+          <t>Keep. Whitefields £2 was topsoil and seed only, not planting.</t>
+        </is>
       </c>
     </row>
     <row r="146" spans="1:15" ht="25.5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
NRM1 v5.12: apply the owner's approved rates from the project evidence
The owner marked v5.11's suggestion column: green = accept (42 rows),
amber = his figure (ventilation 75, passenger lift 60,000, foul drainage
10), red = no change (toilets, accessible WCs). 25 rows change; Basic,
High and New build Std/High move by the same ratio as Standard.

5.1b and 5.1d become figures (were = 5.1a x factor); rows derived from
them and 5.8b stay formulas with refreshed cached values. 5.2b is frozen
at its figures so it keeps 19.5. Changed rows' Source = 'Your figure'.

Tests: rate pins moved with the owner's figures; the report dagger test
now uses the ground source heat pump (still unverified). 557 pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QB69m6diVrBfvTZaLwAazz
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4236" uniqueCount="1790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4236" uniqueCount="1791">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5401,6 +5401,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.12 (October 2026)</t>
   </si>
 </sst>
 </file>
@@ -6021,7 +6024,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BBCD35-3C7D-4CAC-A46E-6C3CC3E31849}">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.7109375" style="8" customWidth="1"/>
@@ -6032,7 +6035,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1788</v>
+        <v>1790</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -6723,136 +6726,148 @@
     <row r="81" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="17" t="inlineStr">
         <is>
+          <t>v5.12 — 4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B81" s="17" t="inlineStr">
+        <is>
+          <t>Rates updated from the owner's review of the v5.11 suggestions (column AA marked green = accept, amber = owner's figure, red = no change). 25 rows changed; each row's Basic, Standard, High and New build Std / High move by the same ratio as Standard (new Std ÷ old Std), rounded. Std (Refurb &amp; Fit-out): demolition 130→100; roof 110→190; external walls 60→100; windows 120→140; internal walls 110→150; internal doors 60→100; floor finishes 75→85; ceilings 50→80; staff kitchenette 4,000→6,000; signage 10→12; catering kitchen 690→1,000; ASHP full system 78→190 and district heating full system 54→120 (now figures, not = 5.1a × factor; their plant-only / radiators-only rows still follow by formula); water and drainage 65→80; ventilation 45→75 (owner); extract fans 19→22; BMS 15→25; lighting 33→80 (5.8b follows at 75%); fire alarm 18→35; data 18→20; security 15→20; passenger lift 40,000→60,000 (owner); builder's work 18→12; foul drainage 6→10 (owner); external utilities 10→25. Kept: toilets and accessible WCs (owner: no change) and the 20 'keep' rows; 5.2b visible-fittings water fixed at its figures (19.5 Std, Lakeside tender) so it does not follow 5.2a. Changed rows' Source = 'Your figure'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="17" t="inlineStr">
+        <is>
           <t>v5.11 — 4 Oct 2026</t>
         </is>
       </c>
-      <c r="B81" s="17" t="inlineStr">
+      <c r="B82" s="17" t="inlineStr">
         <is>
           <t>Evidence only, no rates changed. Six more project columns on '2. Rates' beside Whitefields (R) and Claycroft (S), each a plain figure in the row's unit on this workbook's basis: T Lakeside S&amp;F (15 rows), U Computer Science (6), V Scarman Public Toilets Phase 2, high spec (12), W Co-op store fit-out (19), X IBRB café (7), Y Riley Court Psychology refurbishment (27, from the signed contract CSA). Column Z averages R–Y on 47 rows. Row 24 explains the columns and lists the evidence that has no row (scaffold, retail refrigeration and equipment, preliminaries %). Columns AA–AB: Claude's suggested Refurb &amp; Fit-out Std rate and the reason, on all 47 rows (25 raise, 2 lower, 20 keep).</t>
         </is>
       </c>
     </row>
-    <row r="82" spans="1:3" s="54" customFormat="1" ht="104.0" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="17" t="s">
+    <row r="83" spans="1:3" s="54" customFormat="1" ht="104.0" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="17" t="s">
         <v>1778</v>
       </c>
-      <c r="B82" s="17" t="s">
+      <c r="B83" s="17" t="s">
         <v>1779</v>
       </c>
-      <c r="C82" s="60"/>
-    </row>
-    <row r="83" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="17" t="s">
+      <c r="C83" s="60"/>
+    </row>
+    <row r="84" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="17" t="s">
         <v>1748</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B84" s="17" t="s">
         <v>1783</v>
-      </c>
-      <c r="C83" s="60"/>
-    </row>
-    <row r="84" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A84" s="17" t="s">
-        <v>1722</v>
-      </c>
-      <c r="B84" s="17" t="s">
-        <v>1737</v>
       </c>
       <c r="C84" s="60"/>
     </row>
     <row r="85" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A85" s="17" t="s">
-        <v>1711</v>
+        <v>1722</v>
       </c>
       <c r="B85" s="17" t="s">
-        <v>1712</v>
+        <v>1737</v>
       </c>
       <c r="C85" s="60"/>
     </row>
     <row r="86" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A86" s="17" t="s">
+        <v>1711</v>
+      </c>
+      <c r="B86" s="17" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C86" s="60"/>
+    </row>
+    <row r="87" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A87" s="17" t="s">
         <v>1632</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B87" s="17" t="s">
         <v>1634</v>
       </c>
-      <c r="C86" s="60"/>
-    </row>
-    <row r="87" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A87" s="15" t="s">
+      <c r="C87" s="60"/>
+    </row>
+    <row r="88" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A88" s="15" t="s">
         <v>1620</v>
       </c>
-      <c r="B87" s="17" t="s">
+      <c r="B88" s="17" t="s">
         <v>1621</v>
       </c>
-      <c r="C87" s="33"/>
-    </row>
-    <row r="88" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A88" s="15" t="s">
+      <c r="C88" s="33"/>
+    </row>
+    <row r="89" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A89" s="15" t="s">
         <v>1060</v>
       </c>
-      <c r="B88" s="17" t="s">
+      <c r="B89" s="17" t="s">
         <v>1061</v>
       </c>
-      <c r="C88" s="33"/>
-    </row>
-    <row r="89" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A89" s="15" t="s">
+      <c r="C89" s="33"/>
+    </row>
+    <row r="90" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A90" s="15" t="s">
         <v>1051</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="B90" s="17" t="s">
         <v>1052</v>
       </c>
-      <c r="C89" s="33"/>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A90" s="15" t="s">
+      <c r="C90" s="33"/>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B90" s="17" t="s">
+      <c r="B91" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C90" s="33"/>
-    </row>
-    <row r="91" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A91" s="15" t="s">
+      <c r="C91" s="33"/>
+    </row>
+    <row r="92" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A92" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B91" s="17" t="s">
+      <c r="B92" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C91" s="33"/>
-    </row>
-    <row r="92" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A92" s="15" t="s">
+      <c r="C92" s="33"/>
+    </row>
+    <row r="93" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A93" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B92" s="17" t="s">
+      <c r="B93" s="17" t="s">
         <v>28</v>
-      </c>
-      <c r="C92" s="33"/>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A93" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B93" s="17" t="s">
-        <v>30</v>
       </c>
       <c r="C93" s="33"/>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B94" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C94" s="33"/>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B94" s="17" t="s">
+      <c r="B95" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C94" s="33"/>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A95" s="15"/>
-      <c r="B95" s="17"/>
       <c r="C95" s="33"/>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96" s="15"/>
+      <c r="B96" s="17"/>
+      <c r="C96" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7104,15 +7119,17 @@
       </c>
       <c r="H8" s="39"/>
       <c r="I8" s="40">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="J8" s="39"/>
       <c r="K8" s="40">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="L8" s="39"/>
-      <c r="M8" s="22" t="s">
-        <v>1076</v>
+      <c r="M8" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N8" s="22" t="s">
         <v>1080</v>
@@ -7834,22 +7851,24 @@
         <v>705</v>
       </c>
       <c r="H25" s="39">
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="I25" s="40">
-        <v>110</v>
+        <v>190</v>
       </c>
       <c r="J25" s="39">
-        <v>200</v>
+        <v>345</v>
       </c>
       <c r="K25" s="40">
-        <v>220</v>
+        <v>380</v>
       </c>
       <c r="L25" s="39">
-        <v>300</v>
-      </c>
-      <c r="M25" s="22" t="s">
-        <v>1098</v>
+        <v>518</v>
+      </c>
+      <c r="M25" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N25" s="22" t="s">
         <v>1132</v>
@@ -7958,22 +7977,24 @@
         <v>1075</v>
       </c>
       <c r="H27" s="39">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I27" s="40">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="J27" s="39">
-        <v>110</v>
+        <v>183</v>
       </c>
       <c r="K27" s="40">
-        <v>220</v>
+        <v>367</v>
       </c>
       <c r="L27" s="39">
-        <v>340</v>
-      </c>
-      <c r="M27" s="22" t="s">
-        <v>1098</v>
+        <v>567</v>
+      </c>
+      <c r="M27" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N27" s="22" t="s">
         <v>1135</v>
@@ -8024,22 +8045,24 @@
         <v>1075</v>
       </c>
       <c r="H28" s="39">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="I28" s="40">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="J28" s="39">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="K28" s="40">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="L28" s="39">
-        <v>260</v>
-      </c>
-      <c r="M28" s="22" t="s">
-        <v>1098</v>
+        <v>303</v>
+      </c>
+      <c r="M28" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N28" s="22" t="s">
         <v>1138</v>
@@ -8093,22 +8116,24 @@
         <v>1075</v>
       </c>
       <c r="H29" s="39">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I29" s="40">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="J29" s="39">
-        <v>160</v>
+        <v>218</v>
       </c>
       <c r="K29" s="40">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="L29" s="39">
-        <v>160</v>
-      </c>
-      <c r="M29" s="22" t="s">
-        <v>1098</v>
+        <v>218</v>
+      </c>
+      <c r="M29" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N29" s="22" t="s">
         <v>1141</v>
@@ -8156,22 +8181,24 @@
         <v>1075</v>
       </c>
       <c r="H30" s="39">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I30" s="40">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="J30" s="39">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="K30" s="40">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="L30" s="39">
-        <v>120</v>
-      </c>
-      <c r="M30" s="22" t="s">
-        <v>1098</v>
+        <v>200</v>
+      </c>
+      <c r="M30" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N30" s="22" t="s">
         <v>1145</v>
@@ -8394,22 +8421,24 @@
         <v>1075</v>
       </c>
       <c r="H34" s="39">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="I34" s="40">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="J34" s="39">
-        <v>200</v>
+        <v>227</v>
       </c>
       <c r="K34" s="40">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="L34" s="39">
-        <v>200</v>
-      </c>
-      <c r="M34" s="22" t="s">
-        <v>1118</v>
+        <v>227</v>
+      </c>
+      <c r="M34" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N34" s="22" t="s">
         <v>1156</v>
@@ -8577,22 +8606,24 @@
         <v>1075</v>
       </c>
       <c r="H37" s="39">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="I37" s="40">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="J37" s="39">
-        <v>140</v>
+        <v>224</v>
       </c>
       <c r="K37" s="40">
-        <v>70</v>
+        <v>112</v>
       </c>
       <c r="L37" s="39">
-        <v>140</v>
-      </c>
-      <c r="M37" s="22" t="s">
-        <v>1098</v>
+        <v>224</v>
+      </c>
+      <c r="M37" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N37" s="22" t="s">
         <v>1162</v>
@@ -8771,7 +8802,7 @@
       </c>
       <c r="AB40" s="22" t="inlineStr">
         <is>
-          <t>Raise. Scarman £7,650 (high spec) and Riley Court £14,600 incl. tiling both far above £3,950.</t>
+          <t>Keep as is (owner, 4 Oct 2026).</t>
         </is>
       </c>
     </row>
@@ -8831,7 +8862,7 @@
       </c>
       <c r="AB41" s="22" t="inlineStr">
         <is>
-          <t>Raise. Riley Court £16,000 per accessible WC incl. tiling and shower; £5,500 too low.</t>
+          <t>Keep as is (owner, 4 Oct 2026).</t>
         </is>
       </c>
     </row>
@@ -9126,22 +9157,24 @@
         <v>1626</v>
       </c>
       <c r="H47" s="50">
-        <v>2500</v>
+        <v>3750</v>
       </c>
       <c r="I47" s="51">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="J47" s="50">
-        <v>7000</v>
+        <v>10500</v>
       </c>
       <c r="K47" s="51">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="L47" s="50">
-        <v>7000</v>
-      </c>
-      <c r="M47" s="49" t="s">
-        <v>1174</v>
+        <v>10500</v>
+      </c>
+      <c r="M47" s="49" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N47" s="49" t="s">
         <v>1195</v>
@@ -9255,22 +9288,24 @@
         <v>1075</v>
       </c>
       <c r="H49" s="39">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I49" s="40">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J49" s="39">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="K49" s="40">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L49" s="39">
-        <v>15</v>
-      </c>
-      <c r="M49" s="22" t="s">
-        <v>1179</v>
+        <v>18</v>
+      </c>
+      <c r="M49" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N49" s="22" t="s">
         <v>1202</v>
@@ -9543,22 +9578,24 @@
         <v>1219</v>
       </c>
       <c r="H55" s="39">
-        <v>373</v>
+        <v>541</v>
       </c>
       <c r="I55" s="40">
-        <v>690</v>
+        <v>1000</v>
       </c>
       <c r="J55" s="39">
-        <v>1455</v>
+        <v>2100</v>
       </c>
       <c r="K55" s="40">
-        <v>690</v>
+        <v>1000</v>
       </c>
       <c r="L55" s="39">
-        <v>1455</v>
-      </c>
-      <c r="M55" s="22" t="s">
-        <v>1179</v>
+        <v>2100</v>
+      </c>
+      <c r="M55" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N55" s="22"/>
       <c r="O55" s="24" t="s">
@@ -9917,27 +9954,24 @@
         <v>1075</v>
       </c>
       <c r="H64" s="57">
-        <f>H63*1.3</f>
-        <v>39</v>
+        <v>95</v>
       </c>
       <c r="I64" s="58">
-        <f>I63*1.3</f>
-        <v>78</v>
+        <v>190</v>
       </c>
       <c r="J64" s="57">
-        <f>J63*1.3</f>
-        <v>175.5</v>
+        <v>427</v>
       </c>
       <c r="K64" s="58">
-        <f>K63*1.3</f>
-        <v>78</v>
+        <v>190</v>
       </c>
       <c r="L64" s="57">
-        <f>L63*1.3</f>
-        <v>136.5</v>
-      </c>
-      <c r="M64" s="56" t="s">
-        <v>1247</v>
+        <v>332</v>
+      </c>
+      <c r="M64" s="56" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N64" s="56"/>
       <c r="O64" s="59" t="s">
@@ -10035,27 +10069,24 @@
         <v>1075</v>
       </c>
       <c r="H66" s="57">
-        <f>H63*0.9</f>
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="I66" s="58">
-        <f>I63*0.9</f>
-        <v>54</v>
+        <v>120</v>
       </c>
       <c r="J66" s="57">
-        <f>J63*0.9</f>
-        <v>121.5</v>
+        <v>270</v>
       </c>
       <c r="K66" s="58">
-        <f>K63*0.9</f>
-        <v>54</v>
+        <v>120</v>
       </c>
       <c r="L66" s="57">
-        <f>L63*0.9</f>
-        <v>94.5</v>
-      </c>
-      <c r="M66" s="56" t="s">
-        <v>1255</v>
+        <v>210</v>
+      </c>
+      <c r="M66" s="56" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N66" s="56"/>
       <c r="O66" s="59" t="s">
@@ -10251,23 +10282,23 @@
       </c>
       <c r="H70" s="57">
         <f>H64*0.45</f>
-        <v>17.55</v>
+        <v>42.75</v>
       </c>
       <c r="I70" s="58">
         <f>I64*0.45</f>
-        <v>35.1</v>
+        <v>85.5</v>
       </c>
       <c r="J70" s="57">
         <f>J64*0.45</f>
-        <v>78.975000000000009</v>
+        <v>192.15</v>
       </c>
       <c r="K70" s="58">
         <f>K64*0.45</f>
-        <v>35.1</v>
+        <v>85.5</v>
       </c>
       <c r="L70" s="57">
         <f>L64*0.45</f>
-        <v>61.425000000000004</v>
+        <v>149.4</v>
       </c>
       <c r="M70" s="56" t="s">
         <v>1271</v>
@@ -10301,23 +10332,23 @@
       </c>
       <c r="H71" s="57">
         <f>H64*0.3</f>
-        <v>11.7</v>
+        <v>28.5</v>
       </c>
       <c r="I71" s="58">
         <f>I64*0.3</f>
-        <v>23.4</v>
+        <v>57</v>
       </c>
       <c r="J71" s="57">
         <f>J64*0.3</f>
-        <v>52.65</v>
+        <v>128.1</v>
       </c>
       <c r="K71" s="58">
         <f>K64*0.3</f>
-        <v>23.4</v>
+        <v>57</v>
       </c>
       <c r="L71" s="57">
         <f>L64*0.3</f>
-        <v>40.949999999999996</v>
+        <v>99.6</v>
       </c>
       <c r="M71" s="56" t="s">
         <v>1275</v>
@@ -10451,23 +10482,23 @@
       </c>
       <c r="H74" s="57">
         <f t="shared" si="0"/>
-        <v>8.1</v>
+        <v>18.0</v>
       </c>
       <c r="I74" s="58">
         <f t="shared" si="0"/>
-        <v>16.2</v>
+        <v>36.0</v>
       </c>
       <c r="J74" s="57">
         <f t="shared" si="0"/>
-        <v>36.449999999999996</v>
+        <v>81.0</v>
       </c>
       <c r="K74" s="58">
         <f t="shared" si="0"/>
-        <v>16.2</v>
+        <v>36.0</v>
       </c>
       <c r="L74" s="57">
         <f t="shared" si="0"/>
-        <v>28.349999999999998</v>
+        <v>63.0</v>
       </c>
       <c r="M74" s="56" t="s">
         <v>1287</v>
@@ -10501,23 +10532,23 @@
       </c>
       <c r="H75" s="57">
         <f>H66*0.3</f>
-        <v>8.1</v>
+        <v>18</v>
       </c>
       <c r="I75" s="58">
         <f>I66*0.3</f>
-        <v>16.2</v>
+        <v>36</v>
       </c>
       <c r="J75" s="57">
         <f>J66*0.3</f>
-        <v>36.449999999999996</v>
+        <v>81</v>
       </c>
       <c r="K75" s="58">
         <f>K66*0.3</f>
-        <v>16.2</v>
+        <v>36</v>
       </c>
       <c r="L75" s="57">
         <f>L66*0.3</f>
-        <v>28.349999999999998</v>
+        <v>63</v>
       </c>
       <c r="M75" s="56" t="s">
         <v>1287</v>
@@ -10650,22 +10681,24 @@
         <v>1075</v>
       </c>
       <c r="H78" s="39">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="I78" s="40">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="J78" s="39">
-        <v>180</v>
+        <v>222</v>
       </c>
       <c r="K78" s="40">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="L78" s="39">
-        <v>90</v>
-      </c>
-      <c r="M78" s="22" t="s">
-        <v>1179</v>
+        <v>111</v>
+      </c>
+      <c r="M78" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N78" s="22" t="s">
         <v>1303</v>
@@ -10727,27 +10760,24 @@
         <v>1075</v>
       </c>
       <c r="H79" s="39">
-        <f>H78*0.3</f>
         <v>9</v>
       </c>
       <c r="I79" s="40">
-        <f>I78*0.3</f>
         <v>19.5</v>
       </c>
       <c r="J79" s="39">
-        <f>J78*0.3</f>
         <v>54</v>
       </c>
       <c r="K79" s="40">
-        <f>K78*0.3</f>
         <v>9</v>
       </c>
       <c r="L79" s="39">
-        <f>L78*0.3</f>
         <v>27</v>
       </c>
-      <c r="M79" s="22" t="s">
-        <v>1307</v>
+      <c r="M79" s="22" t="inlineStr">
+        <is>
+          <t>Tender – Lakeside S&amp;F (Sep 2026)</t>
+        </is>
       </c>
       <c r="N79" s="22"/>
       <c r="O79" s="24" t="s">
@@ -10795,22 +10825,24 @@
         <v>1075</v>
       </c>
       <c r="H80" s="39">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="I80" s="40">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="J80" s="39">
-        <v>90</v>
+        <v>150</v>
       </c>
       <c r="K80" s="40">
-        <v>40</v>
+        <v>67</v>
       </c>
       <c r="L80" s="39">
-        <v>70</v>
-      </c>
-      <c r="M80" s="22" t="s">
-        <v>1179</v>
+        <v>117</v>
+      </c>
+      <c r="M80" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N80" s="22" t="s">
         <v>1310</v>
@@ -10832,7 +10864,7 @@
         <v>122.75</v>
       </c>
       <c r="AA80" s="40">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="AB80" s="22" t="inlineStr">
         <is>
@@ -10863,20 +10895,22 @@
         <v>1075</v>
       </c>
       <c r="H81" s="39">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I81" s="40">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="J81" s="39">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="K81" s="40">
         <v>0</v>
       </c>
       <c r="L81" s="39"/>
-      <c r="M81" s="22" t="s">
-        <v>1637</v>
+      <c r="M81" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N81" s="22"/>
       <c r="O81" s="24" t="s">
@@ -10992,22 +11026,24 @@
         <v>1075</v>
       </c>
       <c r="H83" s="39">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I83" s="40">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="J83" s="39">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="K83" s="40">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="L83" s="39">
-        <v>22</v>
-      </c>
-      <c r="M83" s="22" t="s">
-        <v>1179</v>
+        <v>37</v>
+      </c>
+      <c r="M83" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N83" s="22" t="s">
         <v>1316</v>
@@ -11366,22 +11402,24 @@
         <v>1075</v>
       </c>
       <c r="H90" s="39">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="I90" s="40">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="J90" s="39">
-        <v>52</v>
+        <v>126</v>
       </c>
       <c r="K90" s="40">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="L90" s="39">
-        <v>52</v>
-      </c>
-      <c r="M90" s="22" t="s">
-        <v>1179</v>
+        <v>126</v>
+      </c>
+      <c r="M90" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N90" s="22" t="s">
         <v>1341</v>
@@ -11444,23 +11482,23 @@
       </c>
       <c r="H91" s="39">
         <f>H90*0.75</f>
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="I91" s="40">
         <f>I90*0.75</f>
-        <v>24.75</v>
+        <v>60</v>
       </c>
       <c r="J91" s="39">
         <f>J90*0.75</f>
-        <v>39</v>
+        <v>94.5</v>
       </c>
       <c r="K91" s="40">
         <f>K90*0.75</f>
-        <v>24.75</v>
+        <v>60</v>
       </c>
       <c r="L91" s="39">
         <f>L90*0.75</f>
-        <v>39</v>
+        <v>94.5</v>
       </c>
       <c r="M91" s="22" t="s">
         <v>1345</v>
@@ -11773,22 +11811,24 @@
         <v>1075</v>
       </c>
       <c r="H99" s="39">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="I99" s="40">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="J99" s="39">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="K99" s="40">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="L99" s="39">
-        <v>25</v>
-      </c>
-      <c r="M99" s="22" t="s">
-        <v>1179</v>
+        <v>49</v>
+      </c>
+      <c r="M99" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N99" s="22" t="s">
         <v>1371</v>
@@ -11934,22 +11974,24 @@
         <v>1075</v>
       </c>
       <c r="H102" s="39">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I102" s="40">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J102" s="39">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="K102" s="40">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="L102" s="39">
-        <v>30</v>
-      </c>
-      <c r="M102" s="22" t="s">
-        <v>1179</v>
+        <v>33</v>
+      </c>
+      <c r="M102" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N102" s="22" t="s">
         <v>1379</v>
@@ -12068,22 +12110,24 @@
         <v>1075</v>
       </c>
       <c r="H104" s="39">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I104" s="40">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="J104" s="39">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="K104" s="40">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="L104" s="39">
-        <v>20</v>
-      </c>
-      <c r="M104" s="22" t="s">
-        <v>1179</v>
+        <v>27</v>
+      </c>
+      <c r="M104" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N104" s="22" t="s">
         <v>1316</v>
@@ -12139,22 +12183,24 @@
         <v>1385</v>
       </c>
       <c r="H105" s="39">
-        <v>25000</v>
+        <v>37500</v>
       </c>
       <c r="I105" s="40">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="J105" s="39">
+        <v>90000</v>
+      </c>
+      <c r="K105" s="40">
         <v>60000</v>
       </c>
-      <c r="K105" s="40">
-        <v>40000</v>
-      </c>
       <c r="L105" s="39">
-        <v>60000</v>
-      </c>
-      <c r="M105" s="22" t="s">
-        <v>1179</v>
+        <v>90000</v>
+      </c>
+      <c r="M105" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N105" s="22" t="s">
         <v>1386</v>
@@ -12173,7 +12219,7 @@
         <v>112847.0</v>
       </c>
       <c r="AA105" s="40">
-        <v>100000</v>
+        <v>60000</v>
       </c>
       <c r="AB105" s="22" t="inlineStr">
         <is>
@@ -12891,22 +12937,24 @@
         <v>1075</v>
       </c>
       <c r="H123" s="39">
+        <v>5</v>
+      </c>
+      <c r="I123" s="40">
+        <v>12</v>
+      </c>
+      <c r="J123" s="39">
+        <v>20</v>
+      </c>
+      <c r="K123" s="40">
         <v>8</v>
       </c>
-      <c r="I123" s="40">
-        <v>18</v>
-      </c>
-      <c r="J123" s="39">
-        <v>30</v>
-      </c>
-      <c r="K123" s="40">
-        <v>12</v>
-      </c>
       <c r="L123" s="39">
-        <v>24</v>
-      </c>
-      <c r="M123" s="22" t="s">
-        <v>1179</v>
+        <v>16</v>
+      </c>
+      <c r="M123" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N123" s="22" t="s">
         <v>1433</v>
@@ -13417,22 +13465,24 @@
         <v>1075</v>
       </c>
       <c r="H134" s="39">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I134" s="40">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J134" s="39">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="K134" s="40">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="L134" s="39">
-        <v>15</v>
-      </c>
-      <c r="M134" s="22" t="s">
-        <v>1179</v>
+        <v>25</v>
+      </c>
+      <c r="M134" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N134" s="22" t="s">
         <v>1462</v>
@@ -13448,7 +13498,7 @@
         <v>35.4</v>
       </c>
       <c r="AA134" s="40">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AB134" s="22" t="inlineStr">
         <is>
@@ -13477,22 +13527,24 @@
         <v>1075</v>
       </c>
       <c r="H135" s="39">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="I135" s="40">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="J135" s="39">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="K135" s="40">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="L135" s="39">
-        <v>20</v>
-      </c>
-      <c r="M135" s="22" t="s">
-        <v>1179</v>
+        <v>50</v>
+      </c>
+      <c r="M135" s="22" t="inlineStr">
+        <is>
+          <t>Your figure</t>
+        </is>
       </c>
       <c r="N135" s="22" t="s">
         <v>1465</v>
@@ -14320,7 +14372,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>507</v>
+        <v>298</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>

</xml_diff>

<commit_message>
Scope dependencies for all projects (workbook v5.13) and flagged scope gaps
SUGGEST rules: kitchens/bathrooms -> ventilation (+ internal doors); strip-out -> fire stopping, emergency lighting, asbestos removal; full power installation -> fire stopping, emergency lighting. Unticked dependencies and items normal at the level of works are flagged in the cost assumptions. A 'No' attribute is no longer printed in line descriptions.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4236" uniqueCount="1791">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1797">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5404,6 +5404,24 @@
   </si>
   <si>
     <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.12 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUGGEST: S-0020 Fire stopping · SUGGEST: S-0047 Emergency lighting · SUGGEST: S-0001 Asbestos removal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUGGEST: S-0041 Ventilation · SUGGEST: S-0019 Internal doors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUGGEST: S-0041 Ventilation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUGGEST: S-0020 Fire stopping · SUGGEST: S-0047 Emergency lighting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.13 (October 2026)</t>
   </si>
 </sst>
 </file>
@@ -6035,7 +6053,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -14372,7 +14390,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>298</v>
+        <v>365</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -14383,7 +14401,7 @@
         <v>751</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>1789</v>
+        <v>1795</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -21229,7 +21247,9 @@
       <c r="J93" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="K93" s="15"/>
+      <c r="K93" s="15" t="s">
+        <v>1791</v>
+      </c>
       <c r="L93" s="15" t="s">
         <v>1701</v>
       </c>
@@ -22319,7 +22339,9 @@
       <c r="J123" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="K123" s="15"/>
+      <c r="K123" s="15" t="s">
+        <v>1792</v>
+      </c>
       <c r="L123" s="15" t="s">
         <v>1702</v>
       </c>
@@ -22353,7 +22375,9 @@
       <c r="J124" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="K124" s="15"/>
+      <c r="K124" s="15" t="s">
+        <v>1792</v>
+      </c>
       <c r="L124" s="15" t="s">
         <v>265</v>
       </c>
@@ -22425,7 +22449,9 @@
       <c r="J126" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="K126" s="15"/>
+      <c r="K126" s="15" t="s">
+        <v>1792</v>
+      </c>
       <c r="L126" s="15" t="s">
         <v>1703</v>
       </c>
@@ -22461,7 +22487,9 @@
       <c r="J127" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="K127" s="15"/>
+      <c r="K127" s="15" t="s">
+        <v>1793</v>
+      </c>
       <c r="L127" s="15" t="s">
         <v>280</v>
       </c>
@@ -23853,7 +23881,9 @@
       <c r="J166" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="K166" s="15"/>
+      <c r="K166" s="15" t="s">
+        <v>1794</v>
+      </c>
       <c r="L166" s="15" t="s">
         <v>452</v>
       </c>
@@ -23889,7 +23919,9 @@
       <c r="J167" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="K167" s="15"/>
+      <c r="K167" s="15" t="s">
+        <v>1794</v>
+      </c>
       <c r="L167" s="15" t="s">
         <v>1704</v>
       </c>

</xml_diff>

<commit_message>
Prelims 7-11% by complexity and programme, higher in London (workbook v5.14)
Base 7% (relaxed, vacant, no restrictions); occupation, restricted hours, shared access, long programme, 4+ M&E items, heritage, hard deadline and speed-first add up to a cap of 11%. Outer London +2 and Inner London +3 with a cap of 14%. The cap is the highest cap among the rules that fire.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1797">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1799">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5422,6 +5422,12 @@
   </si>
   <si>
     <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.13 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.14 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-06</t>
   </si>
 </sst>
 </file>
@@ -6053,7 +6059,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1796</v>
+        <v>1797</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -14339,7 +14345,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G197"/>
+  <dimension ref="A1:G203"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14390,7 +14396,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>365</v>
+        <v>437</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -14401,7 +14407,7 @@
         <v>751</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>1795</v>
+        <v>1798</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -16170,14 +16176,16 @@
       <c r="C131" s="2" t="s">
         <v>944</v>
       </c>
-      <c r="D131" s="2" t="s">
-        <v>945</v>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>Base 7% — vacant, no restrictions, relaxed programme</t>
+        </is>
       </c>
       <c r="E131" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F131" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
@@ -16197,7 +16205,7 @@
         <v>2</v>
       </c>
       <c r="F132" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.25">
@@ -16237,7 +16245,7 @@
         <v>0.5</v>
       </c>
       <c r="F134" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.25">
@@ -16257,7 +16265,7 @@
         <v>0.5</v>
       </c>
       <c r="F135" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.25">
@@ -16277,172 +16285,196 @@
         <v>0.5</v>
       </c>
       <c r="F136" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>952</v>
+        <v>942</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>953</v>
+        <v>943</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>954</v>
-      </c>
-      <c r="D137" s="2" t="s">
-        <v>955</v>
+        <v>946</v>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>Q2.3 has ≥4 M&amp;E items (complex services)</t>
+        </is>
       </c>
       <c r="E137" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F137" s="2">
         <v>11</v>
       </c>
-      <c r="F137" s="2"/>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>952</v>
+        <v>942</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>953</v>
+        <v>943</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>954</v>
-      </c>
-      <c r="D138" s="2" t="s">
-        <v>956</v>
+        <v>946</v>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>Q1.4 = Pre-1900 OR Q3.4 includes Listed Building Consent (heritage complexity)</t>
+        </is>
       </c>
       <c r="E138" s="2">
-        <v>9.5</v>
-      </c>
-      <c r="F138" s="2"/>
+        <v>0.5</v>
+      </c>
+      <c r="F138" s="2">
+        <v>11</v>
+      </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>952</v>
+        <v>942</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>953</v>
+        <v>943</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>954</v>
-      </c>
-      <c r="D139" s="2" t="s">
-        <v>957</v>
+        <v>946</v>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>Q4.1 = Hard deadline (condensed programme)</t>
+        </is>
       </c>
       <c r="E139" s="2">
-        <v>8.5</v>
-      </c>
-      <c r="F139" s="2"/>
+        <v>1.5</v>
+      </c>
+      <c r="F139" s="2">
+        <v>11</v>
+      </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>958</v>
+        <v>942</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>959</v>
+        <v>943</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>944</v>
-      </c>
-      <c r="D140" s="2" t="s">
-        <v>960</v>
+        <v>946</v>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Q4.4 top priority = Speed (condensed programme)</t>
+        </is>
       </c>
       <c r="E140" s="2">
-        <v>13.5</v>
-      </c>
-      <c r="F140" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="F140" s="2">
+        <v>11</v>
+      </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>958</v>
+        <v>942</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>959</v>
+        <v>943</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>944</v>
-      </c>
-      <c r="D141" s="2" t="s">
-        <v>961</v>
+        <v>946</v>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Region = Outer London</t>
+        </is>
       </c>
       <c r="E141" s="2">
-        <v>11.5</v>
-      </c>
-      <c r="F141" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="F141" s="2">
+        <v>14</v>
+      </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>958</v>
+        <v>942</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>959</v>
+        <v>943</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>944</v>
-      </c>
-      <c r="D142" s="2" t="s">
-        <v>962</v>
+        <v>946</v>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>Region = Inner London</t>
+        </is>
       </c>
       <c r="E142" s="2">
-        <v>8.5</v>
-      </c>
-      <c r="F142" s="2"/>
+        <v>3</v>
+      </c>
+      <c r="F142" s="2">
+        <v>14</v>
+      </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>959</v>
+        <v>953</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>944</v>
+        <v>954</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>963</v>
+        <v>955</v>
       </c>
       <c r="E143" s="2">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F143" s="2"/>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>959</v>
+        <v>953</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>946</v>
+        <v>954</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>1046</v>
+        <v>956</v>
       </c>
       <c r="E144" s="2">
-        <v>1.5</v>
+        <v>9.5</v>
       </c>
       <c r="F144" s="2"/>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>958</v>
+        <v>952</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>959</v>
+        <v>953</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>946</v>
+        <v>954</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>964</v>
+        <v>957</v>
       </c>
       <c r="E145" s="2">
-        <v>1</v>
+        <v>8.5</v>
       </c>
       <c r="F145" s="2"/>
     </row>
-    <row r="146" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>958</v>
       </c>
@@ -16450,121 +16482,121 @@
         <v>959</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="E146" s="2">
-        <v>2</v>
+        <v>13.5</v>
       </c>
       <c r="F146" s="2"/>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>966</v>
+        <v>958</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>967</v>
+        <v>959</v>
       </c>
       <c r="C147" s="2" t="s">
         <v>944</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>968</v>
+        <v>961</v>
       </c>
       <c r="E147" s="2">
-        <v>3.5</v>
+        <v>11.5</v>
       </c>
       <c r="F147" s="2"/>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>966</v>
+        <v>958</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>967</v>
+        <v>959</v>
       </c>
       <c r="C148" s="2" t="s">
         <v>944</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>969</v>
+        <v>962</v>
       </c>
       <c r="E148" s="2">
-        <v>4</v>
+        <v>8.5</v>
       </c>
       <c r="F148" s="2"/>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>966</v>
+        <v>958</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>967</v>
+        <v>959</v>
       </c>
       <c r="C149" s="2" t="s">
         <v>944</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>970</v>
+        <v>963</v>
       </c>
       <c r="E149" s="2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F149" s="2"/>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>966</v>
+        <v>958</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>967</v>
+        <v>959</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>944</v>
+        <v>946</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>971</v>
+        <v>1046</v>
       </c>
       <c r="E150" s="2">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="F150" s="2"/>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>966</v>
+        <v>958</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>967</v>
+        <v>959</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>944</v>
+        <v>946</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>972</v>
+        <v>964</v>
       </c>
       <c r="E151" s="2">
+        <v>1</v>
+      </c>
+      <c r="F151" s="2"/>
+    </row>
+    <row r="152" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A152" s="2" t="s">
+        <v>958</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>959</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>946</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>965</v>
+      </c>
+      <c r="E152" s="2">
         <v>2</v>
-      </c>
-      <c r="F151" s="2"/>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A152" s="2" t="s">
-        <v>966</v>
-      </c>
-      <c r="B152" s="2" t="s">
-        <v>967</v>
-      </c>
-      <c r="C152" s="2" t="s">
-        <v>944</v>
-      </c>
-      <c r="D152" s="2" t="s">
-        <v>973</v>
-      </c>
-      <c r="E152" s="2">
-        <v>3</v>
       </c>
       <c r="F152" s="2"/>
     </row>
@@ -16576,17 +16608,17 @@
         <v>967</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>974</v>
+        <v>968</v>
       </c>
       <c r="E153" s="2">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="F153" s="2"/>
     </row>
-    <row r="154" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>966</v>
       </c>
@@ -16597,7 +16629,7 @@
         <v>944</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>975</v>
+        <v>969</v>
       </c>
       <c r="E154" s="2">
         <v>4</v>
@@ -16606,123 +16638,111 @@
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>976</v>
+        <v>966</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>977</v>
+        <v>967</v>
       </c>
       <c r="C155" s="2" t="s">
         <v>944</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>978</v>
+        <v>970</v>
       </c>
       <c r="E155" s="2">
-        <v>5</v>
-      </c>
-      <c r="F155" s="2">
-        <v>10</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="F155" s="2"/>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>976</v>
+        <v>966</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>977</v>
+        <v>967</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>979</v>
+        <v>971</v>
       </c>
       <c r="E156" s="2">
-        <v>2</v>
-      </c>
-      <c r="F156" s="2">
-        <v>10</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="F156" s="2"/>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>976</v>
+        <v>966</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>977</v>
+        <v>967</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>980</v>
+        <v>972</v>
       </c>
       <c r="E157" s="2">
         <v>2</v>
       </c>
-      <c r="F157" s="2">
-        <v>10</v>
-      </c>
+      <c r="F157" s="2"/>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>976</v>
+        <v>966</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>977</v>
+        <v>967</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>981</v>
+        <v>973</v>
       </c>
       <c r="E158" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="F158" s="2">
-        <v>10</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="F158" s="2"/>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>976</v>
+        <v>966</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>977</v>
+        <v>967</v>
       </c>
       <c r="C159" s="2" t="s">
         <v>946</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>982</v>
+        <v>974</v>
       </c>
       <c r="E159" s="2">
-        <v>1.5</v>
-      </c>
-      <c r="F159" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+        <v>0.5</v>
+      </c>
+      <c r="F159" s="2"/>
+    </row>
+    <row r="160" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>976</v>
+        <v>966</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>977</v>
+        <v>967</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>983</v>
+        <v>975</v>
       </c>
       <c r="E160" s="2">
-        <v>1</v>
-      </c>
-      <c r="F160" s="2">
-        <v>10</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="F160" s="2"/>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
@@ -16732,13 +16752,13 @@
         <v>977</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>984</v>
+        <v>978</v>
       </c>
       <c r="E161" s="2">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="F161" s="2">
         <v>10</v>
@@ -16755,10 +16775,10 @@
         <v>946</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>985</v>
+        <v>979</v>
       </c>
       <c r="E162" s="2">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="F162" s="2">
         <v>10</v>
@@ -16775,10 +16795,10 @@
         <v>946</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>986</v>
+        <v>980</v>
       </c>
       <c r="E163" s="2">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="F163" s="2">
         <v>10</v>
@@ -16795,10 +16815,10 @@
         <v>946</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>987</v>
+        <v>981</v>
       </c>
       <c r="E164" s="2">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F164" s="2">
         <v>10</v>
@@ -16815,10 +16835,10 @@
         <v>946</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>988</v>
+        <v>982</v>
       </c>
       <c r="E165" s="2">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F165" s="2">
         <v>10</v>
@@ -16835,153 +16855,153 @@
         <v>946</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>947</v>
+        <v>983</v>
       </c>
       <c r="E166" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F166" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="167" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>989</v>
+        <v>976</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>990</v>
+        <v>977</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>991</v>
+        <v>946</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>992</v>
+        <v>984</v>
       </c>
       <c r="E167" s="2">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="F167" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>993</v>
+        <v>976</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>994</v>
+        <v>977</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>995</v>
+        <v>946</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>996</v>
+        <v>985</v>
       </c>
       <c r="E168" s="2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F168" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>993</v>
+        <v>976</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>994</v>
+        <v>977</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>995</v>
+        <v>946</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>997</v>
+        <v>986</v>
       </c>
       <c r="E169" s="2">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="F169" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>993</v>
+        <v>976</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>994</v>
+        <v>977</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>995</v>
+        <v>946</v>
       </c>
       <c r="D170" s="2" t="s">
-        <v>998</v>
+        <v>987</v>
       </c>
       <c r="E170" s="2">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="F170" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>993</v>
+        <v>976</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>994</v>
+        <v>977</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>995</v>
+        <v>946</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>999</v>
+        <v>988</v>
       </c>
       <c r="E171" s="2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F171" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>993</v>
+        <v>976</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>1000</v>
+        <v>977</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>995</v>
+        <v>946</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>1001</v>
+        <v>947</v>
       </c>
       <c r="E172" s="2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F172" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>993</v>
+        <v>989</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>1000</v>
+        <v>990</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>995</v>
+        <v>991</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>1002</v>
+        <v>992</v>
       </c>
       <c r="E173" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F173" s="2">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.25">
@@ -16989,16 +17009,16 @@
         <v>993</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>1000</v>
+        <v>994</v>
       </c>
       <c r="C174" s="2" t="s">
         <v>995</v>
       </c>
       <c r="D174" s="2" t="s">
-        <v>1003</v>
+        <v>996</v>
       </c>
       <c r="E174" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F174" s="2">
         <v>12</v>
@@ -17009,16 +17029,16 @@
         <v>993</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>1000</v>
+        <v>994</v>
       </c>
       <c r="C175" s="2" t="s">
         <v>995</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>1004</v>
+        <v>997</v>
       </c>
       <c r="E175" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F175" s="2">
         <v>12</v>
@@ -17029,185 +17049,203 @@
         <v>993</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>1000</v>
+        <v>994</v>
       </c>
       <c r="C176" s="2" t="s">
         <v>995</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>1005</v>
+        <v>998</v>
       </c>
       <c r="E176" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F176" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="177" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
+        <v>993</v>
+      </c>
+      <c r="B177" s="2" t="s">
+        <v>994</v>
+      </c>
+      <c r="C177" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>999</v>
+      </c>
+      <c r="E177" s="2">
+        <v>6</v>
+      </c>
+      <c r="F177" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A178" s="2" t="s">
+        <v>993</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>1001</v>
+      </c>
+      <c r="E178" s="2">
+        <v>1</v>
+      </c>
+      <c r="F178" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A179" s="2" t="s">
+        <v>993</v>
+      </c>
+      <c r="B179" s="2" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="D179" s="2" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E179" s="2">
+        <v>2</v>
+      </c>
+      <c r="F179" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A180" s="2" t="s">
+        <v>993</v>
+      </c>
+      <c r="B180" s="2" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="D180" s="2" t="s">
+        <v>1003</v>
+      </c>
+      <c r="E180" s="2">
+        <v>3</v>
+      </c>
+      <c r="F180" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A181" s="2" t="s">
+        <v>993</v>
+      </c>
+      <c r="B181" s="2" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="D181" s="2" t="s">
+        <v>1004</v>
+      </c>
+      <c r="E181" s="2">
+        <v>4</v>
+      </c>
+      <c r="F181" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A182" s="2" t="s">
+        <v>993</v>
+      </c>
+      <c r="B182" s="2" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="D182" s="2" t="s">
+        <v>1005</v>
+      </c>
+      <c r="E182" s="2">
+        <v>5</v>
+      </c>
+      <c r="F182" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A183" s="2" t="s">
         <v>1006</v>
       </c>
-      <c r="B177" s="2" t="s">
+      <c r="B183" s="2" t="s">
         <v>1007</v>
       </c>
-      <c r="C177" s="2" t="s">
+      <c r="C183" s="2" t="s">
         <v>991</v>
       </c>
-      <c r="D177" s="2" t="s">
+      <c r="D183" s="2" t="s">
         <v>1008</v>
       </c>
-      <c r="E177" s="2">
+      <c r="E183" s="2">
         <v>20</v>
       </c>
-      <c r="F177" s="2">
+      <c r="F183" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A179" s="3" t="s">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A185" s="3" t="s">
         <v>1009</v>
       </c>
-      <c r="B179" s="3" t="s">
+      <c r="B185" s="3" t="s">
         <v>1010</v>
       </c>
-      <c r="C179" s="4"/>
-      <c r="D179" s="4"/>
-      <c r="E179" s="4"/>
-      <c r="F179" s="4"/>
-      <c r="G179" s="4"/>
-    </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A180" s="6" t="s">
+      <c r="C185" s="4"/>
+      <c r="D185" s="4"/>
+      <c r="E185" s="4"/>
+      <c r="F185" s="4"/>
+      <c r="G185" s="4"/>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A186" s="6" t="s">
         <v>1011</v>
       </c>
-      <c r="B180" s="6" t="s">
+      <c r="B186" s="6" t="s">
         <v>1012</v>
       </c>
-      <c r="C180" s="6" t="s">
+      <c r="C186" s="6" t="s">
         <v>1013</v>
       </c>
-      <c r="D180" s="6" t="s">
+      <c r="D186" s="6" t="s">
         <v>1014</v>
       </c>
-      <c r="E180" s="6" t="s">
+      <c r="E186" s="6" t="s">
         <v>751</v>
-      </c>
-    </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A181" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="B181" s="2" t="s">
-        <v>1015</v>
-      </c>
-      <c r="C181" s="2" t="s">
-        <v>1016</v>
-      </c>
-      <c r="D181" s="2" t="s">
-        <v>1017</v>
-      </c>
-      <c r="E181" s="2" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A182" s="2" t="s">
-        <v>1018</v>
-      </c>
-      <c r="B182" s="2" t="s">
-        <v>1019</v>
-      </c>
-      <c r="C182" s="2" t="s">
-        <v>1016</v>
-      </c>
-      <c r="D182" s="2" t="s">
-        <v>1020</v>
-      </c>
-      <c r="E182" s="2" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A183" s="2" t="s">
-        <v>1021</v>
-      </c>
-      <c r="B183" s="2" t="s">
-        <v>1022</v>
-      </c>
-      <c r="C183" s="2" t="s">
-        <v>1016</v>
-      </c>
-      <c r="D183" s="2" t="s">
-        <v>1023</v>
-      </c>
-      <c r="E183" s="2" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A184" s="2" t="s">
-        <v>1024</v>
-      </c>
-      <c r="B184" s="2" t="s">
-        <v>1025</v>
-      </c>
-      <c r="C184" s="2" t="s">
-        <v>1016</v>
-      </c>
-      <c r="D184" s="2" t="s">
-        <v>1026</v>
-      </c>
-      <c r="E184" s="2" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A185" s="2" t="s">
-        <v>1027</v>
-      </c>
-      <c r="B185" s="2" t="s">
-        <v>1028</v>
-      </c>
-      <c r="C185" s="2" t="s">
-        <v>1016</v>
-      </c>
-      <c r="D185" s="2" t="s">
-        <v>1029</v>
-      </c>
-      <c r="E185" s="2" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A186" s="2" t="s">
-        <v>1030</v>
-      </c>
-      <c r="B186" s="2" t="s">
-        <v>1031</v>
-      </c>
-      <c r="C186" s="2" t="s">
-        <v>1016</v>
-      </c>
-      <c r="D186" s="2" t="s">
-        <v>1032</v>
-      </c>
-      <c r="E186" s="2" t="s">
-        <v>752</v>
       </c>
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>1033</v>
+        <v>291</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>1034</v>
+        <v>1015</v>
       </c>
       <c r="C187" s="2" t="s">
         <v>1016</v>
       </c>
       <c r="D187" s="2" t="s">
-        <v>1035</v>
+        <v>1017</v>
       </c>
       <c r="E187" s="2" t="s">
         <v>752</v>
@@ -17215,126 +17253,228 @@
     </row>
     <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>1036</v>
+        <v>1018</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>1037</v>
+        <v>1019</v>
       </c>
       <c r="C188" s="2" t="s">
         <v>1016</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>1038</v>
+        <v>1020</v>
       </c>
       <c r="E188" s="2" t="s">
         <v>752</v>
       </c>
     </row>
-    <row r="189" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>1039</v>
+        <v>1021</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>1040</v>
+        <v>1022</v>
       </c>
       <c r="C189" s="2" t="s">
         <v>1016</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>1041</v>
+        <v>1023</v>
       </c>
       <c r="E189" s="2" t="s">
         <v>752</v>
       </c>
     </row>
-    <row r="190" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A190" s="30" t="s">
-        <v>735</v>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A190" s="2" t="s">
+        <v>1024</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>734</v>
+        <v>1025</v>
       </c>
       <c r="C190" s="2" t="s">
         <v>1016</v>
       </c>
       <c r="D190" s="2" t="s">
+        <v>1026</v>
+      </c>
+      <c r="E190" s="2" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A191" s="2" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B191" s="2" t="s">
+        <v>1028</v>
+      </c>
+      <c r="C191" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D191" s="2" t="s">
+        <v>1029</v>
+      </c>
+      <c r="E191" s="2" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A192" s="2" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B192" s="2" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C192" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D192" s="2" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E192" s="2" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A193" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B193" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C193" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D193" s="2" t="s">
+        <v>1035</v>
+      </c>
+      <c r="E193" s="2" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A194" s="2" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C194" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D194" s="2" t="s">
+        <v>1038</v>
+      </c>
+      <c r="E194" s="2" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A195" s="2" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B195" s="2" t="s">
+        <v>1040</v>
+      </c>
+      <c r="C195" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D195" s="2" t="s">
+        <v>1041</v>
+      </c>
+      <c r="E195" s="2" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A196" s="30" t="s">
+        <v>735</v>
+      </c>
+      <c r="B196" s="2" t="s">
+        <v>734</v>
+      </c>
+      <c r="C196" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D196" s="2" t="s">
         <v>1630</v>
       </c>
-      <c r="E190" s="30" t="s">
+      <c r="E196" s="30" t="s">
         <v>1629</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A192" s="3" t="s">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A198" s="3" t="s">
         <v>1047</v>
       </c>
-      <c r="B192" s="3" t="s">
+      <c r="B198" s="3" t="s">
         <v>1048</v>
       </c>
-      <c r="C192" s="4"/>
-      <c r="D192" s="4"/>
-      <c r="E192" s="4"/>
-      <c r="F192" s="4"/>
-      <c r="G192" s="4"/>
-    </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A193" s="6" t="s">
+      <c r="C198" s="4"/>
+      <c r="D198" s="4"/>
+      <c r="E198" s="4"/>
+      <c r="F198" s="4"/>
+      <c r="G198" s="4"/>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A199" s="6" t="s">
         <v>1049</v>
       </c>
-      <c r="B193" s="6" t="s">
+      <c r="B199" s="6" t="s">
         <v>819</v>
       </c>
-      <c r="C193" s="6" t="s">
+      <c r="C199" s="6" t="s">
         <v>801</v>
       </c>
-      <c r="D193" s="6" t="s">
+      <c r="D199" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="194" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A194" s="2" t="s">
+    <row r="200" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A200" s="2" t="s">
         <v>942</v>
       </c>
-      <c r="B194" s="2">
+      <c r="B200" s="2">
         <v>0.9</v>
       </c>
-      <c r="C194" s="2">
+      <c r="C200" s="2">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D194" s="2" t="s">
+      <c r="D200" s="2" t="s">
         <v>1050</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A195" s="2" t="s">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A201" s="2" t="s">
         <v>952</v>
       </c>
-      <c r="B195" s="2">
+      <c r="B201" s="2">
         <v>0.85</v>
       </c>
-      <c r="C195" s="2">
+      <c r="C201" s="2">
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A196" s="2" t="s">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A202" s="2" t="s">
         <v>958</v>
       </c>
-      <c r="B196" s="2">
+      <c r="B202" s="2">
         <v>0.8</v>
       </c>
-      <c r="C196" s="2">
+      <c r="C202" s="2">
         <v>1.25</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A197" s="2" t="s">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A203" s="2" t="s">
         <v>966</v>
       </c>
-      <c r="B197" s="2">
+      <c r="B203" s="2">
         <v>0.75</v>
       </c>
-      <c r="C197" s="2">
+      <c r="C203" s="2">
         <v>1.3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook: percentage_rules header states the on-cost order and prelims rules the app applies
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1799">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1800">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5428,6 +5428,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Additions A–H, applied in the NRM1 order the app uses: A Prelims = % × Works; B OH&amp;P = % × (Works + A); Construction = Works + A + B; C Fees and D Developer costs = % × Construction; Base = Construction + C + D; E Risk and H Contingency = % × Base; F Inflation = % × (Base + E + H). A Prelims: 7% base (relaxed, vacant, no restrictions) plus the ADD rows that apply, capped at 11% outside London; London rows add 2 (Outer) or 3 (Inner) points with a 14% cap. The cap used is the highest cap among the rows that apply. Every figure here is read by the app — change it here, not in the code.</t>
   </si>
 </sst>
 </file>
@@ -16138,7 +16141,7 @@
         <v>935</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>936</v>
+        <v>1799</v>
       </c>
       <c r="C129" s="4"/>
       <c r="D129" s="4"/>

</xml_diff>

<commit_message>
Confidence grade scored from the workbook (v5.15), ranges skewed upwards, factors printed
'3. Settings' gains a ▶ confidence table: points per factor (stage, surveys, existing building, age, occupancy, High risks, share of client quantities, sense-check and scope gaps), grade thresholds and caps (Stage 0-1 at B; existing building with neither a condition nor an R&D survey at C). ▶ range_widths now A -10/+15, B -10/+20, C -15/+25, D -20/+35. The cost assumptions print the grade's factors; the finished record keeps the confidence object. Sample report regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1800">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1802">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5431,6 +5431,12 @@
   </si>
   <si>
     <t xml:space="preserve">Additions A–H, applied in the NRM1 order the app uses: A Prelims = % × Works; B OH&amp;P = % × (Works + A); Construction = Works + A + B; C Fees and D Developer costs = % × Construction; Base = Construction + C + D; E Risk and H Contingency = % × Base; F Inflation = % × (Base + E + H). A Prelims: 7% base (relaxed, vacant, no restrictions) plus the ADD rows that apply, capped at 11% outside London; London rows add 2 (Outer) or 3 (Inner) points with a 14% cap. The cap used is the highest cap among the rows that apply. Every figure here is read by the app — change it here, not in the code.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.15 (October 2026)</t>
   </si>
 </sst>
 </file>
@@ -6062,7 +6068,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1797</v>
+        <v>1801</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -14348,7 +14354,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G203"/>
+  <dimension ref="A1:G228"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14399,7 +14405,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>437</v>
+        <v>563</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -14410,7 +14416,7 @@
         <v>751</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>1798</v>
+        <v>1800</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -17442,7 +17448,7 @@
         <v>0.9</v>
       </c>
       <c r="C200" s="2">
-        <v>1.1000000000000001</v>
+        <v>1.15</v>
       </c>
       <c r="D200" s="2" t="s">
         <v>1050</v>
@@ -17453,10 +17459,10 @@
         <v>952</v>
       </c>
       <c r="B201" s="2">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="C201" s="2">
-        <v>1.1499999999999999</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
@@ -17464,7 +17470,7 @@
         <v>958</v>
       </c>
       <c r="B202" s="2">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="C202" s="2">
         <v>1.25</v>
@@ -17475,11 +17481,441 @@
         <v>966</v>
       </c>
       <c r="B203" s="2">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="C203" s="2">
-        <v>1.3</v>
-      </c>
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>▶ confidence</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>Confidence grade: points per factor that applies, grade thresholds, and grade caps. The app adds up the points of every factor that applies, takes the grade from the GRADE rows, then applies the lowest cap of any factor that applies. Keys are read by the app — do not rename them.</t>
+        </is>
+      </c>
+      <c r="C205" s="4"/>
+      <c r="D205" s="4"/>
+      <c r="E205" s="4"/>
+      <c r="F205" s="4"/>
+      <c r="G205" s="4"/>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A206" s="6" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B206" s="6" t="inlineStr">
+        <is>
+          <t>Factor (as printed)</t>
+        </is>
+      </c>
+      <c r="C206" s="6" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="D206" s="6" t="inlineStr">
+        <is>
+          <t>Threshold</t>
+        </is>
+      </c>
+      <c r="E206" s="6" t="inlineStr">
+        <is>
+          <t>Caps grade at</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>GRADE_A</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>Grade A when the total points are at most</t>
+        </is>
+      </c>
+      <c r="C207" s="2">
+        <v>1</v>
+      </c>
+      <c r="D207" s="2"/>
+      <c r="E207" s="2"/>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>GRADE_B</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>Grade B when the total points are at most</t>
+        </is>
+      </c>
+      <c r="C208" s="2">
+        <v>3</v>
+      </c>
+      <c r="D208" s="2"/>
+      <c r="E208" s="2"/>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>GRADE_C</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>Grade C when the total points are at most (above this: D)</t>
+        </is>
+      </c>
+      <c r="C209" s="2">
+        <v>6</v>
+      </c>
+      <c r="D209" s="2"/>
+      <c r="E209" s="2"/>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>STAGE_0_1</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>design at Stage 0–1</t>
+        </is>
+      </c>
+      <c r="C210" s="2">
+        <v>1</v>
+      </c>
+      <c r="D210" s="2"/>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>NO_SURVEYS</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>no surveys in the last 5 years</t>
+        </is>
+      </c>
+      <c r="C211" s="2">
+        <v>2</v>
+      </c>
+      <c r="D211" s="2"/>
+      <c r="E211" s="2"/>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>NO_CONDITION_SURVEY</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>no condition survey</t>
+        </is>
+      </c>
+      <c r="C212" s="2">
+        <v>1</v>
+      </c>
+      <c r="D212" s="2"/>
+      <c r="E212" s="2"/>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>NO_RD_SURVEY</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>no asbestos R&amp;D survey (pre-2000 building)</t>
+        </is>
+      </c>
+      <c r="C213" s="2">
+        <v>1</v>
+      </c>
+      <c r="D213" s="2"/>
+      <c r="E213" s="2"/>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>NO_CONDITION_OR_RD</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>neither a condition nor an asbestos R&amp;D survey</t>
+        </is>
+      </c>
+      <c r="C214" s="2">
+        <v>0</v>
+      </c>
+      <c r="D214" s="2"/>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>CONDITION_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>building condition unknown</t>
+        </is>
+      </c>
+      <c r="C215" s="2">
+        <v>1</v>
+      </c>
+      <c r="D215" s="2"/>
+      <c r="E215" s="2"/>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>PLANNING_UNSURE</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>planning route not established</t>
+        </is>
+      </c>
+      <c r="C216" s="2">
+        <v>1</v>
+      </c>
+      <c r="D216" s="2"/>
+      <c r="E216" s="2"/>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>EXISTING_BUILDING</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>existing building</t>
+        </is>
+      </c>
+      <c r="C217" s="2">
+        <v>1</v>
+      </c>
+      <c r="D217" s="2"/>
+      <c r="E217" s="2"/>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>AGE_PRE_1980</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>built before 1980</t>
+        </is>
+      </c>
+      <c r="C218" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D218" s="2"/>
+      <c r="E218" s="2"/>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>OCCUPIED_FULL</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>fully occupied during works</t>
+        </is>
+      </c>
+      <c r="C219" s="2">
+        <v>1</v>
+      </c>
+      <c r="D219" s="2"/>
+      <c r="E219" s="2"/>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>OCCUPIED_PARTIAL</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>partly occupied during works</t>
+        </is>
+      </c>
+      <c r="C220" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D220" s="2"/>
+      <c r="E220" s="2"/>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>HIGH_RISKS</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>risks rated High (Threshold = how many)</t>
+        </is>
+      </c>
+      <c r="C221" s="2">
+        <v>1</v>
+      </c>
+      <c r="D221" s="2">
+        <v>2</v>
+      </c>
+      <c r="E221" s="2"/>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>CLIENT_SHARE_LOW</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>few client-confirmed quantities (Threshold = share of works cost below which it applies)</t>
+        </is>
+      </c>
+      <c r="C222" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D222" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="E222" s="2"/>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>SENSE_HIGH</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>high-severity sense-check warning</t>
+        </is>
+      </c>
+      <c r="C223" s="2">
+        <v>2</v>
+      </c>
+      <c r="D223" s="2"/>
+      <c r="E223" s="2"/>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>SENSE_MEDIUM</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>sense-check warnings</t>
+        </is>
+      </c>
+      <c r="C224" s="2">
+        <v>1</v>
+      </c>
+      <c r="D224" s="2"/>
+      <c r="E224" s="2"/>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>BENCHMARK_MISSING</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>no published cost benchmark to check against</t>
+        </is>
+      </c>
+      <c r="C225" s="2">
+        <v>1</v>
+      </c>
+      <c r="D225" s="2"/>
+      <c r="E225" s="2"/>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>EXCLUDED_ITEMS</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>scope items excluded pending quantities</t>
+        </is>
+      </c>
+      <c r="C226" s="2">
+        <v>1</v>
+      </c>
+      <c r="D226" s="2"/>
+      <c r="E226" s="2"/>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>RATIO_ESTIMATES</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>quantities estimated from typical ratios</t>
+        </is>
+      </c>
+      <c r="C227" s="2">
+        <v>1</v>
+      </c>
+      <c r="D227" s="2"/>
+      <c r="E227" s="2"/>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST_UNPRICED</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>specialist scope not priced</t>
+        </is>
+      </c>
+      <c r="C228" s="2">
+        <v>1</v>
+      </c>
+      <c r="D228" s="2"/>
+      <c r="E228" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Risk allowance in the four NRM1 categories (workbook v5.16), no double counting
'3. Settings' ▶ risk_allowance (owner-approved 8 Oct 2026), % of base cost: design development (by design stage, condition survey, ageing M&E, higher-risk building), construction (new/existing base, asbestos, structural, contamination, damp/fire/drainage, pre-1980), employer change (by stage), employer other (planning unsure, grant, heritage); cap 25%. Replaces E and the fixed 5% H. Items already priced in the scope reduce or remove their row; occupation, deadline and phasing stay in prelims and programme only. The cost table shows one row per category; the build-up line names what applied. Lakeside: 13% (was 10.5%). Sample regenerated; fit check passes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1802">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1805">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5437,6 +5437,15 @@
   </si>
   <si>
     <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.15 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.16 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Additions A–H, applied in the NRM1 order the app uses: A Prelims = % × Works; B OH&amp;P = % × (Works + A); Construction = Works + A + B; C Fees and D Developer costs = % × Construction; Base = Construction + C + D; E Risk and H Contingency = % × Base; F Inflation = % × (Base + E + H). A Prelims: 7% base (relaxed, vacant, no restrictions) plus the ADD rows that apply, capped at 11% outside London; London rows add 2 (Outer) or 3 (Inner) points with a 14% cap. The cap used is the highest cap among the rows that apply. Every figure here is read by the app — change it here, not in the code. Since v5.16 the E and H rows below are not used: risk is set by ▶ risk_allowance (four NRM1 categories, no separate contingency); they are kept only for older copies of the app.</t>
   </si>
 </sst>
 </file>
@@ -6068,7 +6077,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1801</v>
+        <v>1803</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -14354,7 +14363,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G228"/>
+  <dimension ref="A1:G258"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14405,7 +14414,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>563</v>
+        <v>523</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -14416,7 +14425,7 @@
         <v>751</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>1800</v>
+        <v>1802</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -16147,7 +16156,7 @@
         <v>935</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>1799</v>
+        <v>1804</v>
       </c>
       <c r="C129" s="4"/>
       <c r="D129" s="4"/>
@@ -17916,6 +17925,677 @@
       </c>
       <c r="D228" s="2"/>
       <c r="E228" s="2"/>
+    </row>
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>▶ risk_allowance</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>Risk allowance in the four NRM1 categories, % of base cost (construction + fees). The app adds the rows that apply in each category and caps the total; it replaces the E and H rows of ▶ percentage_rules. Nothing already priced in the scope, prelims, fees or programme is charged again (occupation, deadlines and phasing are in prelims and programme; inflation is F). Keys are read by the app — do not rename them.</t>
+        </is>
+      </c>
+      <c r="C230" s="4"/>
+      <c r="D230" s="4"/>
+      <c r="E230" s="4"/>
+      <c r="F230" s="4"/>
+      <c r="G230" s="4"/>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A231" s="6" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B231" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C231" s="6" t="inlineStr">
+        <is>
+          <t>Applies when (as printed)</t>
+        </is>
+      </c>
+      <c r="D231" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E231" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>DD_STAGE_0_1</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>Design development</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>design at Stage 0–1</t>
+        </is>
+      </c>
+      <c r="D232" s="2">
+        <v>5</v>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>Base: by design stage reached (Q4.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>DD_STAGE_2</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>Design development</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>design at Stage 2</t>
+        </is>
+      </c>
+      <c r="D233" s="2">
+        <v>3</v>
+      </c>
+      <c r="E233" s="2"/>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>DD_STAGE_3</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>Design development</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>design at Stage 3</t>
+        </is>
+      </c>
+      <c r="D234" s="2">
+        <v>2</v>
+      </c>
+      <c r="E234" s="2"/>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>DD_STAGE_4</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>Design development</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>design at Stage 4</t>
+        </is>
+      </c>
+      <c r="D235" s="2">
+        <v>1</v>
+      </c>
+      <c r="E235" s="2"/>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>DD_NO_CONDITION_SURVEY</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>Design development</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>no condition survey</t>
+        </is>
+      </c>
+      <c r="D236" s="2">
+        <v>1</v>
+      </c>
+      <c r="E236" s="2"/>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>DD_AGEING_ME</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>Design development</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>ageing M&amp;E</t>
+        </is>
+      </c>
+      <c r="D237" s="2">
+        <v>1</v>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>Not at full systems replacement</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>DD_AGEING_ME_REPLACED</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>Design development</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>ageing M&amp;E (being replaced)</t>
+        </is>
+      </c>
+      <c r="D238" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>At full systems replacement (the replacement is priced)</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>DD_HIGHER_RISK</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>Design development</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>higher-risk building</t>
+        </is>
+      </c>
+      <c r="D239" s="2">
+        <v>1</v>
+      </c>
+      <c r="E239" s="2"/>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>CR_NEW</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>new build</t>
+        </is>
+      </c>
+      <c r="D240" s="2">
+        <v>2</v>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>Base: new build, external works</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>CR_EXISTING</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>existing building</t>
+        </is>
+      </c>
+      <c r="D241" s="2">
+        <v>4</v>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>Base: refurbishment, fit-out, extension, demolition, mixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>CR_ASBESTOS</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>no asbestos R&amp;D survey, removal not priced</t>
+        </is>
+      </c>
+      <c r="D242" s="2">
+        <v>2</v>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>Pre-2000 building or asbestos known</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>CR_ASBESTOS_PRICED</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>no asbestos R&amp;D survey, removal priced</t>
+        </is>
+      </c>
+      <c r="D243" s="2">
+        <v>1</v>
+      </c>
+      <c r="E243" s="2"/>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>CR_STRUCTURAL</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>structural concerns</t>
+        </is>
+      </c>
+      <c r="D244" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>Not priced (no repairs or alterations item)</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>CR_STRUCTURAL_PRICED</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>structural concerns (repairs priced)</t>
+        </is>
+      </c>
+      <c r="D245" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="E245" s="2"/>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>CR_CONTAMINATED</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>contaminated land</t>
+        </is>
+      </c>
+      <c r="D246" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>Not priced</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>CR_CONTAMINATED_PRICED</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>contaminated land (remediation priced)</t>
+        </is>
+      </c>
+      <c r="D247" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E247" s="2"/>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>CR_DAMP</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>damp</t>
+        </is>
+      </c>
+      <c r="D248" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>0 when damp treatment is priced</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>CR_FIRE</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>fire safety issues</t>
+        </is>
+      </c>
+      <c r="D249" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>0 when fire stopping is priced</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>CR_DRAINAGE</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>drainage issues</t>
+        </is>
+      </c>
+      <c r="D250" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>0 when drainage is priced</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>CR_PRE_1980</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>pre-1980 building</t>
+        </is>
+      </c>
+      <c r="D251" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>Existing buildings only</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>EC_STAGE_0_1</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>Employer change</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>design at Stage 0–1</t>
+        </is>
+      </c>
+      <c r="D252" s="2">
+        <v>3</v>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>EC_LATER</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>Employer change</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>design past Stage 1</t>
+        </is>
+      </c>
+      <c r="D253" s="2">
+        <v>2</v>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>EO_BASE</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>Employer other</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D254" s="2">
+        <v>1</v>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>EO_PLANNING_UNSURE</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>Employer other</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>planning route unsure</t>
+        </is>
+      </c>
+      <c r="D255" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E255" s="2"/>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>EO_GRANT</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>Employer other</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>grant funding</t>
+        </is>
+      </c>
+      <c r="D256" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E256" s="2"/>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>EO_HERITAGE</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>Employer other</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>listed or conservation area</t>
+        </is>
+      </c>
+      <c r="D257" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E257" s="2"/>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>CAP</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>total risk allowance cap</t>
+        </is>
+      </c>
+      <c r="D258" s="2">
+        <v>25</v>
+      </c>
+      <c r="E258" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Inflation from the rate base date to mid-construction (workbook v5.17)
'3. Settings' ▶ inflation (owner-approved 8 Oct 2026): rates at Q3 2026 (15 Aug 2026), 3.5% a year compounded to the programme's construction mid-point, cap 12%. Replaces the banded F rows. The pipeline passes the construction mid-point from the programme's own dates; the report's build-up line states the base date, the mid-point and the months; cost.baseDate is now 'Q3 2026'. Sample regenerated; fit check passes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1805">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1806">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5446,6 +5446,9 @@
   </si>
   <si>
     <t xml:space="preserve">Additions A–H, applied in the NRM1 order the app uses: A Prelims = % × Works; B OH&amp;P = % × (Works + A); Construction = Works + A + B; C Fees and D Developer costs = % × Construction; Base = Construction + C + D; E Risk and H Contingency = % × Base; F Inflation = % × (Base + E + H). A Prelims: 7% base (relaxed, vacant, no restrictions) plus the ADD rows that apply, capped at 11% outside London; London rows add 2 (Outer) or 3 (Inner) points with a 14% cap. The cap used is the highest cap among the rows that apply. Every figure here is read by the app — change it here, not in the code. Since v5.16 the E and H rows below are not used: risk is set by ▶ risk_allowance (four NRM1 categories, no separate contingency); they are kept only for older copies of the app.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.17 (October 2026)</t>
   </si>
 </sst>
 </file>
@@ -6077,7 +6080,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1803</v>
+        <v>1805</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -14363,7 +14366,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G258"/>
+  <dimension ref="A1:G265"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14414,7 +14417,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>523</v>
+        <v>1395</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -18596,6 +18599,104 @@
         <v>25</v>
       </c>
       <c r="E258" s="2"/>
+    </row>
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A260" s="3" t="inlineStr">
+        <is>
+          <t>▶ inflation</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t>Inflation (F) from the rate base date to the mid-point of construction (the programme's own dates): % = (1 + annual rate) ^ years − 1, capped. Replaces the banded F rows of ▶ percentage_rules. Keys are read by the app — do not rename them.</t>
+        </is>
+      </c>
+      <c r="C260" s="4"/>
+      <c r="D260" s="4"/>
+      <c r="E260" s="4"/>
+      <c r="F260" s="4"/>
+      <c r="G260" s="4"/>
+    </row>
+    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A261" s="6" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B261" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C261" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>RATE_BASE_DATE</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>The date every rate on '2. Rates' is priced at (Q3 2026, taken as mid-quarter). Text, YYYY-MM-DD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>RATE_BASE_LABEL</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>How the base date is printed in the report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>ANNUAL_PCT</t>
+        </is>
+      </c>
+      <c r="B264" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>Construction price inflation, % a year (estimate from published tender price forecasts, 2026–28).</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>CAP_PCT</t>
+        </is>
+      </c>
+      <c r="B265" s="2">
+        <v>12</v>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>Maximum inflation allowance, %.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Professional fees by procurement route (workbook v5.18)
'3. Settings' ▶ route_fees (owner-approved 8 Oct 2026): design and build -3 points on client fees + contractor's design 2% of construction (Claycroft D&B 2.1%); two-stage -1.5 + 1%; traditional and construction management unchanged. Only while Stage 4 is still to do. The preferred route from the Procurement Reference drives it (final cost passes); contractor's design is its own row in the cost table and sits in the base cost; project totals now come from the on-cost chain. Across the 42 test scenarios: 30 traditional unchanged, D&B -0.8 to -0.9%, two-stage -0.4 to -0.5%. Cost page fit: trailing '(…)' notes no longer printed in the build-up. Sample regenerated; fit check passes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1806">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1807">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5449,6 +5449,9 @@
   </si>
   <si>
     <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.17 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.18 (October 2026)</t>
   </si>
 </sst>
 </file>
@@ -6080,7 +6083,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1805</v>
+        <v>1806</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -14366,7 +14369,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G265"/>
+  <dimension ref="A1:G272"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14417,7 +14420,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>1395</v>
+        <v>528</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -18120,7 +18123,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>ageing M&amp;E (being replaced)</t>
+          <t>ageing M&amp;E, being replaced</t>
         </is>
       </c>
       <c r="D238" s="2">
@@ -18695,6 +18698,117 @@
       <c r="C265" s="2" t="inlineStr">
         <is>
           <t>Maximum inflation allowance, %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A267" s="3" t="inlineStr">
+        <is>
+          <t>▶ route_fees</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>Professional fees by the preferred procurement route (from the Procurement Reference). The client-fee adjustment (points) is added to C; the contractor's design (% of construction) is its own row. Applies only while Stage 4 is not yet complete (Q4.5). Route names must match the Procurement Reference exactly.</t>
+        </is>
+      </c>
+      <c r="C267" s="4"/>
+      <c r="D267" s="4"/>
+      <c r="E267" s="4"/>
+      <c r="F267" s="4"/>
+      <c r="G267" s="4"/>
+    </row>
+    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A268" s="6" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B268" s="6" t="inlineStr">
+        <is>
+          <t>Client fee adjustment (points)</t>
+        </is>
+      </c>
+      <c r="C268" s="6" t="inlineStr">
+        <is>
+          <t>Contractor's design %</t>
+        </is>
+      </c>
+      <c r="D268" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>Traditional</t>
+        </is>
+      </c>
+      <c r="B269" s="2">
+        <v>0</v>
+      </c>
+      <c r="C269" s="2">
+        <v>0</v>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>The client's design team does every stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>Design and build (single stage)</t>
+        </is>
+      </c>
+      <c r="B270" s="2">
+        <v>-3</v>
+      </c>
+      <c r="C270" s="2">
+        <v>2</v>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>The contractor's team does Stage 4. Contractor's design 2% (Claycroft, Morgan Sindall D&amp;B: 2.1%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>Two-stage (PCSA)</t>
+        </is>
+      </c>
+      <c r="B271" s="2">
+        <v>-1.5</v>
+      </c>
+      <c r="C271" s="2">
+        <v>1</v>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>Stage 4 is shared with the contractor during the pre-construction stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>Construction management</t>
+        </is>
+      </c>
+      <c r="B272" s="2">
+        <v>0</v>
+      </c>
+      <c r="C272" s="2">
+        <v>0</v>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>Unchanged: the CM fee replaces part of the contractor's OH&amp;P (not modelled).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook update log v5.13-v5.18, every UK postcode district, consistency checks in the admin list
- '1. Instructions': six update-log lines (v5.13 to v5.18), newest first; nothing references the shifted rows.
- Postcode validation checks every UK district (lib/data/ukPostcodeDistricts.js, 2,932 districts in 125 areas, generated from Wikipedia's Royal Mail list); the old CV-only table also wrongly refused CV9.
- The admin report list shows each report's consistency findings (count, expandable messages); the award-vs-start-on-site check is removed because the owner chose no mobilisation stage.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -6072,7 +6072,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BBCD35-3C7D-4CAC-A46E-6C3CC3E31849}">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.7109375" style="8" customWidth="1"/>
@@ -6774,148 +6774,220 @@
     <row r="81" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="17" t="inlineStr">
         <is>
-          <t>v5.12 — 4 Oct 2026</t>
+          <t>v5.18 — 8 Oct 2026</t>
         </is>
       </c>
       <c r="B81" s="17" t="inlineStr">
         <is>
-          <t>Rates updated from the owner's review of the v5.11 suggestions (column AA marked green = accept, amber = owner's figure, red = no change). 25 rows changed; each row's Basic, Standard, High and New build Std / High move by the same ratio as Standard (new Std ÷ old Std), rounded. Std (Refurb &amp; Fit-out): demolition 130→100; roof 110→190; external walls 60→100; windows 120→140; internal walls 110→150; internal doors 60→100; floor finishes 75→85; ceilings 50→80; staff kitchenette 4,000→6,000; signage 10→12; catering kitchen 690→1,000; ASHP full system 78→190 and district heating full system 54→120 (now figures, not = 5.1a × factor; their plant-only / radiators-only rows still follow by formula); water and drainage 65→80; ventilation 45→75 (owner); extract fans 19→22; BMS 15→25; lighting 33→80 (5.8b follows at 75%); fire alarm 18→35; data 18→20; security 15→20; passenger lift 40,000→60,000 (owner); builder's work 18→12; foul drainage 6→10 (owner); external utilities 10→25. Kept: toilets and accessible WCs (owner: no change) and the 20 'keep' rows; 5.2b visible-fittings water fixed at its figures (19.5 Std, Lakeside tender) so it does not follow 5.2a. Changed rows' Source = 'Your figure'.</t>
+          <t>Professional fees by procurement route: new ▶ route_fees on '3. Settings'. Design and build: client fees −3 points and contractor's design 2% of construction (Claycroft D&amp;B 2.1%); two-stage (PCSA): −1.5 and 1%; traditional and construction management unchanged. Only while Stage 4 is still to do. The preferred route comes from the Procurement Reference.</t>
         </is>
       </c>
     </row>
     <row r="82" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="17" t="inlineStr">
         <is>
+          <t>v5.17 — 8 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B82" s="17" t="inlineStr">
+        <is>
+          <t>Inflation from the rate base date: new ▶ inflation on '3. Settings'. Rates are at Q3 2026 (15 Aug 2026); 3.5% a year compounded to the programme's construction mid-point, capped at 12%. Replaces the banded F rows of ▶ percentage_rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="17" t="inlineStr">
+        <is>
+          <t>v5.16 — 8 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B83" s="17" t="inlineStr">
+        <is>
+          <t>Risk allowance in the four NRM1 categories: new ▶ risk_allowance on '3. Settings' (design development by design stage, construction, employer change, employer other; cap 25%). Replaces E and the fixed 5% contingency H. Items already priced in the scope reduce or remove their risk row; occupation, deadline and phasing stay in prelims and programme only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>v5.15 — 7 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="17" t="inlineStr">
+        <is>
+          <t>Confidence grade scored from the workbook: new ▶ confidence on '3. Settings' (points per factor, grade thresholds, caps: Stage 0–1 at B; existing building with neither a condition nor an R&amp;D survey at C). ▶ range_widths skewed upwards: A −10/+15, B −10/+20, C −15/+25, D −20/+35.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>v5.14 — 6 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="17" t="inlineStr">
+        <is>
+          <t>Preliminaries: 7% base (relaxed, vacant, no restrictions) plus occupation, restricted hours, shared access, programme over 18 months, 4+ M&amp;E items, heritage, hard deadline and speed-first, capped at 11%; Outer London +2 and Inner London +3 with a 14% cap. The ▶ percentage_rules header states the on-cost order the app uses (OH&amp;P on works + prelims; risk on base cost; inflation on the cost limit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>v5.13 — 5 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="17" t="inlineStr">
+        <is>
+          <t>Scope dependencies ('When selected' SUGGEST on '4. Scope rules'): kitchens and bathrooms → ventilation (domestic also → internal doors); strip-out → fire stopping, emergency lighting, asbestos removal; full power installation → fire stopping, emergency lighting. The report flags any that are not ticked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t>v5.12 — 4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B87" s="17" t="inlineStr">
+        <is>
+          <t>Rates updated from the owner's review of the v5.11 suggestions (column AA marked green = accept, amber = owner's figure, red = no change). 25 rows changed; each row's Basic, Standard, High and New build Std / High move by the same ratio as Standard (new Std ÷ old Std), rounded. Std (Refurb &amp; Fit-out): demolition 130→100; roof 110→190; external walls 60→100; windows 120→140; internal walls 110→150; internal doors 60→100; floor finishes 75→85; ceilings 50→80; staff kitchenette 4,000→6,000; signage 10→12; catering kitchen 690→1,000; ASHP full system 78→190 and district heating full system 54→120 (now figures, not = 5.1a × factor; their plant-only / radiators-only rows still follow by formula); water and drainage 65→80; ventilation 45→75 (owner); extract fans 19→22; BMS 15→25; lighting 33→80 (5.8b follows at 75%); fire alarm 18→35; data 18→20; security 15→20; passenger lift 40,000→60,000 (owner); builder's work 18→12; foul drainage 6→10 (owner); external utilities 10→25. Kept: toilets and accessible WCs (owner: no change) and the 20 'keep' rows; 5.2b visible-fittings water fixed at its figures (19.5 Std, Lakeside tender) so it does not follow 5.2a. Changed rows' Source = 'Your figure'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="17" t="inlineStr">
+        <is>
           <t>v5.11 — 4 Oct 2026</t>
         </is>
       </c>
-      <c r="B82" s="17" t="inlineStr">
+      <c r="B88" s="17" t="inlineStr">
         <is>
           <t>Evidence only, no rates changed. Six more project columns on '2. Rates' beside Whitefields (R) and Claycroft (S), each a plain figure in the row's unit on this workbook's basis: T Lakeside S&amp;F (15 rows), U Computer Science (6), V Scarman Public Toilets Phase 2, high spec (12), W Co-op store fit-out (19), X IBRB café (7), Y Riley Court Psychology refurbishment (27, from the signed contract CSA). Column Z averages R–Y on 47 rows. Row 24 explains the columns and lists the evidence that has no row (scaffold, retail refrigeration and equipment, preliminaries %). Columns AA–AB: Claude's suggested Refurb &amp; Fit-out Std rate and the reason, on all 47 rows (25 raise, 2 lower, 20 keep).</t>
         </is>
       </c>
     </row>
-    <row r="83" spans="1:3" s="54" customFormat="1" ht="104.0" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="17" t="s">
+    <row r="89" spans="1:3" s="54" customFormat="1" ht="104.0" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="17" t="s">
         <v>1778</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B89" s="17" t="s">
         <v>1779</v>
       </c>
-      <c r="C83" s="60"/>
-    </row>
-    <row r="84" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="17" t="s">
+      <c r="C89" s="60"/>
+    </row>
+    <row r="90" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="17" t="s">
         <v>1748</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B90" s="17" t="s">
         <v>1783</v>
       </c>
-      <c r="C84" s="60"/>
-    </row>
-    <row r="85" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A85" s="17" t="s">
+      <c r="C90" s="60"/>
+    </row>
+    <row r="91" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A91" s="17" t="s">
         <v>1722</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B91" s="17" t="s">
         <v>1737</v>
       </c>
-      <c r="C85" s="60"/>
-    </row>
-    <row r="86" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A86" s="17" t="s">
+      <c r="C91" s="60"/>
+    </row>
+    <row r="92" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A92" s="17" t="s">
         <v>1711</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B92" s="17" t="s">
         <v>1712</v>
       </c>
-      <c r="C86" s="60"/>
-    </row>
-    <row r="87" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A87" s="17" t="s">
+      <c r="C92" s="60"/>
+    </row>
+    <row r="93" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A93" s="17" t="s">
         <v>1632</v>
       </c>
-      <c r="B87" s="17" t="s">
+      <c r="B93" s="17" t="s">
         <v>1634</v>
       </c>
-      <c r="C87" s="60"/>
-    </row>
-    <row r="88" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A88" s="15" t="s">
+      <c r="C93" s="60"/>
+    </row>
+    <row r="94" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A94" s="15" t="s">
         <v>1620</v>
       </c>
-      <c r="B88" s="17" t="s">
+      <c r="B94" s="17" t="s">
         <v>1621</v>
       </c>
-      <c r="C88" s="33"/>
-    </row>
-    <row r="89" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A89" s="15" t="s">
+      <c r="C94" s="33"/>
+    </row>
+    <row r="95" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A95" s="15" t="s">
         <v>1060</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="B95" s="17" t="s">
         <v>1061</v>
       </c>
-      <c r="C89" s="33"/>
-    </row>
-    <row r="90" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A90" s="15" t="s">
+      <c r="C95" s="33"/>
+    </row>
+    <row r="96" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A96" s="15" t="s">
         <v>1051</v>
       </c>
-      <c r="B90" s="17" t="s">
+      <c r="B96" s="17" t="s">
         <v>1052</v>
       </c>
-      <c r="C90" s="33"/>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A91" s="15" t="s">
+      <c r="C96" s="33"/>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B91" s="17" t="s">
+      <c r="B97" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C91" s="33"/>
-    </row>
-    <row r="92" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A92" s="15" t="s">
+      <c r="C97" s="33"/>
+    </row>
+    <row r="98" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A98" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B92" s="17" t="s">
+      <c r="B98" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C92" s="33"/>
-    </row>
-    <row r="93" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A93" s="15" t="s">
+      <c r="C98" s="33"/>
+    </row>
+    <row r="99" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A99" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B93" s="17" t="s">
+      <c r="B99" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C93" s="33"/>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A94" s="15" t="s">
+      <c r="C99" s="33"/>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B94" s="17" t="s">
+      <c r="B100" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C94" s="33"/>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A95" s="15" t="s">
+      <c r="C100" s="33"/>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A101" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B95" s="17" t="s">
+      <c r="B101" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C95" s="33"/>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A96" s="15"/>
-      <c r="B96" s="17"/>
-      <c r="C96" s="33"/>
+      <c r="C101" s="33"/>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" s="15"/>
+      <c r="B102" s="17"/>
+      <c r="C102" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Report wording: cap-only confidence factor shown only when it set the grade; 'ageing M&E being replaced' (workbook v5.19)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1807">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4243" uniqueCount="1809">
   <si>
     <t>3. Settings</t>
   </si>
@@ -5452,6 +5452,12 @@
   </si>
   <si>
     <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.18 (October 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRM1 COST ESTIMATE TOOL — v5.19 (October 2026)</t>
   </si>
 </sst>
 </file>
@@ -6072,7 +6078,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BBCD35-3C7D-4CAC-A46E-6C3CC3E31849}">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.7109375" style="8" customWidth="1"/>
@@ -6083,7 +6089,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>1806</v>
+        <v>1808</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="33"/>
@@ -6774,220 +6780,232 @@
     <row r="81" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="17" t="inlineStr">
         <is>
-          <t>v5.18 — 8 Oct 2026</t>
+          <t>v5.19 — 9 Oct 2026</t>
         </is>
       </c>
       <c r="B81" s="17" t="inlineStr">
         <is>
-          <t>Professional fees by procurement route: new ▶ route_fees on '3. Settings'. Design and build: client fees −3 points and contractor's design 2% of construction (Claycroft D&amp;B 2.1%); two-stage (PCSA): −1.5 and 1%; traditional and construction management unchanged. Only while Stage 4 is still to do. The preferred route comes from the Procurement Reference.</t>
+          <t>Wording only, no figure changed: ▶ risk_allowance label 'ageing M&amp;E, being replaced' → 'ageing M&amp;E being replaced' (it read as two items in the report).</t>
         </is>
       </c>
     </row>
     <row r="82" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="17" t="inlineStr">
         <is>
-          <t>v5.17 — 8 Oct 2026</t>
+          <t>v5.18 — 8 Oct 2026</t>
         </is>
       </c>
       <c r="B82" s="17" t="inlineStr">
         <is>
-          <t>Inflation from the rate base date: new ▶ inflation on '3. Settings'. Rates are at Q3 2026 (15 Aug 2026); 3.5% a year compounded to the programme's construction mid-point, capped at 12%. Replaces the banded F rows of ▶ percentage_rules.</t>
+          <t>Professional fees by procurement route: new ▶ route_fees on '3. Settings'. Design and build: client fees −3 points and contractor's design 2% of construction (Claycroft D&amp;B 2.1%); two-stage (PCSA): −1.5 and 1%; traditional and construction management unchanged. Only while Stage 4 is still to do. The preferred route comes from the Procurement Reference.</t>
         </is>
       </c>
     </row>
     <row r="83" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="17" t="inlineStr">
         <is>
-          <t>v5.16 — 8 Oct 2026</t>
+          <t>v5.17 — 8 Oct 2026</t>
         </is>
       </c>
       <c r="B83" s="17" t="inlineStr">
         <is>
-          <t>Risk allowance in the four NRM1 categories: new ▶ risk_allowance on '3. Settings' (design development by design stage, construction, employer change, employer other; cap 25%). Replaces E and the fixed 5% contingency H. Items already priced in the scope reduce or remove their risk row; occupation, deadline and phasing stay in prelims and programme only.</t>
+          <t>Inflation from the rate base date: new ▶ inflation on '3. Settings'. Rates are at Q3 2026 (15 Aug 2026); 3.5% a year compounded to the programme's construction mid-point, capped at 12%. Replaces the banded F rows of ▶ percentage_rules.</t>
         </is>
       </c>
     </row>
     <row r="84" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A84" s="17" t="inlineStr">
         <is>
-          <t>v5.15 — 7 Oct 2026</t>
+          <t>v5.16 — 8 Oct 2026</t>
         </is>
       </c>
       <c r="B84" s="17" t="inlineStr">
         <is>
-          <t>Confidence grade scored from the workbook: new ▶ confidence on '3. Settings' (points per factor, grade thresholds, caps: Stage 0–1 at B; existing building with neither a condition nor an R&amp;D survey at C). ▶ range_widths skewed upwards: A −10/+15, B −10/+20, C −15/+25, D −20/+35.</t>
+          <t>Risk allowance in the four NRM1 categories: new ▶ risk_allowance on '3. Settings' (design development by design stage, construction, employer change, employer other; cap 25%). Replaces E and the fixed 5% contingency H. Items already priced in the scope reduce or remove their risk row; occupation, deadline and phasing stay in prelims and programme only.</t>
         </is>
       </c>
     </row>
     <row r="85" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A85" s="17" t="inlineStr">
         <is>
-          <t>v5.14 — 6 Oct 2026</t>
+          <t>v5.15 — 7 Oct 2026</t>
         </is>
       </c>
       <c r="B85" s="17" t="inlineStr">
         <is>
-          <t>Preliminaries: 7% base (relaxed, vacant, no restrictions) plus occupation, restricted hours, shared access, programme over 18 months, 4+ M&amp;E items, heritage, hard deadline and speed-first, capped at 11%; Outer London +2 and Inner London +3 with a 14% cap. The ▶ percentage_rules header states the on-cost order the app uses (OH&amp;P on works + prelims; risk on base cost; inflation on the cost limit).</t>
+          <t>Confidence grade scored from the workbook: new ▶ confidence on '3. Settings' (points per factor, grade thresholds, caps: Stage 0–1 at B; existing building with neither a condition nor an R&amp;D survey at C). ▶ range_widths skewed upwards: A −10/+15, B −10/+20, C −15/+25, D −20/+35.</t>
         </is>
       </c>
     </row>
     <row r="86" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A86" s="17" t="inlineStr">
         <is>
-          <t>v5.13 — 5 Oct 2026</t>
+          <t>v5.14 — 6 Oct 2026</t>
         </is>
       </c>
       <c r="B86" s="17" t="inlineStr">
         <is>
-          <t>Scope dependencies ('When selected' SUGGEST on '4. Scope rules'): kitchens and bathrooms → ventilation (domestic also → internal doors); strip-out → fire stopping, emergency lighting, asbestos removal; full power installation → fire stopping, emergency lighting. The report flags any that are not ticked.</t>
+          <t>Preliminaries: 7% base (relaxed, vacant, no restrictions) plus occupation, restricted hours, shared access, programme over 18 months, 4+ M&amp;E items, heritage, hard deadline and speed-first, capped at 11%; Outer London +2 and Inner London +3 with a 14% cap. The ▶ percentage_rules header states the on-cost order the app uses (OH&amp;P on works + prelims; risk on base cost; inflation on the cost limit).</t>
         </is>
       </c>
     </row>
     <row r="87" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A87" s="17" t="inlineStr">
         <is>
-          <t>v5.12 — 4 Oct 2026</t>
+          <t>v5.13 — 5 Oct 2026</t>
         </is>
       </c>
       <c r="B87" s="17" t="inlineStr">
         <is>
-          <t>Rates updated from the owner's review of the v5.11 suggestions (column AA marked green = accept, amber = owner's figure, red = no change). 25 rows changed; each row's Basic, Standard, High and New build Std / High move by the same ratio as Standard (new Std ÷ old Std), rounded. Std (Refurb &amp; Fit-out): demolition 130→100; roof 110→190; external walls 60→100; windows 120→140; internal walls 110→150; internal doors 60→100; floor finishes 75→85; ceilings 50→80; staff kitchenette 4,000→6,000; signage 10→12; catering kitchen 690→1,000; ASHP full system 78→190 and district heating full system 54→120 (now figures, not = 5.1a × factor; their plant-only / radiators-only rows still follow by formula); water and drainage 65→80; ventilation 45→75 (owner); extract fans 19→22; BMS 15→25; lighting 33→80 (5.8b follows at 75%); fire alarm 18→35; data 18→20; security 15→20; passenger lift 40,000→60,000 (owner); builder's work 18→12; foul drainage 6→10 (owner); external utilities 10→25. Kept: toilets and accessible WCs (owner: no change) and the 20 'keep' rows; 5.2b visible-fittings water fixed at its figures (19.5 Std, Lakeside tender) so it does not follow 5.2a. Changed rows' Source = 'Your figure'.</t>
+          <t>Scope dependencies ('When selected' SUGGEST on '4. Scope rules'): kitchens and bathrooms → ventilation (domestic also → internal doors); strip-out → fire stopping, emergency lighting, asbestos removal; full power installation → fire stopping, emergency lighting. The report flags any that are not ticked.</t>
         </is>
       </c>
     </row>
     <row r="88" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A88" s="17" t="inlineStr">
         <is>
+          <t>v5.12 — 4 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B88" s="17" t="inlineStr">
+        <is>
+          <t>Rates updated from the owner's review of the v5.11 suggestions (column AA marked green = accept, amber = owner's figure, red = no change). 25 rows changed; each row's Basic, Standard, High and New build Std / High move by the same ratio as Standard (new Std ÷ old Std), rounded. Std (Refurb &amp; Fit-out): demolition 130→100; roof 110→190; external walls 60→100; windows 120→140; internal walls 110→150; internal doors 60→100; floor finishes 75→85; ceilings 50→80; staff kitchenette 4,000→6,000; signage 10→12; catering kitchen 690→1,000; ASHP full system 78→190 and district heating full system 54→120 (now figures, not = 5.1a × factor; their plant-only / radiators-only rows still follow by formula); water and drainage 65→80; ventilation 45→75 (owner); extract fans 19→22; BMS 15→25; lighting 33→80 (5.8b follows at 75%); fire alarm 18→35; data 18→20; security 15→20; passenger lift 40,000→60,000 (owner); builder's work 18→12; foul drainage 6→10 (owner); external utilities 10→25. Kept: toilets and accessible WCs (owner: no change) and the 20 'keep' rows; 5.2b visible-fittings water fixed at its figures (19.5 Std, Lakeside tender) so it does not follow 5.2a. Changed rows' Source = 'Your figure'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="17" t="inlineStr">
+        <is>
           <t>v5.11 — 4 Oct 2026</t>
         </is>
       </c>
-      <c r="B88" s="17" t="inlineStr">
+      <c r="B89" s="17" t="inlineStr">
         <is>
           <t>Evidence only, no rates changed. Six more project columns on '2. Rates' beside Whitefields (R) and Claycroft (S), each a plain figure in the row's unit on this workbook's basis: T Lakeside S&amp;F (15 rows), U Computer Science (6), V Scarman Public Toilets Phase 2, high spec (12), W Co-op store fit-out (19), X IBRB café (7), Y Riley Court Psychology refurbishment (27, from the signed contract CSA). Column Z averages R–Y on 47 rows. Row 24 explains the columns and lists the evidence that has no row (scaffold, retail refrigeration and equipment, preliminaries %). Columns AA–AB: Claude's suggested Refurb &amp; Fit-out Std rate and the reason, on all 47 rows (25 raise, 2 lower, 20 keep).</t>
         </is>
       </c>
     </row>
-    <row r="89" spans="1:3" s="54" customFormat="1" ht="104.0" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="17" t="s">
+    <row r="90" spans="1:3" s="54" customFormat="1" ht="104.0" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="17" t="s">
         <v>1778</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="B90" s="17" t="s">
         <v>1779</v>
       </c>
-      <c r="C89" s="60"/>
-    </row>
-    <row r="90" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="17" t="s">
+      <c r="C90" s="60"/>
+    </row>
+    <row r="91" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="17" t="s">
         <v>1748</v>
       </c>
-      <c r="B90" s="17" t="s">
+      <c r="B91" s="17" t="s">
         <v>1783</v>
-      </c>
-      <c r="C90" s="60"/>
-    </row>
-    <row r="91" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A91" s="17" t="s">
-        <v>1722</v>
-      </c>
-      <c r="B91" s="17" t="s">
-        <v>1737</v>
       </c>
       <c r="C91" s="60"/>
     </row>
     <row r="92" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A92" s="17" t="s">
-        <v>1711</v>
+        <v>1722</v>
       </c>
       <c r="B92" s="17" t="s">
-        <v>1712</v>
+        <v>1737</v>
       </c>
       <c r="C92" s="60"/>
     </row>
     <row r="93" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A93" s="17" t="s">
+        <v>1711</v>
+      </c>
+      <c r="B93" s="17" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C93" s="60"/>
+    </row>
+    <row r="94" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A94" s="17" t="s">
         <v>1632</v>
       </c>
-      <c r="B93" s="17" t="s">
+      <c r="B94" s="17" t="s">
         <v>1634</v>
       </c>
-      <c r="C93" s="60"/>
-    </row>
-    <row r="94" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A94" s="15" t="s">
+      <c r="C94" s="60"/>
+    </row>
+    <row r="95" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A95" s="15" t="s">
         <v>1620</v>
       </c>
-      <c r="B94" s="17" t="s">
+      <c r="B95" s="17" t="s">
         <v>1621</v>
       </c>
-      <c r="C94" s="33"/>
-    </row>
-    <row r="95" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A95" s="15" t="s">
+      <c r="C95" s="33"/>
+    </row>
+    <row r="96" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A96" s="15" t="s">
         <v>1060</v>
       </c>
-      <c r="B95" s="17" t="s">
+      <c r="B96" s="17" t="s">
         <v>1061</v>
       </c>
-      <c r="C95" s="33"/>
-    </row>
-    <row r="96" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A96" s="15" t="s">
+      <c r="C96" s="33"/>
+    </row>
+    <row r="97" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A97" s="15" t="s">
         <v>1051</v>
       </c>
-      <c r="B96" s="17" t="s">
+      <c r="B97" s="17" t="s">
         <v>1052</v>
       </c>
-      <c r="C96" s="33"/>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A97" s="15" t="s">
+      <c r="C97" s="33"/>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B97" s="17" t="s">
+      <c r="B98" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C97" s="33"/>
-    </row>
-    <row r="98" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A98" s="15" t="s">
+      <c r="C98" s="33"/>
+    </row>
+    <row r="99" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A99" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B98" s="17" t="s">
+      <c r="B99" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C98" s="33"/>
-    </row>
-    <row r="99" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A99" s="15" t="s">
+      <c r="C99" s="33"/>
+    </row>
+    <row r="100" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A100" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B99" s="17" t="s">
+      <c r="B100" s="17" t="s">
         <v>28</v>
-      </c>
-      <c r="C99" s="33"/>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A100" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B100" s="17" t="s">
-        <v>30</v>
       </c>
       <c r="C100" s="33"/>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B101" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C101" s="33"/>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B101" s="17" t="s">
+      <c r="B102" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C101" s="33"/>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A102" s="15"/>
-      <c r="B102" s="17"/>
       <c r="C102" s="33"/>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103" s="15"/>
+      <c r="B103" s="17"/>
+      <c r="C103" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14492,7 +14510,7 @@
         <v>749</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>750</v>
@@ -14503,7 +14521,7 @@
         <v>751</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>1802</v>
+        <v>1807</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -18195,7 +18213,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>ageing M&amp;E, being replaced</t>
+          <t>ageing M&amp;E being replaced</t>
         </is>
       </c>
       <c r="D238" s="2">

</xml_diff>

<commit_message>
No backup numbers in code: every figure from the workbooks (NRM1 v5.23)
- Cost: removed the fallback prelims 8/10, OH&P 11, fee ladder 6-13.5 and
  risk 5/10. The loader now refuses A/E BASE rows without a cap, OH&P (B)
  rows that leave a works value uncovered and fee (C) BASE rows that leave
  a design stage 0-4 uncovered. A blank Q4.5 reads as Stage 0.
- Programme: removed the Q23 / OCC / ACC / PH-1 / FN-1 / PROG-FLOAT
  defaults; REQUIRED_MODIFIERS are checked at load.
- Time to tender is the programme's construction start week, not
  "programme - construction - 2 weeks".
- Report risk level limits (Low <= 11%, Medium <= 13%) moved to ▶ factors
  risk_level_low_max / risk_level_medium_max (NRM1 v5.23, via Excel COM;
  nothing else in the workbook changed).

All 63 saved test scenarios price identically before and after; 721 tests pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NRM1_Cost_Estimate_Tool_v5_2.xlsx
+++ b/NRM1_Cost_Estimate_Tool_v5_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nabil\estates-ai-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC8CEDBA-193B-44AD-83E1-FA7C8520DD6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8930164-0AD5-4E3B-93E8-2E6FB0A3A4B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4603" uniqueCount="2013">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4612" uniqueCount="2020">
   <si>
     <t>3. Settings</t>
   </si>
@@ -6070,6 +6070,27 @@
   </si>
   <si>
     <t>No rate changed. Industrial / warehouse new build and extensions are split into offices and the main space (owner, 10 Oct 2026): new inputs OFFICES (Q1.3a share × GIFA; default GIFA × r.office_share) and PRODUCTION (Q1.3b Factory / production → the rest of the floor, Storage / warehouse → 0); new ratio office_share 0.10 (suggestion, AI estimate – verify). On those projects internal walls, internal doors, wall / floor / ceiling finishes, signage and data are measured on OFFICES, and heating, water, ventilation, power and builder's work on OFFICES + PRODUCTION. Every other building use and project type is measured on GIFA as before.</t>
+  </si>
+  <si>
+    <t>risk_level_low_max</t>
+  </si>
+  <si>
+    <t>Report risk level: risk + contingency % at or below this reads Low</t>
+  </si>
+  <si>
+    <t>Every report (label only; never changes the estimate)</t>
+  </si>
+  <si>
+    <t>risk_level_medium_max</t>
+  </si>
+  <si>
+    <t>Report risk level: at or below this reads Medium; above it, High</t>
+  </si>
+  <si>
+    <t>v5.23 — 11 Oct 2026</t>
+  </si>
+  <si>
+    <t>No figure the estimate uses changed. The last number the app held in its code now lives here: ▶ factors gains risk_level_low_max (11) and risk_level_medium_max (13) — the risk + contingency % at or below which the report's risk level reads Low or Medium (above: High). The app now also refuses this workbook if a prelims (A) or risk (E) BASE row loses its cap, the OH&amp;P (B) rows leave a works value uncovered, or the fee (C) BASE rows leave a design stage 0–4 uncovered — it no longer has backup percentages to fall back on.</t>
   </si>
 </sst>
 </file>
@@ -6696,7 +6717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1BBCD35-3C7D-4CAC-A46E-6C3CC3E31849}">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.7109375" style="8" customWidth="1"/>
@@ -7391,223 +7412,231 @@
       <c r="B80" s="16"/>
       <c r="C80" s="34"/>
     </row>
-    <row r="81" spans="1:3" s="54" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3" s="54" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A81" s="17" t="s">
-        <v>2011</v>
+        <v>2018</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>2012</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="82" spans="1:3" s="54" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A82" s="17" t="s">
-        <v>1998</v>
+        <v>2011</v>
       </c>
       <c r="B82" s="17" t="s">
-        <v>1999</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="83" spans="1:3" s="54" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
       <c r="A83" s="17" t="s">
+        <v>1998</v>
+      </c>
+      <c r="B83" s="17" t="s">
+        <v>1999</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" s="54" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A84" s="17" t="s">
         <v>1969</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B84" s="17" t="s">
         <v>1970</v>
       </c>
     </row>
-    <row r="84" spans="1:3" s="54" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A84" s="17" t="s">
+    <row r="85" spans="1:3" s="54" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A85" s="17" t="s">
         <v>1731</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B85" s="17" t="s">
         <v>1732</v>
       </c>
     </row>
-    <row r="85" spans="1:3" s="54" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A85" s="17" t="s">
+    <row r="86" spans="1:3" s="54" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A86" s="17" t="s">
         <v>1733</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B86" s="17" t="s">
         <v>1734</v>
       </c>
     </row>
-    <row r="86" spans="1:3" s="54" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A86" s="17" t="s">
+    <row r="87" spans="1:3" s="54" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A87" s="17" t="s">
         <v>1735</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B87" s="17" t="s">
         <v>1736</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" s="54" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A87" s="17" t="s">
-        <v>1737</v>
-      </c>
-      <c r="B87" s="17" t="s">
-        <v>1738</v>
       </c>
     </row>
     <row r="88" spans="1:3" s="54" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A88" s="17" t="s">
-        <v>1739</v>
+        <v>1737</v>
       </c>
       <c r="B88" s="17" t="s">
-        <v>1740</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="89" spans="1:3" s="54" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A89" s="17" t="s">
-        <v>1741</v>
+        <v>1739</v>
       </c>
       <c r="B89" s="17" t="s">
-        <v>1742</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="90" spans="1:3" s="54" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A90" s="17" t="s">
+        <v>1741</v>
+      </c>
+      <c r="B90" s="17" t="s">
+        <v>1742</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" s="54" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A91" s="17" t="s">
         <v>1743</v>
       </c>
-      <c r="B90" s="17" t="s">
+      <c r="B91" s="17" t="s">
         <v>1744</v>
       </c>
     </row>
-    <row r="91" spans="1:3" s="54" customFormat="1" ht="114.75" x14ac:dyDescent="0.2">
-      <c r="A91" s="17" t="s">
+    <row r="92" spans="1:3" s="54" customFormat="1" ht="114.75" x14ac:dyDescent="0.2">
+      <c r="A92" s="17" t="s">
         <v>1745</v>
       </c>
-      <c r="B91" s="17" t="s">
+      <c r="B92" s="17" t="s">
         <v>1746</v>
       </c>
     </row>
-    <row r="92" spans="1:3" s="54" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A92" s="17" t="s">
+    <row r="93" spans="1:3" s="54" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A93" s="17" t="s">
         <v>1747</v>
       </c>
-      <c r="B92" s="17" t="s">
+      <c r="B93" s="17" t="s">
         <v>1748</v>
       </c>
     </row>
-    <row r="93" spans="1:3" s="54" customFormat="1" ht="104.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="17" t="s">
+    <row r="94" spans="1:3" s="54" customFormat="1" ht="104.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A94" s="17" t="s">
         <v>1715</v>
       </c>
-      <c r="B93" s="17" t="s">
+      <c r="B94" s="17" t="s">
         <v>1716</v>
       </c>
-      <c r="C93" s="60"/>
-    </row>
-    <row r="94" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="17" t="s">
+      <c r="C94" s="60"/>
+    </row>
+    <row r="95" spans="1:3" s="54" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="17" t="s">
         <v>1689</v>
       </c>
-      <c r="B94" s="17" t="s">
+      <c r="B95" s="17" t="s">
         <v>1718</v>
       </c>
-      <c r="C94" s="60"/>
-    </row>
-    <row r="95" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A95" s="17" t="s">
+      <c r="C95" s="60"/>
+    </row>
+    <row r="96" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A96" s="17" t="s">
         <v>1680</v>
       </c>
-      <c r="B95" s="17" t="s">
+      <c r="B96" s="17" t="s">
         <v>1686</v>
       </c>
-      <c r="C95" s="60"/>
-    </row>
-    <row r="96" spans="1:3" s="54" customFormat="1" ht="89.25" x14ac:dyDescent="0.2">
-      <c r="A96" s="17" t="s">
+      <c r="C96" s="60"/>
+    </row>
+    <row r="97" spans="1:3" s="54" customFormat="1" ht="89.25" x14ac:dyDescent="0.2">
+      <c r="A97" s="17" t="s">
         <v>1678</v>
       </c>
-      <c r="B96" s="17" t="s">
+      <c r="B97" s="17" t="s">
         <v>1679</v>
       </c>
-      <c r="C96" s="60"/>
-    </row>
-    <row r="97" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A97" s="17" t="s">
+      <c r="C97" s="60"/>
+    </row>
+    <row r="98" spans="1:3" s="54" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A98" s="17" t="s">
         <v>1619</v>
       </c>
-      <c r="B97" s="17" t="s">
+      <c r="B98" s="17" t="s">
         <v>1621</v>
       </c>
-      <c r="C97" s="60"/>
-    </row>
-    <row r="98" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A98" s="15" t="s">
+      <c r="C98" s="60"/>
+    </row>
+    <row r="99" spans="1:3" ht="102" x14ac:dyDescent="0.2">
+      <c r="A99" s="15" t="s">
         <v>1608</v>
       </c>
-      <c r="B98" s="17" t="s">
+      <c r="B99" s="17" t="s">
         <v>1609</v>
       </c>
-      <c r="C98" s="33"/>
-    </row>
-    <row r="99" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A99" s="15" t="s">
+      <c r="C99" s="33"/>
+    </row>
+    <row r="100" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A100" s="15" t="s">
         <v>1051</v>
       </c>
-      <c r="B99" s="17" t="s">
+      <c r="B100" s="17" t="s">
         <v>1052</v>
       </c>
-      <c r="C99" s="33"/>
-    </row>
-    <row r="100" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A100" s="15" t="s">
+      <c r="C100" s="33"/>
+    </row>
+    <row r="101" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A101" s="15" t="s">
         <v>1042</v>
       </c>
-      <c r="B100" s="17" t="s">
+      <c r="B101" s="17" t="s">
         <v>1043</v>
       </c>
-      <c r="C100" s="33"/>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A101" s="15" t="s">
+      <c r="C101" s="33"/>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B101" s="17" t="s">
+      <c r="B102" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C101" s="33"/>
-    </row>
-    <row r="102" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A102" s="15" t="s">
+      <c r="C102" s="33"/>
+    </row>
+    <row r="103" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A103" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B102" s="17" t="s">
+      <c r="B103" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C102" s="33"/>
-    </row>
-    <row r="103" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A103" s="15" t="s">
+      <c r="C103" s="33"/>
+    </row>
+    <row r="104" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A104" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B103" s="17" t="s">
+      <c r="B104" s="17" t="s">
         <v>28</v>
-      </c>
-      <c r="C103" s="33"/>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A104" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B104" s="17" t="s">
-        <v>30</v>
       </c>
       <c r="C104" s="33"/>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B105" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C105" s="33"/>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A106" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B105" s="17" t="s">
+      <c r="B106" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C105" s="33"/>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A106" s="15"/>
-      <c r="B106" s="17"/>
       <c r="C106" s="33"/>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A107" s="15"/>
+      <c r="B107" s="17"/>
+      <c r="C107" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14894,7 +14923,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G290"/>
+  <dimension ref="A1:G292"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -14944,8 +14973,8 @@
       <c r="A6" s="2" t="s">
         <v>743</v>
       </c>
-      <c r="B6" s="61" t="s">
-        <v>1404</v>
+      <c r="B6" s="61">
+        <v>5.23</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>744</v>
@@ -14956,7 +14985,7 @@
         <v>745</v>
       </c>
       <c r="B7" s="62">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -16897,80 +16926,74 @@
         <v>1982</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A142" s="3" t="s">
+    <row r="141" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A141" s="2" t="s">
+        <v>2013</v>
+      </c>
+      <c r="B141" s="2">
+        <v>11</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>2014</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>2015</v>
+      </c>
+      <c r="E141" s="7" t="s">
+        <v>1982</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A142" s="2" t="s">
+        <v>2016</v>
+      </c>
+      <c r="B142" s="2">
+        <v>13</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>2017</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>2015</v>
+      </c>
+      <c r="E142" s="7" t="s">
+        <v>1982</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A144" s="3" t="s">
         <v>929</v>
       </c>
-      <c r="B142" s="3" t="s">
+      <c r="B144" s="3" t="s">
         <v>1727</v>
       </c>
-      <c r="C142" s="4"/>
-      <c r="D142" s="4"/>
-      <c r="E142" s="4"/>
-      <c r="F142" s="4"/>
-      <c r="G142" s="4"/>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A143" s="6" t="s">
+      <c r="C144" s="4"/>
+      <c r="D144" s="4"/>
+      <c r="E144" s="4"/>
+      <c r="F144" s="4"/>
+      <c r="G144" s="4"/>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A145" s="6" t="s">
         <v>750</v>
       </c>
-      <c r="B143" s="6" t="s">
+      <c r="B145" s="6" t="s">
         <v>930</v>
       </c>
-      <c r="C143" s="6" t="s">
+      <c r="C145" s="6" t="s">
         <v>931</v>
       </c>
-      <c r="D143" s="6" t="s">
+      <c r="D145" s="6" t="s">
         <v>932</v>
       </c>
-      <c r="E143" s="6" t="s">
+      <c r="E145" s="6" t="s">
         <v>933</v>
       </c>
-      <c r="F143" s="6" t="s">
+      <c r="F145" s="6" t="s">
         <v>934</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A144" s="2" t="s">
-        <v>935</v>
-      </c>
-      <c r="B144" s="2" t="s">
-        <v>936</v>
-      </c>
-      <c r="C144" s="2" t="s">
-        <v>937</v>
-      </c>
-      <c r="D144" s="2" t="s">
-        <v>1804</v>
-      </c>
-      <c r="E144" s="2">
-        <v>7</v>
-      </c>
-      <c r="F144" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A145" s="2" t="s">
-        <v>935</v>
-      </c>
-      <c r="B145" s="2" t="s">
-        <v>936</v>
-      </c>
-      <c r="C145" s="2" t="s">
-        <v>938</v>
-      </c>
-      <c r="D145" s="2" t="s">
-        <v>939</v>
-      </c>
-      <c r="E145" s="2">
-        <v>2</v>
-      </c>
-      <c r="F145" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>935</v>
       </c>
@@ -16978,13 +17001,13 @@
         <v>936</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>940</v>
+        <v>1804</v>
       </c>
       <c r="E146" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F146" s="2">
         <v>11</v>
@@ -17001,16 +17024,16 @@
         <v>938</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="E147" s="2">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="F147" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="148" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>935</v>
       </c>
@@ -17021,16 +17044,16 @@
         <v>938</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>1959</v>
+        <v>940</v>
       </c>
       <c r="E148" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F148" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="149" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>935</v>
       </c>
@@ -17041,7 +17064,7 @@
         <v>938</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>1960</v>
+        <v>941</v>
       </c>
       <c r="E149" s="2">
         <v>0.5</v>
@@ -17061,7 +17084,7 @@
         <v>938</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>1961</v>
+        <v>1959</v>
       </c>
       <c r="E150" s="2">
         <v>0.5</v>
@@ -17081,7 +17104,7 @@
         <v>938</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>1962</v>
+        <v>1960</v>
       </c>
       <c r="E151" s="2">
         <v>0.5</v>
@@ -17090,7 +17113,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>935</v>
       </c>
@@ -17101,7 +17124,7 @@
         <v>938</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>942</v>
+        <v>1961</v>
       </c>
       <c r="E152" s="2">
         <v>0.5</v>
@@ -17110,7 +17133,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>935</v>
       </c>
@@ -17121,7 +17144,7 @@
         <v>938</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>1805</v>
+        <v>1962</v>
       </c>
       <c r="E153" s="2">
         <v>0.5</v>
@@ -17130,7 +17153,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="154" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>935</v>
       </c>
@@ -17141,7 +17164,7 @@
         <v>938</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>1806</v>
+        <v>942</v>
       </c>
       <c r="E154" s="2">
         <v>0.5</v>
@@ -17161,16 +17184,16 @@
         <v>938</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>1807</v>
+        <v>1805</v>
       </c>
       <c r="E155" s="2">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="F155" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>935</v>
       </c>
@@ -17181,10 +17204,10 @@
         <v>938</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>1808</v>
+        <v>1806</v>
       </c>
       <c r="E156" s="2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F156" s="2">
         <v>11</v>
@@ -17201,13 +17224,13 @@
         <v>938</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>1809</v>
+        <v>1807</v>
       </c>
       <c r="E157" s="2">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="F157" s="2">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.25">
@@ -17221,50 +17244,54 @@
         <v>938</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>1810</v>
+        <v>1808</v>
       </c>
       <c r="E158" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F158" s="2">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>943</v>
+        <v>935</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>944</v>
+        <v>936</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>945</v>
+        <v>938</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>946</v>
+        <v>1809</v>
       </c>
       <c r="E159" s="2">
-        <v>11</v>
-      </c>
-      <c r="F159" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="F159" s="2">
+        <v>14</v>
+      </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>943</v>
+        <v>935</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>944</v>
+        <v>936</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>945</v>
+        <v>938</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>947</v>
+        <v>1810</v>
       </c>
       <c r="E160" s="2">
-        <v>9.5</v>
-      </c>
-      <c r="F160" s="2"/>
+        <v>3</v>
+      </c>
+      <c r="F160" s="2">
+        <v>14</v>
+      </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
@@ -17277,46 +17304,46 @@
         <v>945</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="E161" s="2">
-        <v>8.5</v>
+        <v>11</v>
       </c>
       <c r="F161" s="2"/>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>949</v>
+        <v>943</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>937</v>
+        <v>945</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>951</v>
+        <v>947</v>
       </c>
       <c r="E162" s="2">
-        <v>13.5</v>
+        <v>9.5</v>
       </c>
       <c r="F162" s="2"/>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>949</v>
+        <v>943</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>937</v>
+        <v>945</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>952</v>
+        <v>948</v>
       </c>
       <c r="E163" s="2">
-        <v>11.5</v>
+        <v>8.5</v>
       </c>
       <c r="F163" s="2"/>
     </row>
@@ -17331,10 +17358,10 @@
         <v>937</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="E164" s="2">
-        <v>8.5</v>
+        <v>13.5</v>
       </c>
       <c r="F164" s="2"/>
     </row>
@@ -17349,10 +17376,10 @@
         <v>937</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="E165" s="2">
-        <v>6</v>
+        <v>11.5</v>
       </c>
       <c r="F165" s="2"/>
     </row>
@@ -17364,13 +17391,13 @@
         <v>950</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>1037</v>
+        <v>953</v>
       </c>
       <c r="E166" s="2">
-        <v>1.5</v>
+        <v>8.5</v>
       </c>
       <c r="F166" s="2"/>
     </row>
@@ -17382,17 +17409,17 @@
         <v>950</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="E167" s="2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F167" s="2"/>
     </row>
-    <row r="168" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>949</v>
       </c>
@@ -17403,46 +17430,46 @@
         <v>938</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>956</v>
+        <v>1037</v>
       </c>
       <c r="E168" s="2">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="F168" s="2"/>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>957</v>
+        <v>949</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>958</v>
+        <v>950</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>959</v>
+        <v>955</v>
       </c>
       <c r="E169" s="2">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="F169" s="2"/>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>957</v>
+        <v>949</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>958</v>
+        <v>950</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="D170" s="2" t="s">
-        <v>960</v>
+        <v>956</v>
       </c>
       <c r="E170" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F170" s="2"/>
     </row>
@@ -17457,10 +17484,10 @@
         <v>937</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="E171" s="2">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="F171" s="2"/>
     </row>
@@ -17475,10 +17502,10 @@
         <v>937</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
       <c r="E172" s="2">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="F172" s="2"/>
     </row>
@@ -17493,10 +17520,10 @@
         <v>937</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="E173" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F173" s="2"/>
     </row>
@@ -17511,10 +17538,10 @@
         <v>937</v>
       </c>
       <c r="D174" s="2" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="E174" s="2">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F174" s="2"/>
     </row>
@@ -17526,17 +17553,17 @@
         <v>958</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="E175" s="2">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="F175" s="2"/>
     </row>
-    <row r="176" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>957</v>
       </c>
@@ -17547,52 +17574,48 @@
         <v>937</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
       <c r="E176" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F176" s="2"/>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>967</v>
+        <v>957</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>968</v>
+        <v>958</v>
       </c>
       <c r="C177" s="2" t="s">
+        <v>938</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>965</v>
+      </c>
+      <c r="E177" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F177" s="2"/>
+    </row>
+    <row r="178" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A178" s="2" t="s">
+        <v>957</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>958</v>
+      </c>
+      <c r="C178" s="2" t="s">
         <v>937</v>
       </c>
-      <c r="D177" s="2" t="s">
-        <v>969</v>
-      </c>
-      <c r="E177" s="2">
-        <v>5</v>
-      </c>
-      <c r="F177" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A178" s="2" t="s">
-        <v>967</v>
-      </c>
-      <c r="B178" s="2" t="s">
-        <v>968</v>
-      </c>
-      <c r="C178" s="2" t="s">
-        <v>938</v>
-      </c>
       <c r="D178" s="2" t="s">
-        <v>970</v>
+        <v>966</v>
       </c>
       <c r="E178" s="2">
-        <v>2</v>
-      </c>
-      <c r="F178" s="2">
-        <v>10</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="F178" s="2"/>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
@@ -17602,13 +17625,13 @@
         <v>968</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
       <c r="E179" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F179" s="2">
         <v>10</v>
@@ -17625,10 +17648,10 @@
         <v>938</v>
       </c>
       <c r="D180" s="2" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="E180" s="2">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="F180" s="2">
         <v>10</v>
@@ -17645,10 +17668,10 @@
         <v>938</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
       <c r="E181" s="2">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="F181" s="2">
         <v>10</v>
@@ -17665,10 +17688,10 @@
         <v>938</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="E182" s="2">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F182" s="2">
         <v>10</v>
@@ -17685,10 +17708,10 @@
         <v>938</v>
       </c>
       <c r="D183" s="2" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
       <c r="E183" s="2">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F183" s="2">
         <v>10</v>
@@ -17705,10 +17728,10 @@
         <v>938</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="E184" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F184" s="2">
         <v>10</v>
@@ -17725,7 +17748,7 @@
         <v>938</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="E185" s="2">
         <v>0.5</v>
@@ -17745,7 +17768,7 @@
         <v>938</v>
       </c>
       <c r="D186" s="2" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="E186" s="2">
         <v>0.5</v>
@@ -17765,10 +17788,10 @@
         <v>938</v>
       </c>
       <c r="D187" s="2" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="E187" s="2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F187" s="2">
         <v>10</v>
@@ -17785,7 +17808,7 @@
         <v>938</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>939</v>
+        <v>978</v>
       </c>
       <c r="E188" s="2">
         <v>0.5</v>
@@ -17794,64 +17817,64 @@
         <v>10</v>
       </c>
     </row>
-    <row r="189" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>980</v>
+        <v>967</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>981</v>
+        <v>968</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>982</v>
+        <v>938</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
       <c r="E189" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F189" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>984</v>
+        <v>967</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>985</v>
+        <v>968</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>986</v>
+        <v>938</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>987</v>
+        <v>939</v>
       </c>
       <c r="E190" s="2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F190" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>984</v>
+        <v>980</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>986</v>
+        <v>982</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>988</v>
+        <v>983</v>
       </c>
       <c r="E191" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F191" s="2">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.25">
@@ -17865,10 +17888,10 @@
         <v>986</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="E192" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F192" s="2">
         <v>12</v>
@@ -17885,10 +17908,10 @@
         <v>986</v>
       </c>
       <c r="D193" s="2" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="E193" s="2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F193" s="2">
         <v>12</v>
@@ -17899,16 +17922,16 @@
         <v>984</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>991</v>
+        <v>985</v>
       </c>
       <c r="C194" s="2" t="s">
         <v>986</v>
       </c>
       <c r="D194" s="2" t="s">
-        <v>992</v>
+        <v>989</v>
       </c>
       <c r="E194" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F194" s="2">
         <v>12</v>
@@ -17919,16 +17942,16 @@
         <v>984</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>991</v>
+        <v>985</v>
       </c>
       <c r="C195" s="2" t="s">
         <v>986</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>993</v>
+        <v>990</v>
       </c>
       <c r="E195" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F195" s="2">
         <v>12</v>
@@ -17945,10 +17968,10 @@
         <v>986</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="E196" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F196" s="2">
         <v>12</v>
@@ -17965,10 +17988,10 @@
         <v>986</v>
       </c>
       <c r="D197" s="2" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
       <c r="E197" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F197" s="2">
         <v>12</v>
@@ -17985,111 +18008,117 @@
         <v>986</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
       <c r="E198" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F198" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="199" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
+        <v>984</v>
+      </c>
+      <c r="B199" s="2" t="s">
+        <v>991</v>
+      </c>
+      <c r="C199" s="2" t="s">
+        <v>986</v>
+      </c>
+      <c r="D199" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="E199" s="2">
+        <v>4</v>
+      </c>
+      <c r="F199" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A200" s="2" t="s">
+        <v>984</v>
+      </c>
+      <c r="B200" s="2" t="s">
+        <v>991</v>
+      </c>
+      <c r="C200" s="2" t="s">
+        <v>986</v>
+      </c>
+      <c r="D200" s="2" t="s">
+        <v>996</v>
+      </c>
+      <c r="E200" s="2">
+        <v>5</v>
+      </c>
+      <c r="F200" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A201" s="2" t="s">
         <v>997</v>
       </c>
-      <c r="B199" s="2" t="s">
+      <c r="B201" s="2" t="s">
         <v>998</v>
       </c>
-      <c r="C199" s="2" t="s">
+      <c r="C201" s="2" t="s">
         <v>982</v>
       </c>
-      <c r="D199" s="2" t="s">
+      <c r="D201" s="2" t="s">
         <v>999</v>
       </c>
-      <c r="E199" s="2">
+      <c r="E201" s="2">
         <v>20</v>
       </c>
-      <c r="F199" s="2">
+      <c r="F201" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A201" s="3" t="s">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A203" s="3" t="s">
         <v>1000</v>
       </c>
-      <c r="B201" s="3" t="s">
+      <c r="B203" s="3" t="s">
         <v>1001</v>
       </c>
-      <c r="C201" s="4"/>
-      <c r="D201" s="4"/>
-      <c r="E201" s="4"/>
-      <c r="F201" s="4"/>
-      <c r="G201" s="4"/>
-    </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A202" s="6" t="s">
+      <c r="C203" s="4"/>
+      <c r="D203" s="4"/>
+      <c r="E203" s="4"/>
+      <c r="F203" s="4"/>
+      <c r="G203" s="4"/>
+    </row>
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A204" s="6" t="s">
         <v>1002</v>
       </c>
-      <c r="B202" s="6" t="s">
+      <c r="B204" s="6" t="s">
         <v>1003</v>
       </c>
-      <c r="C202" s="6" t="s">
+      <c r="C204" s="6" t="s">
         <v>1004</v>
       </c>
-      <c r="D202" s="6" t="s">
+      <c r="D204" s="6" t="s">
         <v>1005</v>
       </c>
-      <c r="E202" s="6" t="s">
+      <c r="E204" s="6" t="s">
         <v>745</v>
-      </c>
-    </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A203" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="B203" s="2" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C203" s="2" t="s">
-        <v>1007</v>
-      </c>
-      <c r="D203" s="2" t="s">
-        <v>1008</v>
-      </c>
-      <c r="E203" s="2" t="s">
-        <v>746</v>
-      </c>
-    </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A204" s="2" t="s">
-        <v>1009</v>
-      </c>
-      <c r="B204" s="2" t="s">
-        <v>1010</v>
-      </c>
-      <c r="C204" s="2" t="s">
-        <v>1007</v>
-      </c>
-      <c r="D204" s="2" t="s">
-        <v>1011</v>
-      </c>
-      <c r="E204" s="2" t="s">
-        <v>746</v>
       </c>
     </row>
     <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>1012</v>
+        <v>287</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>1013</v>
+        <v>1006</v>
       </c>
       <c r="C205" s="2" t="s">
         <v>1007</v>
       </c>
       <c r="D205" s="2" t="s">
-        <v>1014</v>
+        <v>1008</v>
       </c>
       <c r="E205" s="2" t="s">
         <v>746</v>
@@ -18097,16 +18126,16 @@
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>1015</v>
+        <v>1009</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>1016</v>
+        <v>1010</v>
       </c>
       <c r="C206" s="2" t="s">
         <v>1007</v>
       </c>
       <c r="D206" s="2" t="s">
-        <v>1017</v>
+        <v>1011</v>
       </c>
       <c r="E206" s="2" t="s">
         <v>746</v>
@@ -18114,16 +18143,16 @@
     </row>
     <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
-        <v>1018</v>
+        <v>1012</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>1019</v>
+        <v>1013</v>
       </c>
       <c r="C207" s="2" t="s">
         <v>1007</v>
       </c>
       <c r="D207" s="2" t="s">
-        <v>1020</v>
+        <v>1014</v>
       </c>
       <c r="E207" s="2" t="s">
         <v>746</v>
@@ -18131,16 +18160,16 @@
     </row>
     <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
-        <v>1021</v>
+        <v>1015</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>1022</v>
+        <v>1016</v>
       </c>
       <c r="C208" s="2" t="s">
         <v>1007</v>
       </c>
       <c r="D208" s="2" t="s">
-        <v>1023</v>
+        <v>1017</v>
       </c>
       <c r="E208" s="2" t="s">
         <v>746</v>
@@ -18148,16 +18177,16 @@
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
-        <v>1024</v>
+        <v>1018</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>1025</v>
+        <v>1019</v>
       </c>
       <c r="C209" s="2" t="s">
         <v>1007</v>
       </c>
       <c r="D209" s="2" t="s">
-        <v>1026</v>
+        <v>1020</v>
       </c>
       <c r="E209" s="2" t="s">
         <v>746</v>
@@ -18165,287 +18194,293 @@
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>1027</v>
+        <v>1021</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>1028</v>
+        <v>1022</v>
       </c>
       <c r="C210" s="2" t="s">
         <v>1007</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>1029</v>
+        <v>1023</v>
       </c>
       <c r="E210" s="2" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="211" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>1030</v>
+        <v>1024</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>1031</v>
+        <v>1025</v>
       </c>
       <c r="C211" s="2" t="s">
         <v>1007</v>
       </c>
       <c r="D211" s="2" t="s">
-        <v>1032</v>
+        <v>1026</v>
       </c>
       <c r="E211" s="2" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="212" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A212" s="30" t="s">
-        <v>729</v>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A212" s="2" t="s">
+        <v>1027</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>728</v>
+        <v>1028</v>
       </c>
       <c r="C212" s="2" t="s">
         <v>1007</v>
       </c>
       <c r="D212" s="2" t="s">
+        <v>1029</v>
+      </c>
+      <c r="E212" s="2" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A213" s="2" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B213" s="2" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C213" s="2" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D213" s="2" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E213" s="2" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="214" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A214" s="30" t="s">
+        <v>729</v>
+      </c>
+      <c r="B214" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="C214" s="2" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D214" s="2" t="s">
         <v>1618</v>
       </c>
-      <c r="E212" s="30" t="s">
+      <c r="E214" s="30" t="s">
         <v>1617</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A214" s="3" t="s">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A216" s="3" t="s">
         <v>1038</v>
       </c>
-      <c r="B214" s="3" t="s">
+      <c r="B216" s="3" t="s">
         <v>1039</v>
       </c>
-      <c r="C214" s="4"/>
-      <c r="D214" s="4"/>
-      <c r="E214" s="4"/>
-      <c r="F214" s="4"/>
-      <c r="G214" s="4"/>
-    </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A215" s="6" t="s">
+      <c r="C216" s="4"/>
+      <c r="D216" s="4"/>
+      <c r="E216" s="4"/>
+      <c r="F216" s="4"/>
+      <c r="G216" s="4"/>
+    </row>
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A217" s="6" t="s">
         <v>1040</v>
       </c>
-      <c r="B215" s="6" t="s">
+      <c r="B217" s="6" t="s">
         <v>813</v>
       </c>
-      <c r="C215" s="6" t="s">
+      <c r="C217" s="6" t="s">
         <v>795</v>
       </c>
-      <c r="D215" s="6" t="s">
+      <c r="D217" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="216" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A216" s="2" t="s">
+    <row r="218" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A218" s="2" t="s">
         <v>935</v>
       </c>
-      <c r="B216" s="2">
+      <c r="B218" s="2">
         <v>0.9</v>
       </c>
-      <c r="C216" s="2">
+      <c r="C218" s="2">
         <v>1.1499999999999999</v>
       </c>
-      <c r="D216" s="2" t="s">
+      <c r="D218" s="2" t="s">
         <v>1041</v>
-      </c>
-    </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A217" s="2" t="s">
-        <v>943</v>
-      </c>
-      <c r="B217" s="2">
-        <v>0.9</v>
-      </c>
-      <c r="C217" s="2">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A218" s="2" t="s">
-        <v>949</v>
-      </c>
-      <c r="B218" s="2">
-        <v>0.85</v>
-      </c>
-      <c r="C218" s="2">
-        <v>1.25</v>
       </c>
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
-        <v>957</v>
+        <v>943</v>
       </c>
       <c r="B219" s="2">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="C219" s="2">
-        <v>1.35</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
+        <v>949</v>
+      </c>
+      <c r="B220" s="2">
+        <v>0.85</v>
+      </c>
+      <c r="C220" s="2">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A221" s="2" t="s">
+        <v>957</v>
+      </c>
+      <c r="B221" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="C221" s="2">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A222" s="2" t="s">
         <v>1973</v>
       </c>
-      <c r="B220" s="2">
+      <c r="B222" s="2">
         <v>0.89</v>
       </c>
-      <c r="C220" s="2">
+      <c r="C222" s="2">
         <v>1.1100000000000001</v>
       </c>
-      <c r="D220" t="s">
+      <c r="D222" t="s">
         <v>1974</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A222" s="3" t="s">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A224" s="3" t="s">
         <v>1811</v>
       </c>
-      <c r="B222" s="3" t="s">
+      <c r="B224" s="3" t="s">
         <v>1812</v>
       </c>
-      <c r="C222" s="4"/>
-      <c r="D222" s="4"/>
-      <c r="E222" s="4"/>
-      <c r="F222" s="4"/>
-      <c r="G222" s="4"/>
-    </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A223" s="6" t="s">
+      <c r="C224" s="4"/>
+      <c r="D224" s="4"/>
+      <c r="E224" s="4"/>
+      <c r="F224" s="4"/>
+      <c r="G224" s="4"/>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A225" s="6" t="s">
         <v>874</v>
       </c>
-      <c r="B223" s="6" t="s">
+      <c r="B225" s="6" t="s">
         <v>1813</v>
       </c>
-      <c r="C223" s="6" t="s">
+      <c r="C225" s="6" t="s">
         <v>1814</v>
       </c>
-      <c r="D223" s="6" t="s">
+      <c r="D225" s="6" t="s">
         <v>1815</v>
       </c>
-      <c r="E223" s="6" t="s">
+      <c r="E225" s="6" t="s">
         <v>1816</v>
       </c>
-    </row>
-    <row r="224" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A224" s="2" t="s">
-        <v>1817</v>
-      </c>
-      <c r="B224" s="2" t="s">
-        <v>1818</v>
-      </c>
-      <c r="C224" s="2">
-        <v>1</v>
-      </c>
-      <c r="D224" s="2"/>
-      <c r="E224" s="2"/>
-    </row>
-    <row r="225" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A225" s="2" t="s">
-        <v>1819</v>
-      </c>
-      <c r="B225" s="2" t="s">
-        <v>1820</v>
-      </c>
-      <c r="C225" s="2">
-        <v>3</v>
-      </c>
-      <c r="D225" s="2"/>
-      <c r="E225" s="2"/>
     </row>
     <row r="226" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
-        <v>1821</v>
+        <v>1817</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>1822</v>
+        <v>1818</v>
       </c>
       <c r="C226" s="2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D226" s="2"/>
       <c r="E226" s="2"/>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
-        <v>1823</v>
+        <v>1819</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>1824</v>
+        <v>1820</v>
       </c>
       <c r="C227" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D227" s="2"/>
-      <c r="E227" s="2" t="s">
-        <v>943</v>
-      </c>
-    </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E227" s="2"/>
+    </row>
+    <row r="228" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
-        <v>1825</v>
+        <v>1821</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>1826</v>
+        <v>1822</v>
       </c>
       <c r="C228" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D228" s="2"/>
       <c r="E228" s="2"/>
     </row>
-    <row r="229" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="2" t="s">
-        <v>1827</v>
+        <v>1823</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>1828</v>
+        <v>1824</v>
       </c>
       <c r="C229" s="2">
         <v>1</v>
       </c>
       <c r="D229" s="2"/>
-      <c r="E229" s="2"/>
-    </row>
-    <row r="230" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="E229" s="2" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
-        <v>1829</v>
+        <v>1825</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>1830</v>
+        <v>1826</v>
       </c>
       <c r="C230" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D230" s="2"/>
       <c r="E230" s="2"/>
     </row>
     <row r="231" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
-        <v>1831</v>
+        <v>1827</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>1832</v>
+        <v>1828</v>
       </c>
       <c r="C231" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D231" s="2"/>
-      <c r="E231" s="2" t="s">
-        <v>949</v>
-      </c>
-    </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E231" s="2"/>
+    </row>
+    <row r="232" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A232" s="2" t="s">
-        <v>1833</v>
+        <v>1829</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>1834</v>
+        <v>1830</v>
       </c>
       <c r="C232" s="2">
         <v>1</v>
@@ -18453,25 +18488,27 @@
       <c r="D232" s="2"/>
       <c r="E232" s="2"/>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A233" s="2" t="s">
-        <v>1835</v>
+        <v>1831</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>1836</v>
+        <v>1832</v>
       </c>
       <c r="C233" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D233" s="2"/>
-      <c r="E233" s="2"/>
+      <c r="E233" s="2" t="s">
+        <v>949</v>
+      </c>
     </row>
     <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
-        <v>1837</v>
+        <v>1833</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>1838</v>
+        <v>1834</v>
       </c>
       <c r="C234" s="2">
         <v>1</v>
@@ -18481,23 +18518,23 @@
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
-        <v>1839</v>
+        <v>1835</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>1840</v>
+        <v>1836</v>
       </c>
       <c r="C235" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D235" s="2"/>
       <c r="E235" s="2"/>
     </row>
     <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="2" t="s">
-        <v>1841</v>
+        <v>1837</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>1842</v>
+        <v>1838</v>
       </c>
       <c r="C236" s="2">
         <v>1</v>
@@ -18507,10 +18544,10 @@
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
-        <v>1843</v>
+        <v>1839</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>1844</v>
+        <v>1840</v>
       </c>
       <c r="C237" s="2">
         <v>0.5</v>
@@ -18518,81 +18555,81 @@
       <c r="D237" s="2"/>
       <c r="E237" s="2"/>
     </row>
-    <row r="238" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">
-        <v>1845</v>
+        <v>1841</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>1846</v>
+        <v>1842</v>
       </c>
       <c r="C238" s="2">
         <v>1</v>
       </c>
-      <c r="D238" s="2">
-        <v>2</v>
-      </c>
+      <c r="D238" s="2"/>
       <c r="E238" s="2"/>
     </row>
-    <row r="239" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="2" t="s">
-        <v>1847</v>
+        <v>1843</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>1848</v>
+        <v>1844</v>
       </c>
       <c r="C239" s="2">
         <v>0.5</v>
       </c>
-      <c r="D239" s="2">
+      <c r="D239" s="2"/>
+      <c r="E239" s="2"/>
+    </row>
+    <row r="240" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A240" s="2" t="s">
+        <v>1845</v>
+      </c>
+      <c r="B240" s="2" t="s">
+        <v>1846</v>
+      </c>
+      <c r="C240" s="2">
+        <v>1</v>
+      </c>
+      <c r="D240" s="2">
+        <v>2</v>
+      </c>
+      <c r="E240" s="2"/>
+    </row>
+    <row r="241" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A241" s="2" t="s">
+        <v>1847</v>
+      </c>
+      <c r="B241" s="2" t="s">
+        <v>1848</v>
+      </c>
+      <c r="C241" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D241" s="2">
         <v>0.25</v>
       </c>
-      <c r="E239" s="2"/>
-    </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A240" s="2" t="s">
+      <c r="E241" s="2"/>
+    </row>
+    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A242" s="2" t="s">
         <v>1849</v>
       </c>
-      <c r="B240" s="2" t="s">
+      <c r="B242" s="2" t="s">
         <v>1850</v>
       </c>
-      <c r="C240" s="2">
+      <c r="C242" s="2">
         <v>2</v>
-      </c>
-      <c r="D240" s="2"/>
-      <c r="E240" s="2"/>
-    </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A241" s="2" t="s">
-        <v>1851</v>
-      </c>
-      <c r="B241" s="2" t="s">
-        <v>1852</v>
-      </c>
-      <c r="C241" s="2">
-        <v>1</v>
-      </c>
-      <c r="D241" s="2"/>
-      <c r="E241" s="2"/>
-    </row>
-    <row r="242" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A242" s="2" t="s">
-        <v>1853</v>
-      </c>
-      <c r="B242" s="2" t="s">
-        <v>1854</v>
-      </c>
-      <c r="C242" s="2">
-        <v>1</v>
       </c>
       <c r="D242" s="2"/>
       <c r="E242" s="2"/>
     </row>
-    <row r="243" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A243" s="2" t="s">
-        <v>1855</v>
+        <v>1851</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>1856</v>
+        <v>1852</v>
       </c>
       <c r="C243" s="2">
         <v>1</v>
@@ -18600,12 +18637,12 @@
       <c r="D243" s="2"/>
       <c r="E243" s="2"/>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A244" s="2" t="s">
-        <v>1857</v>
+        <v>1853</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>1858</v>
+        <v>1854</v>
       </c>
       <c r="C244" s="2">
         <v>1</v>
@@ -18615,10 +18652,10 @@
     </row>
     <row r="245" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A245" s="2" t="s">
-        <v>1859</v>
+        <v>1855</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>1860</v>
+        <v>1856</v>
       </c>
       <c r="C245" s="2">
         <v>1</v>
@@ -18626,467 +18663,463 @@
       <c r="D245" s="2"/>
       <c r="E245" s="2"/>
     </row>
-    <row r="246" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A246" s="2" t="s">
+        <v>1857</v>
+      </c>
+      <c r="B246" s="2" t="s">
+        <v>1858</v>
+      </c>
+      <c r="C246" s="2">
+        <v>1</v>
+      </c>
+      <c r="D246" s="2"/>
+      <c r="E246" s="2"/>
+    </row>
+    <row r="247" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A247" s="2" t="s">
+        <v>1859</v>
+      </c>
+      <c r="B247" s="2" t="s">
+        <v>1860</v>
+      </c>
+      <c r="C247" s="2">
+        <v>1</v>
+      </c>
+      <c r="D247" s="2"/>
+      <c r="E247" s="2"/>
+    </row>
+    <row r="248" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A248" s="2" t="s">
         <v>1971</v>
       </c>
-      <c r="B246" s="2" t="s">
+      <c r="B248" s="2" t="s">
         <v>1972</v>
       </c>
-      <c r="C246" s="2">
+      <c r="C248" s="2">
         <v>0</v>
       </c>
-      <c r="D246" s="2">
+      <c r="D248" s="2">
         <v>0.3</v>
       </c>
-      <c r="E246" s="2" t="s">
+      <c r="E248" s="2" t="s">
         <v>957</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A248" s="3" t="s">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A250" s="3" t="s">
         <v>1861</v>
       </c>
-      <c r="B248" s="3" t="s">
+      <c r="B250" s="3" t="s">
         <v>1862</v>
       </c>
-      <c r="C248" s="4"/>
-      <c r="D248" s="4"/>
-      <c r="E248" s="4"/>
-      <c r="F248" s="4"/>
-      <c r="G248" s="4"/>
-    </row>
-    <row r="249" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A249" s="6" t="s">
+      <c r="C250" s="4"/>
+      <c r="D250" s="4"/>
+      <c r="E250" s="4"/>
+      <c r="F250" s="4"/>
+      <c r="G250" s="4"/>
+    </row>
+    <row r="251" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A251" s="6" t="s">
         <v>874</v>
       </c>
-      <c r="B249" s="6" t="s">
+      <c r="B251" s="6" t="s">
         <v>1863</v>
       </c>
-      <c r="C249" s="6" t="s">
+      <c r="C251" s="6" t="s">
         <v>1864</v>
       </c>
-      <c r="D249" s="6" t="s">
+      <c r="D251" s="6" t="s">
         <v>1865</v>
       </c>
-      <c r="E249" s="6" t="s">
+      <c r="E251" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="250" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A250" s="2" t="s">
+    <row r="252" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A252" s="2" t="s">
         <v>1866</v>
-      </c>
-      <c r="B250" s="2" t="s">
-        <v>1867</v>
-      </c>
-      <c r="C250" s="2" t="s">
-        <v>1824</v>
-      </c>
-      <c r="D250" s="2">
-        <v>5</v>
-      </c>
-      <c r="E250" s="2" t="s">
-        <v>1868</v>
-      </c>
-    </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A251" s="2" t="s">
-        <v>1869</v>
-      </c>
-      <c r="B251" s="2" t="s">
-        <v>1867</v>
-      </c>
-      <c r="C251" s="2" t="s">
-        <v>1870</v>
-      </c>
-      <c r="D251" s="2">
-        <v>3</v>
-      </c>
-      <c r="E251" s="2"/>
-    </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A252" s="2" t="s">
-        <v>1871</v>
       </c>
       <c r="B252" s="2" t="s">
         <v>1867</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>1872</v>
+        <v>1824</v>
       </c>
       <c r="D252" s="2">
-        <v>2</v>
-      </c>
-      <c r="E252" s="2"/>
+        <v>5</v>
+      </c>
+      <c r="E252" s="2" t="s">
+        <v>1868</v>
+      </c>
     </row>
     <row r="253" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A253" s="2" t="s">
-        <v>1873</v>
+        <v>1869</v>
       </c>
       <c r="B253" s="2" t="s">
         <v>1867</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>1874</v>
+        <v>1870</v>
       </c>
       <c r="D253" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E253" s="2"/>
     </row>
-    <row r="254" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A254" s="2" t="s">
-        <v>1875</v>
+        <v>1871</v>
       </c>
       <c r="B254" s="2" t="s">
         <v>1867</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>1828</v>
+        <v>1872</v>
       </c>
       <c r="D254" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E254" s="2"/>
     </row>
-    <row r="255" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A255" s="2" t="s">
-        <v>1876</v>
+        <v>1873</v>
       </c>
       <c r="B255" s="2" t="s">
         <v>1867</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>1877</v>
+        <v>1874</v>
       </c>
       <c r="D255" s="2">
         <v>1</v>
       </c>
-      <c r="E255" s="2" t="s">
-        <v>1878</v>
-      </c>
-    </row>
-    <row r="256" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="E255" s="2"/>
+    </row>
+    <row r="256" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A256" s="2" t="s">
-        <v>1879</v>
+        <v>1875</v>
       </c>
       <c r="B256" s="2" t="s">
         <v>1867</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>1880</v>
+        <v>1828</v>
       </c>
       <c r="D256" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="E256" s="2" t="s">
-        <v>1881</v>
-      </c>
-    </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="E256" s="2"/>
+    </row>
+    <row r="257" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A257" s="2" t="s">
-        <v>1882</v>
+        <v>1876</v>
       </c>
       <c r="B257" s="2" t="s">
         <v>1867</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>1883</v>
+        <v>1877</v>
       </c>
       <c r="D257" s="2">
         <v>1</v>
       </c>
-      <c r="E257" s="2"/>
-    </row>
-    <row r="258" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="E257" s="2" t="s">
+        <v>1878</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" ht="51" x14ac:dyDescent="0.25">
       <c r="A258" s="2" t="s">
-        <v>1884</v>
+        <v>1879</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>1885</v>
+        <v>1867</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>1886</v>
+        <v>1880</v>
       </c>
       <c r="D258" s="2">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E258" s="2" t="s">
-        <v>1887</v>
-      </c>
-    </row>
-    <row r="259" spans="1:5" ht="51" x14ac:dyDescent="0.25">
+        <v>1881</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" s="2" t="s">
-        <v>1888</v>
+        <v>1882</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>1885</v>
+        <v>1867</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>1838</v>
+        <v>1883</v>
       </c>
       <c r="D259" s="2">
-        <v>4</v>
-      </c>
-      <c r="E259" s="2" t="s">
-        <v>1889</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E259" s="2"/>
     </row>
     <row r="260" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A260" s="2" t="s">
-        <v>1890</v>
+        <v>1884</v>
       </c>
       <c r="B260" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>1891</v>
+        <v>1886</v>
       </c>
       <c r="D260" s="2">
         <v>2</v>
       </c>
       <c r="E260" s="2" t="s">
-        <v>1892</v>
-      </c>
-    </row>
-    <row r="261" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+        <v>1887</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5" ht="51" x14ac:dyDescent="0.25">
       <c r="A261" s="2" t="s">
-        <v>1893</v>
+        <v>1888</v>
       </c>
       <c r="B261" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>1894</v>
+        <v>1838</v>
       </c>
       <c r="D261" s="2">
-        <v>1</v>
-      </c>
-      <c r="E261" s="2"/>
-    </row>
-    <row r="262" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="E261" s="2" t="s">
+        <v>1889</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A262" s="2" t="s">
-        <v>1895</v>
+        <v>1890</v>
       </c>
       <c r="B262" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>1896</v>
+        <v>1891</v>
       </c>
       <c r="D262" s="2">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E262" s="2" t="s">
-        <v>1897</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="263" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A263" s="2" t="s">
-        <v>1898</v>
+        <v>1893</v>
       </c>
       <c r="B263" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>1899</v>
+        <v>1894</v>
       </c>
       <c r="D263" s="2">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E263" s="2"/>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A264" s="2" t="s">
-        <v>1900</v>
+        <v>1895</v>
       </c>
       <c r="B264" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>1901</v>
+        <v>1896</v>
       </c>
       <c r="D264" s="2">
         <v>1.5</v>
       </c>
       <c r="E264" s="2" t="s">
-        <v>1902</v>
+        <v>1897</v>
       </c>
     </row>
     <row r="265" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A265" s="2" t="s">
-        <v>1903</v>
+        <v>1898</v>
       </c>
       <c r="B265" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>1904</v>
+        <v>1899</v>
       </c>
       <c r="D265" s="2">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="E265" s="2"/>
     </row>
-    <row r="266" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" s="2" t="s">
-        <v>1905</v>
+        <v>1900</v>
       </c>
       <c r="B266" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>1906</v>
+        <v>1901</v>
       </c>
       <c r="D266" s="2">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E266" s="2" t="s">
-        <v>1907</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="267" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
-        <v>1908</v>
+        <v>1903</v>
       </c>
       <c r="B267" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>1909</v>
+        <v>1904</v>
       </c>
       <c r="D267" s="2">
         <v>0.5</v>
       </c>
-      <c r="E267" s="2" t="s">
-        <v>1910</v>
-      </c>
+      <c r="E267" s="2"/>
     </row>
     <row r="268" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A268" s="2" t="s">
-        <v>1911</v>
+        <v>1905</v>
       </c>
       <c r="B268" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>1912</v>
+        <v>1906</v>
       </c>
       <c r="D268" s="2">
         <v>0.5</v>
       </c>
       <c r="E268" s="2" t="s">
-        <v>1913</v>
+        <v>1907</v>
       </c>
     </row>
     <row r="269" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A269" s="2" t="s">
-        <v>1914</v>
+        <v>1908</v>
       </c>
       <c r="B269" s="2" t="s">
         <v>1885</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>1915</v>
+        <v>1909</v>
       </c>
       <c r="D269" s="2">
         <v>0.5</v>
       </c>
       <c r="E269" s="2" t="s">
+        <v>1910</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A270" s="2" t="s">
+        <v>1911</v>
+      </c>
+      <c r="B270" s="2" t="s">
+        <v>1885</v>
+      </c>
+      <c r="C270" s="2" t="s">
+        <v>1912</v>
+      </c>
+      <c r="D270" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E270" s="2" t="s">
+        <v>1913</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A271" s="2" t="s">
+        <v>1914</v>
+      </c>
+      <c r="B271" s="2" t="s">
+        <v>1885</v>
+      </c>
+      <c r="C271" s="2" t="s">
+        <v>1915</v>
+      </c>
+      <c r="D271" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E271" s="2" t="s">
         <v>1916</v>
-      </c>
-    </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A270" s="2" t="s">
-        <v>1917</v>
-      </c>
-      <c r="B270" s="2" t="s">
-        <v>1918</v>
-      </c>
-      <c r="C270" s="2" t="s">
-        <v>1824</v>
-      </c>
-      <c r="D270" s="2">
-        <v>3</v>
-      </c>
-      <c r="E270" s="2" t="s">
-        <v>1919</v>
-      </c>
-    </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A271" s="2" t="s">
-        <v>1920</v>
-      </c>
-      <c r="B271" s="2" t="s">
-        <v>1918</v>
-      </c>
-      <c r="C271" s="2" t="s">
-        <v>1921</v>
-      </c>
-      <c r="D271" s="2">
-        <v>2</v>
-      </c>
-      <c r="E271" s="2" t="s">
-        <v>1919</v>
       </c>
     </row>
     <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="2" t="s">
-        <v>1922</v>
+        <v>1917</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>1923</v>
+        <v>1918</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>1924</v>
+        <v>1824</v>
       </c>
       <c r="D272" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E272" s="2" t="s">
         <v>1919</v>
       </c>
     </row>
-    <row r="273" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A273" s="2" t="s">
-        <v>1925</v>
+        <v>1920</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>1923</v>
+        <v>1918</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>1926</v>
+        <v>1921</v>
       </c>
       <c r="D273" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="E273" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="E273" s="2" t="s">
+        <v>1919</v>
+      </c>
     </row>
     <row r="274" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A274" s="2" t="s">
-        <v>1927</v>
+        <v>1922</v>
       </c>
       <c r="B274" s="2" t="s">
         <v>1923</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>1928</v>
+        <v>1924</v>
       </c>
       <c r="D274" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="E274" s="2"/>
-    </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="E274" s="2" t="s">
+        <v>1919</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A275" s="2" t="s">
-        <v>1929</v>
+        <v>1925</v>
       </c>
       <c r="B275" s="2" t="s">
         <v>1923</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>1930</v>
+        <v>1926</v>
       </c>
       <c r="D275" s="2">
         <v>0.5</v>
@@ -19095,167 +19128,197 @@
     </row>
     <row r="276" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A276" s="2" t="s">
+        <v>1927</v>
+      </c>
+      <c r="B276" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="C276" s="2" t="s">
+        <v>1928</v>
+      </c>
+      <c r="D276" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E276" s="2"/>
+    </row>
+    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A277" s="2" t="s">
+        <v>1929</v>
+      </c>
+      <c r="B277" s="2" t="s">
+        <v>1923</v>
+      </c>
+      <c r="C277" s="2" t="s">
+        <v>1930</v>
+      </c>
+      <c r="D277" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E277" s="2"/>
+    </row>
+    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A278" s="2" t="s">
         <v>1931</v>
       </c>
-      <c r="B276" s="2" t="s">
+      <c r="B278" s="2" t="s">
         <v>1932</v>
       </c>
-      <c r="C276" s="2" t="s">
+      <c r="C278" s="2" t="s">
         <v>1933</v>
       </c>
-      <c r="D276" s="2">
+      <c r="D278" s="2">
         <v>25</v>
       </c>
-      <c r="E276" s="2"/>
-    </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A278" s="3" t="s">
+      <c r="E278" s="2"/>
+    </row>
+    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A280" s="3" t="s">
         <v>1934</v>
       </c>
-      <c r="B278" s="3" t="s">
+      <c r="B280" s="3" t="s">
         <v>1935</v>
       </c>
-      <c r="C278" s="4"/>
-      <c r="D278" s="4"/>
-      <c r="E278" s="4"/>
-      <c r="F278" s="4"/>
-      <c r="G278" s="4"/>
-    </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A279" s="6" t="s">
+      <c r="C280" s="4"/>
+      <c r="D280" s="4"/>
+      <c r="E280" s="4"/>
+      <c r="F280" s="4"/>
+      <c r="G280" s="4"/>
+    </row>
+    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A281" s="6" t="s">
         <v>874</v>
       </c>
-      <c r="B279" s="6" t="s">
+      <c r="B281" s="6" t="s">
         <v>742</v>
       </c>
-      <c r="C279" s="6" t="s">
+      <c r="C281" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="280" spans="1:7" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A280" s="2" t="s">
+    <row r="282" spans="1:7" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A282" s="2" t="s">
         <v>1936</v>
       </c>
-      <c r="B280" s="2" t="s">
+      <c r="B282" s="2" t="s">
         <v>1937</v>
       </c>
-      <c r="C280" s="2" t="s">
+      <c r="C282" s="2" t="s">
         <v>1938</v>
-      </c>
-    </row>
-    <row r="281" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A281" s="2" t="s">
-        <v>1939</v>
-      </c>
-      <c r="B281" s="2" t="s">
-        <v>1940</v>
-      </c>
-      <c r="C281" s="2" t="s">
-        <v>1941</v>
-      </c>
-    </row>
-    <row r="282" spans="1:7" ht="51" x14ac:dyDescent="0.25">
-      <c r="A282" s="2" t="s">
-        <v>1942</v>
-      </c>
-      <c r="B282" s="2">
-        <v>3.5</v>
-      </c>
-      <c r="C282" s="2" t="s">
-        <v>1943</v>
       </c>
     </row>
     <row r="283" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A283" s="2" t="s">
+        <v>1939</v>
+      </c>
+      <c r="B283" s="2" t="s">
+        <v>1940</v>
+      </c>
+      <c r="C283" s="2" t="s">
+        <v>1941</v>
+      </c>
+    </row>
+    <row r="284" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A284" s="2" t="s">
+        <v>1942</v>
+      </c>
+      <c r="B284" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="C284" s="2" t="s">
+        <v>1943</v>
+      </c>
+    </row>
+    <row r="285" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A285" s="2" t="s">
         <v>1944</v>
       </c>
-      <c r="B283" s="2">
+      <c r="B285" s="2">
         <v>12</v>
       </c>
-      <c r="C283" s="2" t="s">
+      <c r="C285" s="2" t="s">
         <v>1945</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A285" s="3" t="s">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A287" s="3" t="s">
         <v>1946</v>
       </c>
-      <c r="B285" s="3" t="s">
+      <c r="B287" s="3" t="s">
         <v>1947</v>
       </c>
-      <c r="C285" s="4"/>
-      <c r="D285" s="4"/>
-      <c r="E285" s="4"/>
-      <c r="F285" s="4"/>
-      <c r="G285" s="4"/>
-    </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A286" s="6" t="s">
+      <c r="C287" s="4"/>
+      <c r="D287" s="4"/>
+      <c r="E287" s="4"/>
+      <c r="F287" s="4"/>
+      <c r="G287" s="4"/>
+    </row>
+    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A288" s="6" t="s">
         <v>1948</v>
       </c>
-      <c r="B286" s="6" t="s">
+      <c r="B288" s="6" t="s">
         <v>1949</v>
       </c>
-      <c r="C286" s="6" t="s">
+      <c r="C288" s="6" t="s">
         <v>1950</v>
       </c>
-      <c r="D286" s="6" t="s">
+      <c r="D288" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A287" s="2" t="s">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A289" s="2" t="s">
         <v>1951</v>
       </c>
-      <c r="B287" s="2">
+      <c r="B289" s="2">
         <v>0</v>
       </c>
-      <c r="C287" s="2">
+      <c r="C289" s="2">
         <v>0</v>
       </c>
-      <c r="D287" s="2" t="s">
+      <c r="D289" s="2" t="s">
         <v>1952</v>
-      </c>
-    </row>
-    <row r="288" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A288" s="2" t="s">
-        <v>1953</v>
-      </c>
-      <c r="B288" s="2">
-        <v>-3</v>
-      </c>
-      <c r="C288" s="2">
-        <v>2</v>
-      </c>
-      <c r="D288" s="2" t="s">
-        <v>1954</v>
-      </c>
-    </row>
-    <row r="289" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A289" s="2" t="s">
-        <v>1955</v>
-      </c>
-      <c r="B289" s="2">
-        <v>-1.5</v>
-      </c>
-      <c r="C289" s="2">
-        <v>1</v>
-      </c>
-      <c r="D289" s="2" t="s">
-        <v>1956</v>
       </c>
     </row>
     <row r="290" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A290" s="2" t="s">
+        <v>1953</v>
+      </c>
+      <c r="B290" s="2">
+        <v>-3</v>
+      </c>
+      <c r="C290" s="2">
+        <v>2</v>
+      </c>
+      <c r="D290" s="2" t="s">
+        <v>1954</v>
+      </c>
+    </row>
+    <row r="291" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A291" s="2" t="s">
+        <v>1955</v>
+      </c>
+      <c r="B291" s="2">
+        <v>-1.5</v>
+      </c>
+      <c r="C291" s="2">
+        <v>1</v>
+      </c>
+      <c r="D291" s="2" t="s">
+        <v>1956</v>
+      </c>
+    </row>
+    <row r="292" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A292" s="2" t="s">
         <v>1957</v>
       </c>
-      <c r="B290" s="2">
+      <c r="B292" s="2">
         <v>0</v>
       </c>
-      <c r="C290" s="2">
+      <c r="C292" s="2">
         <v>0</v>
       </c>
-      <c r="D290" s="2" t="s">
+      <c r="D292" s="2" t="s">
         <v>1958</v>
       </c>
     </row>

</xml_diff>